<commit_message>
Update debates data - 2026-03-03
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -113,6 +113,25 @@
   </si>
   <si>
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik. Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">369583</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guggisberg Lars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
 </sst>
@@ -161,8 +180,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -576,6 +595,35 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-06
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -241,9 +241,9 @@
 Antrag Aeschi [GZ]
 Streichen
 Schriftliche Begründung [GZ]
-Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat z. H. des Parlaments verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, Ständeräte hielten in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrsession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB ins Entlastungspaket 27:
+Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat zuhanden des Parlamentes verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, hielten Ständeräte in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrssession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB in das Entlastungspaket 27:
 1. Die in der Fahne zum Entlastungspaket vorgeschlagene Regelung weicht in zentralen Punkten deutlich vom PLB-Gesetzesvorschlag des Bundesrates ab. So enthält der PLB-Vorschlag gemäss Entlastungspaket bloss die Hälfte der Bestimmungen, die der Bundesrat bei der PLB-Vorlage unterbreitet hatte. Eine fundierte und seriöse Analyse der konkreten Abweichungen war sowohl für die Mitglieder der FK-N als auch für die übrigen Mitglieder des Nationalrats im gegebenen Zeitrahmen nicht möglich. Umso problematischer ist, dass die Gründe für diese erheblichen Differenzen nicht transparent dargelegt wurden. Eine solche Intransparenz erschwert eine sachgerechte parlamentarische Beurteilung und untergräbt die notwendige Nachvollziehbarkeit des Gesetzgebungsprozesses.
-2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
+2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine Ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
 [VS]
 Ch. 34[GZ]
 Proposition de la majorité [GZ]

</xml_diff>

<commit_message>
Update debates data - 2026-03-11
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -129,10 +129,10 @@
     <t xml:space="preserve">BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+    <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
   <si>
@@ -426,6 +426,24 @@
 Si vous deviez l'accepter, le Conseil fédéral poursuivrait le processus de ratification de l'accord. Il élaborera en parallèle une loi, et nous pourrons ainsi faire de notre mieux pour que le soutien à l'Ukraine et les secteurs privés en Suisse puissent débuter l'année prochaine. Je le répète : il serait administrativement et politiquement extrêmement dommage que vous suiviez cet aspect. Je vous invite vivement à rejeter cette motion, pour des raisons d'efficacité.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">371050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich vertrete hier meine Minderheit II, eine starke Minderheit zur Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz". Die Finanzkommission hat hier mit 13 zu 12 Stimmen entschieden.
+Wir beantragen Ihnen, dem Entwurf des Bundesrates zu folgen. 
+Das Weiterbildungsgesetz ist 2017 in Kraft getreten. Hier geht es in erster Linie um Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich vertrete hier meine Minderheit II, eine starke Minderheit zur Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz". Die Finanzkommission hat hier mit 13 zu 12 Stimmen entschieden.
+Wir beantragen Ihnen, dem Entwurf des Bundesrates zu folgen. 
+Das Weiterbildungsgesetz ist 2017 in Kraft getreten. Hier geht es in erster Linie um Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Auch ist gemäss einer Überprüfung der Eidgenössischen Finanzkontrolle aus dem Jahr 2021 unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Es sind also sozusagen Beiträge, die gemäss Bundesrat durchaus gekürzt werden können. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. 
+Daher unterstützen wir den Entwurf des Bundesrates, und wir empfehlen Ihnen, dies auch zu tun.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -472,8 +490,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1057,6 +1075,35 @@
         <v>60</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-16
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -133,7 +133,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ich sage es gleich vorweg: Der Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton, den Kanton Bern, vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. 
-Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt 1 Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. 
+Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. 
+Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
 </t>
   </si>
   <si>
@@ -254,7 +256,7 @@
 Art. 10b texte [GZ]
 Si la FINMA estime, notamment après avoir évalué les risques encourus par une banque d'importance systémique, qu'il pourrait être nécessaire d'ordonner une des mesures visées à l'article 25 alinéa 1, la FINMA communique immédiatement son évaluation au DFF et à la Banque nationale. Une fois avisée par la FINMA, la Banque nationale communique son évaluation au DFF, notamment en ce qui concerne les risques pour l'économie et le système financier suisses.
 Art. 30b al. 3 let. a[GZ]
-a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés ;
+a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés[NB];
 Chapitre XIa titre[GZ]
 Octroi par la Confédération de garanties du risque de défaillance pour les prêts d'aide sous forme de liquidités de la Banque nationale à des banques d'importance systémique
 Art. 32a titre [GZ]
@@ -274,26 +276,26 @@
 Art. 32a al. 6 [GZ]
 Les frais pour des prestations de tiers liés aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance de la Confédération, de la Banque nationale ou de la FINMA sont mis à la charge de l'emprunteur.
 Art. 32a al. 7 [GZ]
-Le Conseil fédéral règle notamment :
-a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties ;
-b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts ;
-c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible ;
-d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale ;
+Le Conseil fédéral règle notamment[NB]:
+a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties[NB];
+b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts[NB];
+c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible[NB];
+d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale[NB];
 e. les obligations de la FINMA et de la Banque nationale en matière de réduction des risques, de surveillance et de rapports.
 Art. 32b titre [GZ]
 Obligations de l'emprunteur liées aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
 Art. 32b al. 1 [GZ]
-L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes :
-a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur ;
-b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes ;
-c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe ;
+L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes[NB]:
+a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur[NB];
+b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes[NB];
+c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe[NB];
 Art. 32b al. 2 [GZ]
 L'emprunteur et les sociétés du groupe qui y sont directement ou indirectement liées n'effectuent pas d'acte qui pourrait retarder ou compromettre le remboursement des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ou le paiement de la totalité des primes et des intérêts visés à l'article 32a, ni n'omettent d'acte qui favoriserait le remboursement des prêts ainsi que le paiement de la totalité de ces primes et intérêts
 Art. 32b al. 3 [GZ]
 L'emprunteur est tenu de rembourser les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance avant les autres prêts d'aide sous forme de liquidités que la Banque nationale lui a octroyés.
 Art. 32b al. 4 [GZ]
 Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
-a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier :
+a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier[NB]:
 1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
 2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
 b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
@@ -302,18 +304,18 @@
 Art. 32c al. 1 [GZ]
 Les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus sont attribués à la troisième classe au sens de l'article 219 alinéa 4 LP.
 Art. 32c al. 2 [GZ]
-S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant :
-a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité ;
-b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus ;
+S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant[NB]:
+a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité[NB];
+b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus[NB];
 c. toutes les autres créances de la troisième classe.
 Art. 32d titre [GZ]
 Traitement des données et échange d'informations
 Art. 32d al. 1 [GZ]
 Le DFF, la FINMA, la Banque nationale, le CDF et les tiers chargés de l'exécution des dispositions du présent chapitre peuvent traiter et se communiquer mutuellement des données personnelles et des données concernant des personnes morales, y compris des données sensibles au sens de l'article 5 lettre c chiffres 1, 2, 5 et 6, de la loi du 25 septembre 2020 sur la protection des données et des données sensibles concernant des personnes morales au sens de l'article 57r alinéa 2 de la loi du 21 mars 1997 sur l'organisation du gouvernement et de l'administration, ainsi que d'autres informations, dans la mesure où cela est nécessaire à l'exécution des dispositions du présent chapitre, notamment pour l'octroi, l'administration, la surveillance, le contrôle et le traitement des prêts d'aide sous forme de liquidités et des garanties du risque de défaillance ainsi que des sûretés, ou pour l'observation du marché.
 Art. 32d al. 2 [GZ]
-Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre :
-a. pour l'évaluation des risques pour le budget de la Confédération : les informations par que la FINMA et la Banque nationale doivent fournir au DFF ; et
-b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés : les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
+Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre[NB]:
+a. pour l'évaluation des risques pour le budget de la Confédération[NB]: les informations par que la FINMA et la Banque nationale doivent fournir au DFF[NB]; et
+b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés[NB]: les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
 Art. 32e titre [GZ]
 Examen des dispositions du présent chapitre
 Art. 32e texte [GZ]

</xml_diff>

<commit_message>
Update debates data - 2026-03-17
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -350,17 +350,17 @@
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
 Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Entwurf des Bundesrates und also dem Be</t>
+Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem </t>
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
 Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Entwurf des Bundesrates und also dem Beschluss des Ständerates. Den Minderheitsantrag Funiciello lehnen wir ab.
+Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
 Bei der Massnahme 11, "Kürzung der Subventionen für ausserschulische Kinder- und Jugendförderung", folgen wir dem Entwurf des Bundesrates. Die Kürzung dieser 1,5 Millionen Franken ist verkraftbar. Die Minderheitsanträge I (Zybach) und II (Gredig) lehnen wir dementsprechend ab.
 Bei den Massnahmen 27 und 30 folgen wir der Mehrheit der Finanzkommission und dem Beschluss des Ständerates.
 Ich komme zu meinen Minderheiten in diesem Block.
-Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen" beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildung und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
-Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
+Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
+Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch, und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
 Bei der Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz", habe ich die Minderheit III eingereicht. Das Weiterbildungsgesetz ist seit 2017 in Kraft. Auch hier beantrage ich, dem Entwurf des Bundesrates zu folgen. Es geht in erster Linie um die Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Gemäss einer Überprüfung der EFK aus dem Jahr 2021 ist unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. Daher unterstützen wir hier ebenfalls den Entwurf des Bundesrates.
 Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
@@ -461,6 +461,33 @@
   </si>
   <si>
     <t xml:space="preserve">Artikel 76e Absatz 1 BPR schreibt vor, dass die Kontrolle über die Korrektheit der Angaben und Dokumente lediglich stichprobenweise erfolgt. Die Eidgenössische Finanzkontrolle ist die zuständige Kontrollbehörde. Sie nimmt ihre Aufgaben im Rahmen der gesetzlichen Vorschriften selbstständig und unabhängig wahr. Sie wählt die Akteure, die sie prüft, risikoorientiert aus. Sie veröffentlicht die Namen der geprüften Akteure auf ihrer Website.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amaudruz Céline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réunie le 8 janvier 2026, la Commission de la sécurité sociale et de la santé publique du Conseil national a procédé à l'examen préalable de la motion 25.3637, "Mesures contraignantes en cas de hausse excessive des coûts, y compris pour les tarifs 'officiels' définis dans la LAMal", qui avait été déposée le 17 juin 2025 par M. Stefan Engler. Cette motion a été adoptée par le Conseil des États le 18 septembre 2025, par 34 voix contre 8 contre et 1 abstention.
+Que vise cette motion ? Elle charge l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réunie le 8 janvier 2026, la Commission de la sécurité sociale et de la santé publique du Conseil national a procédé à l'examen préalable de la motion 25.3637, "Mesures contraignantes en cas de hausse excessive des coûts, y compris pour les tarifs 'officiels' définis dans la LAMal", qui avait été déposée le 17 juin 2025 par M. Stefan Engler. Cette motion a été adoptée par le Conseil des États le 18 septembre 2025, par 34 voix contre 8 contre et 1 abstention.
+Que vise cette motion ? Elle charge le Conseil fédéral de compléter la loi fédérale sur l'assurance-maladie afin que l'évolution des coûts dans le domaine des tarifs officiels fixés par la Confédération fasse également l'objet d'une surveillance en cas de hausse excessive, par analogie avec le mécanisme prévu à l'article 47c LAMal pour les tarifs négociés.
+La hausse des coûts de l'assurance-maladie reste une préoccupation majeure pour la population suisse. Les projections indiquent que les personnes payant des primes ainsi que les contribuables devront assumer des charges croissantes au cours des prochaines décennies. Plusieurs facteurs contribuent à cette évolution, notamment la cherté des médicaments, les thérapies coûteuses pour certaines maladies rares, l'évolution démographique, les prestations inappropriées ou excessives, ainsi que l'augmentation quantitative de certaines prestations. Dans ce contexte, les partenaires tarifaires sont désormais tenus de surveiller l'évolution des coûts dans les domaines relevant des tarifs négociés et de prendre des mesures en cas d'évolution inexpliquée. L'auteur de la motion estime qu'il serait cohérent d'étendre un mécanisme comparable aux tarifs officiels fixés par la Confédération, notamment pour les médicaments, les analyses ou la liste des moyens et appareils.
+Le Conseil fédéral estime que la surveillance de l'évolution des coûts des tarifs officiels est déjà possible en vertu du droit en vigueur et que des mesures correctives peuvent être prises si cela est nécessaire. Il reconnaît toutefois que certaines différences existent entre les règles applicables aux tarifs officiels et celles applicables aux tarifs négociés, notamment en matière de communication et de fourniture de données. Dans ce contexte, il se déclare disposé à procéder à un état des lieux concernant les bases de données disponibles et, le cas échéant, à proposer des adaptations législatives. Toutefois, le Conseil fédéral recommande le rejet de la motion.
+La commission estime qu'une surveillance systématique de l'évolution des coûts de la santé est indispensable, compte tenu de la charge toujours plus lourde que représentent les primes dans le budget des personnes assurées. Cela vaut également pour les prestations fournies dans le cadre des tarifs officiels. En 2024, le domaine ambulatoire, les médicaments utilisés, les analyses de laboratoire, ainsi que les moyens et appareils ont représenté près de trois dixièmes des coûts bruts de l'assurance obligatoire des soins. La commission constate que la Confédération surveille de manière générale l'évolution des coûts dans les domaines soumis à des tarifs officiels et qu'elle prend également des mesures pour les réduire. Cependant, elle considère que des mesures supplémentaires doivent être prises afin que la Confédération puisse surveiller plus efficacement l'évolution des coûts dans ces domaines et exploiter au maximum le potentiel d'économies. La commission relève que, pour une surveillance efficace, il est nécessaire de procéder à des analyses différenciées et de disposer de données détaillées. Le rapport d'audit "Processus destiné à assurer la réalité des coûts dans le domaine des tarifs médicaux" du Contrôle fédéral des finances (CDF), daté du 16 décembre 2024, le confirme. Le CDF indique qu'en ce qui concerne les tarifs officiels, les compétences de la Confédération en matière de communication et de fourniture des données sont moins étendues que pour les tarifs négociés, alors même que ces tarifs sont fixés par les autorités.
+Lors de ses délibérations, la commission a également été informée par l'administration que, dans le domaine des tarifs officiels, les autorités dépendent encore souvent de la coopération des fournisseurs de prestations pour obtenir certaines données nécessaires à l'adaptation des services. Plusieurs membres ont estimé que la motion pouvait contribuer à combler cette lacune et à renforcer la cohérence des instruments de surveillance des coûts. Pour avoir accès aux données nécessaires, les autorités dépendent donc du bon vouloir des fournisseurs de prestations et n'exigent pas non plus de possibilités d'adopter des sanctions.
+En conséquence, la commission salue la volonté du Conseil fédéral de dresser un état des lieux des bases de données. En adoptant la motion, elle entend encourager ces travaux, renforcer le rôle de la Confédération dans ce domaine et donc combler les éventuelles lacunes.
+Je vous recommande donc, au nom de la commission, d'adopter cette motion que nous avons acceptée, par 24 voix contre 0 et 1 abstention.
 </t>
   </si>
 </sst>
@@ -509,8 +536,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I13" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I13"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1150,6 +1177,35 @@
         <v>69</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-18
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -263,7 +263,7 @@
 Garanties du risque de défaillance
 Art. 32a al. 1 [GZ]
 La Confédération peut octroyer à la Banque nationale des garanties du risque de défaillance subsidiaires pour les prêts d'aide sous forme de liquidités qui ont été accordés à des banques d'importance systémique ou faisant partie d'un groupe financier d'importance systémique, si
-a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être; et
+a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être[NB]; et
 b. sans l'octroi de tels prêts, l'économie et le système financier suisses risquent de subir des dommages considérables.
 Art. 32a al. 2 [GZ]
 Une fois par année, la Confédération prélève auprès des banques qui sont d'importance systémique ou font partie d'un groupe financier d'importance systémique un forfait pour risque lié à une éventuelle mise à disposition d'une garantie du risque de défaillance. Le forfait équivaut au produit d'un taux de calcul unique et d'une base de calcul déterminée pour chacune des banques.
@@ -296,7 +296,7 @@
 Art. 32b al. 4 [GZ]
 Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
 a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier[NB]:
-1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
+1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c[NB]; et
 2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
 b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
 Art. 32c titre [GZ]
@@ -488,6 +488,77 @@
 Lors de ses délibérations, la commission a également été informée par l'administration que, dans le domaine des tarifs officiels, les autorités dépendent encore souvent de la coopération des fournisseurs de prestations pour obtenir certaines données nécessaires à l'adaptation des services. Plusieurs membres ont estimé que la motion pouvait contribuer à combler cette lacune et à renforcer la cohérence des instruments de surveillance des coûts. Pour avoir accès aux données nécessaires, les autorités dépendent donc du bon vouloir des fournisseurs de prestations et n'exigent pas non plus de possibilités d'adopter des sanctions.
 En conséquence, la commission salue la volonté du Conseil fédéral de dresser un état des lieux des bases de données. En adoptant la motion, elle entend encourager ces travaux, renforcer le rôle de la Confédération dans ce domaine et donc combler les éventuelles lacunes.
 Je vous recommande donc, au nom de la commission, d'adopter cette motion que nous avons acceptée, par 24 voix contre 0 et 1 abstention.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372428</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260318</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dittli Josef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aus dem Bereich der ständerätlichen Subkommission EDA/VBS berichte ich Ihnen heute über drei massgebliche Geschäfte, welche uns im Jahr 2025 intensiv beschäftigten: erstens die Inspektion der Parlamentarischen Verwaltungskontrolle über die Honorarkonsulate, zweitens die Steuerung der Ruag MRO durch das VBS und drittens die Cybersicherheit der Armee.
+Lassen Sie mich mit den Honorarkonsulaten beginnen. Diese ehrenamtlich geführten Vertretungen sind eine lokale Anlaufstelle für Schweizer Staatsange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aus dem Bereich der ständerätlichen Subkommission EDA/VBS berichte ich Ihnen heute über drei massgebliche Geschäfte, welche uns im Jahr 2025 intensiv beschäftigten: erstens die Inspektion der Parlamentarischen Verwaltungskontrolle über die Honorarkonsulate, zweitens die Steuerung der Ruag MRO durch das VBS und drittens die Cybersicherheit der Armee.
+Lassen Sie mich mit den Honorarkonsulaten beginnen. Diese ehrenamtlich geführten Vertretungen sind eine lokale Anlaufstelle für Schweizer Staatsangehörige und unterstützen unsere Interessensvertretungen im Ausland. Gleichzeitig sind damit jedoch Reputationsrisiken verbunden. Da sich die Zahl der Schweizer Honorarkonsulate im Ausland seit 1990 verdoppelt hat, beauftragten die Geschäftsprüfungskommissionen im Januar 2024 die Parlamentarische Verwaltungskontrolle mit einer Evaluation. Diese untersuchte sowohl den Umgang des EDA mit den Schweizer Vertretungen im Ausland als auch jenen mit den ausländischen Honorarkonsulaten in der Schweiz. 
+Die Evaluation hat gezeigt, dass die Schweizer Honorarkonsulate im Ausland einen Mehrwert erbringen und vom EDA insgesamt angemessen betreut werden. Allerdings hängt die Qualität der Führung stark von der jeweiligen Vertretung im Empfangsstaat ab. Zudem halten sich die Vertretungen bei der Ernennung zwar an die Vorgaben, prüfen aber die Interessenbindungen zu wenig systematisch. Hier empfiehlt die GPK zukünftig eine systematische Prüfung potenzieller Interessenkonflikte. Auch fehlten im Untersuchungszeitraum klare strategische Vorgaben des Bundesrates zum Einsatz der Honorarkonsulate im Ausland. Das EDA hat zwar Ende 2025 eine neue Konsularstrategie publiziert, deren Mehrwert werden wir jedoch im Rahmen der Stellungnahme des Bundesrates erst noch analysieren.
+Kritischer beurteilt die Kommission das Vorgehen gegenüber ausländischen Honorarkonsulaten in der Schweiz, wo sich das EDA aus Rücksicht auf die bilateralen Beziehungen zu stark zurückhält. Wir empfehlen hier ein stringenteres Vorgehen. Wir erwarten auch hier die Stellungnahmen des Bundesrates.
+Ich komme nun zum zweiten Schwerpunkt, der Steuerung der Ruag MRO. Die Abklärungen der GPK-S zur Steuerung durch das VBS als Eigner bestätigten verschiedene erhebliche Mängel. Ein zentraler Punkt betrifft den unzweckmässigen Umgang mit Hinweisen auf Probleme aus dem Jahre 2019. Aus Sicht der Kommission wurde eine damalige Whistleblower-Meldung bei der Ruag Holding AG durch den Eigner suboptimal behandelt. Das VBS reagierte zwar im Prinzip zuerst richtig, indem es eine Anfrage an den Verwaltungsrat stellte. Im Nachhinein zeigte sich jedoch, dass auf dessen Beschwichtigungen kein Verlass war. Es ist für uns nur schwer nachvollziehbar, dass das VBS 2019 nicht in der Lage war, zu erkennen, dass in der Stellungnahme der Geschäftsleitung die Entkräftung des wichtigsten Vorwurfs fehlte, nämlich die Veräusserung von Material deutlich unter Marktpreisen. 
+Ebenfalls kritisch beurteilen wir die verspätete Berücksichtigung der Compliance in den strategischen Zielen. Obwohl der Bundesrat nach der Postauto-Affäre entschieden hatte, dass bundesnahe Unternehmen ein Compliance-Management-System führen müssen, verzichtete er bei der Ruag MRO zunächst darauf. Erst für die Periode 2024 bis 2027 wurde ein entsprechendes Ziel aufgenommen, was aus Sicht der Kommission eindeutig zu spät war. Wir bekräftigen unsere Haltung, dass der Bundesrat dafür sorgen muss, dass die Eignerstellen solche Compliance-Themen regelmässig mit dem Unternehmen besprechen. 
+Ein weiterer Mangel betrifft die zu positive Berichterstattung. Der Verwaltungsrat erstattete zunächst zu optimistisch Bericht, und der Bundesrat hinterfragte diese Zielbeurteilung zu wenig kritisch. In der Folge fiel auch die Information an die parlamentarischen Aufsichtskommissionen zu positiv aus. Wir fordern hier künftig eine transparente und kritische Information der Oberaufsicht. Die Vorfälle rund um den geplanten Verkauf von 96 Leopard-1-Panzern im Jahre 2023 haben diese Fragen zur Aufsicht und Steuerung durch den Eigner massiv verschärft.
+Deshalb haben wir ein Postulat eingereicht, um das aktuelle System der Corporate Governance und das duale Steuerungsmodell grundlegend zu prüfen. Wir erwarten, dass der Bundesrat die anstehende Anpassung der Rechtsform der Ruag MRO strategisch nutzt, um die Erkenntnisse aus den Prüfungen konsequent umzusetzen. Da die forensischen Untersuchungen externer Kanzleien und weitere Prüfungen der Eidgenössischen Finanzkontrolle noch andauern, behält sich die Kommission vor, zu einem späteren Zeitpunkt auf die Ereignisse zurückzukommen. Es wurden verschiedene Empfehlungen ausgesprochen. Der Bundesrat wird zu diesen Empfehlungen Stellung nehmen, und die Subkommission wird zusammen mit der Kommission die Antworten überprüfen.
+Abschliessend zum dritten Schwerpunkt, der Cybersicherheit der Armee. Die GPK-S beschäftigt sich seit 2023 im Nachgang zum Cyberangriff auf den Dienstleister Xplain vertieft mit der zivilen Cybersicherheit der Bundesverwaltung. Im Berichtsjahr hat die Kommission nun auch die Cybersicherheit der Armee behandelt. Dazu liess sie sich vom Kommando Cyber über dessen Organisation, Aufgaben und Herausforderungen informieren. Dabei nahm die Kommission den Stand der Umsetzung der Gesamtkonzeption Cyber vom 13. April 2022 zur Kenntnis.
+Wir konnten feststellen, dass die Rechtsgrundlagen, die Finanzen und das Personal das Kommando Cyber derzeit befähigen, seine Ziele zu erreichen. Herausforderungen bestehen weiterhin, insbesondere im Umgang mit international unterschiedlichen Klassifizierungsstufen und bei möglichen kollateralen Auswirkungen von Störungsaktionen, die das Kommando Cyber betreffen. Dennoch konnte sich die Kommission davon überzeugen, dass der Austausch des Kommandos mit den betroffenen Akteuren zweckmässig ist. Im Umgang mit den erwähnten Klassifizierungsstufen verfolgt das Kommando Cyber nachvollziehbare Ziele.
+Zudem konnten wir feststellen, dass das Kommando das Risiko einer Abhängigkeit von Betreibern grosser Rechenzentren wie Microsoft, Google oder Meta in seinen Umsetzungsarbeiten so weit als möglich angemessen berücksichtigt.
+Ein besonderer Schwerpunkt unserer Befassung war die Rolle des Kommandos Cyber in diversen IT-Projekten, die das VBS als sogenannte Top-Projekte führt. Dazu gehören die Projekte Telekommunikation der Armee, Führungsnetz Schweiz, Neue Digitalisierungsplattform (NDP) sowie das sichere Datenverbundnetz plus (SDVN+). 
+Ein zweiter Schwerpunkt betraf die Zusammenarbeit des Kommandos Cyber mit dem Bundesamt für Cybersicherheit (BACS). Hier stellte die Kommission fest, dass der Informationsaustausch zwischen den Einheiten funktioniert und eine klare Bereitschaft zur gegenseitigen Amtshilfe vorhanden ist. Das Kommando Cyber und das BACS arbeiten zudem gemeinsam daran, die Leistung von Amtshilfe durch Milizeinheiten zugunsten des BACS zu vereinfachen. Das ist entscheidend, um die nötige Reaktionsgeschwindigkeit bei Cybervorfällen sicherstellen zu können. Da die Kommission im Berichtsjahr keinen weiteren Handlungsbedarf bei der Cybersicherheit der Armee auf allgemeiner Ebene feststellte, hat sie ihre Arbeiten zu diesem Thema vorerst abgeschlossen. Sie bleibt aber über die Begleitung der Top-Projekte weiterhin am Ball.
+Auch ich möchte mich zum Schluss beim Sekretariat für die tolle Unterstützung und die getätigten Arbeiten während des Jahres bedanken.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372719</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hegglin Peter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Motion beauftragt den Bundesrat, die Subventionsprüfung gemäss Subventionsgesetz so anzupassen, dass daraus ein Paket für den Abbau von schädlichen Subventionen hervorgeht. Als Begründung wird ausgeführt, dass Subventionen häufig in einem suboptimalen Kosten-Nutzen-Verhältnis stünden, was in der Regel mit Fehlanreizen und Marktverzerrungen einhergehe. Deshalb sei eine sorgfältige Subventionsüberprüfung essenziell. Insbesondere sei es angesichts des sich abzeichnenden strukturellen Defizits i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Motion beauftragt den Bundesrat, die Subventionsprüfung gemäss Subventionsgesetz so anzupassen, dass daraus ein Paket für den Abbau von schädlichen Subventionen hervorgeht. Als Begründung wird ausgeführt, dass Subventionen häufig in einem suboptimalen Kosten-Nutzen-Verhältnis stünden, was in der Regel mit Fehlanreizen und Marktverzerrungen einhergehe. Deshalb sei eine sorgfältige Subventionsüberprüfung essenziell. Insbesondere sei es angesichts des sich abzeichnenden strukturellen Defizits im Bundeshaushalt wichtig, dass der Bund die Subventionen und Aufgaben immer wieder fundiert prüfe. Die Motionäre äussern die Vermutung, dass es, obwohl alle sechs Jahre eine Subventionsüberprüfung durchgeführt werde, beachtliches Optimierungspotenzial gebe. Deshalb sei der Bundesrat zu beauftragen, verschiedene Prüfvarianten zu evaluieren, so einerseits den sechsjährigen Prüfzyklus zu verkürzen und andererseits das Format anzupassen und mit einem Massnahmenpaket zu verbinden. 
+Obwohl der Bundesrat das Anliegen der Motionärin teilt, lehnt er das Motionsbegehren ab. Mit dem Entlastungspaket 27 habe er bei zahlreichen Subventionen einen Verzicht oder eine Reduktion vorgeschlagen. Er hätte auch im Subventionsgesetz festschreiben wollen, dass Finanzhilfen künftig 50 Prozent der Kosten der unterstützten Aufgabe grundsätzlich nicht übersteigen dürfen. Das hätten die Räte dann aber abgelehnt. Aus Sicht des Bundesrates sind Entlastungspakete dann zielführend, wenn sich Defizite abzeichnen. Er erachtet es deshalb als nicht zielführend, die Subventionsüberprüfung zu einem systematischen Entlastungsprogramm umzubauen. 
+Bei der Beratung lag der Kommission ein Bericht der EFK zur Subventionsüberprüfung vor. Die EFK kommt zum Schluss, dass die Prüfung wenig bewirke. Die EFK habe in den zehn Jahren zwischen 2014 und 2024 lediglich vier Fälle gefunden, in denen aus der Überprüfung tatsächlich Einsparungen hervorgegangen seien. Eingespart wurden damit dann nur zwei Millionen Franken. 
+Die Kommissionsmehrheit beurteilt die aktuelle Subventionsprüfung nicht so negativ. Die Prüfresultate der aktuell geprüften Verwaltungseinheiten werden jedes Jahr in den Botschaften zur Jahresrechnung abgedruckt. Finanzdelegation und Finanzkommission haben Einblick und können entsprechende Resultate aufnehmen und korrigieren. Das Ziel der Überprüfung besteht eh darin, die Rechtmässigkeit der Subventionen sicherzustellen. Die Prüfung hat auch einen präventiven Charakter bei den verschiedenen Ämtern und Departementen.
+Die Kommissionsmehrheit ist im Weiteren der Ansicht, dass der Zweck der Subventionsprüfung nicht darin besteht, regelmässig, systematisch und in institutioneller Weise das Sparpotenzial bei den Subventionen aufzuzeigen. Das Streichen oder Kürzen von Subventionen ist ein politischer Entscheid, der in erster Linie dem Parlament obliegen soll. Von erforderlichen Entlastungspaketen einmal abgesehen, sollte sich der gesamte Prozess von der anfänglichen Überlegung bis hin zum definitiven Subventionsbeschluss in den Händen des Parlamentes befinden. Aus Sicht der Kommission hat das Parlament heute schon die Möglichkeit, Subventionen zu befristen und damit eine periodische Überprüfung durch das Parlament zu erwirken, um endlosen Subventionen entgegenzuwirken.
+Im Rahmen von Entlastungspaketen wie dem EP 27 haben generelle Überprüfungen aber ihre Berechtigung und sind erfolgreicher. Gemäss EFK sind die Subventionsüberprüfungen heute unvollständig. Aus ihrer Sicht sind eigentlich auch Steuererleichterungen Subventionen, die alle sechs Jahre überprüft werden müssten. Weil die Politik, also wir, ihr den Zugang zu diesen Daten verwehrt, liegt die letzte Überprüfung schon 15 Jahre zurück. Daran dürfte die Politik, denke ich, auch nichts ändern wollen. 
+Weiter ist der Ausdruck "schädliche Subventionen", wie er im Motionstext steht, nicht eindeutig. Je nach politischer Sichtweise kann man zu einer anderen Einschätzung kommen, was "schädlich" bedeutet. Auch eine andere Wortwahl, z. B. "unnütze" Subventionen, oder gar die Streichung des Adjektivs erachtete die Kommission als nicht zielführend. Wenn die Bundesverwaltung Subventionen regelmässig analysieren und kontrollieren sowie Vorschläge unterbreiten müsste, könnten erhebliche unnötige Kosten entstehen, wenn das Parlament dann im Nachgang identifizierte Sparpotenziale nicht umsetzen würde. So hat das Parlament zum Beispiel beim EP 27 nur rund 60 Prozent der bundesrätlichen Sparvorschläge angenommen - und das trotz ausgewiesenem Sparbedarf. 
+Die Kommission sieht aber durchaus Verbesserungspotenzial: So können wir Subventionsregelungen bei der Ausgestaltung enger fassen, die Subventionsbeträge tief halten, die Subventionen zeitlich begrenzen und sie auch im Budgetprozess hinterfragen. Weiter können natürlich auch Subventionen, die nicht als Kredite ausgestaltet werden, einbezogen werden. Dies betrifft Leistungen, die der Bund kostenlos oder zu reduzierten Kosten anbietet, so beispielsweise Leistungen der Armee für das WEF. Es betrifft aber auch Subventionen, die über Fonds wie den Tabakpräventionsfonds ausgerichtet werden. Auch diese Leistungen sollten zukünftig durch die EFK geprüft werden. 
+Aus all den genannten Gründen lehnt die Kommission den Vorstoss mit 8 zu 4 Stimmen bei 0 Enthaltungen ab. Es gibt eine Minderheit, die ihre Argumente selber vortragen wird. Ich empfehle Ihnen, die Motion abzulehnen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">372747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben eine gleichlautende Motion schon einmal behandelt, und zwar in der Dezembersession des letzten Jahres. Jene Motion haben Sie mit 27 zu 14 Stimmen bei 2 Enthaltungen abgelehnt. Ich möchte Sie im Namen des Bundesrates bitten, auch diese Motion abzulehnen. Dies nicht, weil der Bundesrat nicht auch der Meinung ist, dass man Subventionen überprüfen soll und dass man Subventionen, die ein schlechtes Kosten-Nutzen-Verhältnis aufweisen, abschaffen soll; nein, ganz im Gegenteil. Wir haben ja di</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sie haben eine gleichlautende Motion schon einmal behandelt, und zwar in der Dezembersession des letzten Jahres. Jene Motion haben Sie mit 27 zu 14 Stimmen bei 2 Enthaltungen abgelehnt. Ich möchte Sie im Namen des Bundesrates bitten, auch diese Motion abzulehnen. Dies nicht, weil der Bundesrat nicht auch der Meinung ist, dass man Subventionen überprüfen soll und dass man Subventionen, die ein schlechtes Kosten-Nutzen-Verhältnis aufweisen, abschaffen soll; nein, ganz im Gegenteil. Wir haben ja diese Übung jetzt gemacht, ich komme darauf zurück. 
+Es gibt einen Subventionsüberprüfungsmechanismus, der greift und an und für sich gut eingespielt ist. Wir überprüfen jedes Jahr im Rahmen der Staatsrechnung die Subventionen in einem Departement. Dieses Jahr, mit der Staatsrechnung 2025, war das UVEK betroffen; Sie werden am Freitag die Botschaft bekommen und sehen, dass wir das UVEK überprüft und Massnahmen vorgeschlagen haben. Nächstes Jahr kommt das EDA dran. Die Eidgenössische Finanzkontrolle überprüft derzeit auch diesen Mechanismus und wird Bericht erstatten. Der Bundesrat wird dann die Empfehlungen der EFK selbstverständlich würdigen. Also wir machen das; das ist ein eingespielter Mechanismus.
+Zudem möchte ich Ihnen einfach in Erinnerung rufen, dass wir mit der Gruppe Gaillard eine gross angelegte Aufgaben- und Subventionsüberprüfung gemacht haben. Wir haben Ihnen die entsprechenden Anträge gestellt. So haben wir Ihnen beispielsweise beantragt, das Subventionsgesetz zu schärfen, was Sie aber im Rahmen dieses EP 27 abgelehnt haben. Und wir haben Ihnen fast 60 Massnahmen vorgelegt, insbesondere Subventionsabbau, wobei Sie aber - das ist Ihre Freiheit - rund einen Drittel davon nicht gutgeheissen haben. Der Bundesrat erachtet es deshalb im Moment nicht als nötig, noch einmal eine solche Überprüfung zu machen. Die Massnahmen, die Sie abgelehnt haben, liegen auf dem Tisch, die könnte man wieder hervornehmen. Ob sich aber deren Mehrheitsfähigkeit so schnell ändert, möchte ich bezweifeln.
+Jedenfalls bitte ich Sie, diese Motion abzulehnen. 
+Übrigens bin ich noch auf eine interessante Massnahme gestossen. In den Achtzigerjahren gab es ein Sparpaket und da hat der Bundesrat einfach die Subventionen befristet über drei Jahre um 10 Prozent reduziert hat. Ich finde das auch noch interessant. Aber Sie können sich vorstellen, was das auslösen würde.
 </t>
   </si>
 </sst>
@@ -536,8 +607,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I13" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I16"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1206,6 +1277,91 @@
         <v>75</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" t="s">
+        <v>85</v>
+      </c>
+      <c r="I15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G16" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-19
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -561,6 +561,60 @@
 Übrigens bin ich noch auf eine interessante Massnahme gestossen. In den Achtzigerjahren gab es ein Sparpaket, und da hat der Bundesrat einfach die Subventionen befristet über drei Jahre um 10 Prozent reduziert. Ich finde das auch noch interessant. Aber Sie können sich vorstellen, was das auslösen würde.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">373030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sormanni Daniel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La réponse ou les réponses du Conseil fédéral, à ce jour, sont insuffisantes. On nous parle d'un système "stable" et de 94,3 pour cent des montants versés, mais ces chiffres ne reflètent pas la réalité sur le terrain. La vérité, c'est que des personnes vivent aujourd'hui sans revenu depuis des semaines, depuis des mois. Certaines attendent leurs indemnités depuis septembre 2025, alors même que leurs droits sont reconnus et que toutes les démarches ont été accomplies. Dans ces conditions, parler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La réponse ou les réponses du Conseil fédéral, à ce jour, sont insuffisantes. On nous parle d'un système "stable" et de 94,3 pour cent des montants versés, mais ces chiffres ne reflètent pas la réalité sur le terrain. La vérité, c'est que des personnes vivent aujourd'hui sans revenu depuis des semaines, depuis des mois. Certaines attendent leurs indemnités depuis septembre 2025, alors même que leurs droits sont reconnus et que toutes les démarches ont été accomplies. Dans ces conditions, parler encore de "résorber un retard" est inacceptable. Pour les personnes concernées, ce retard est déjà insupportable.
+Autre problème majeur : le Conseil fédéral ne connaît pas le nombre exact de paiements tardifs. Dans un système financé par les cotisations, cela n'est pas acceptable. Sans transparence, il n'y a pas de confiance. On nous propose des avances, selon l'article 31 de l'ordonnance sur l'assurance-chômage, mais une avance n'est pas une solution ; c'est un palliatif. Encore faudrait-il que cela soit efficace. Les avances compliquent souvent les démarches pour des personnes déjà en difficulté et ne corrigent en rien le dysfonctionnement du système. D'ailleurs, il apparaît que l'octroi d'une avance, avec ce nouveau système, est presque aussi complexe que le traitement d'un dossier, selon certaines caisses de chômage.
+Le Contrôle fédéral des finances a publié six rapports à l'attention du SECO, avant la mise en service de ce nouveau système informatique. Toutes ses recommandations ont été acceptées, mais trop tard. Elles sont en cours d'exécution, mais on a mis en service le nouveau système. Aujourd'hui, il faut, semble-t-il, selon certaines caisses de chômage, environ 30 minutes pour créer un dossier contre 1 minute 30 dans l'ancien système. C'est une régression incompréhensible. L'argument juridique sur les délais de retard est lui aussi déconnecté de la réalité. Quand on dépend de ces prestations pour vivre, chaque jour compte. Les conséquences sont immédiates : loyers impayés, dettes, pression psychologique. Et pourtant, aucune compensation réelle n'existe. Les intérêts moratoires éventuels peuvent intervenir après des délais allant jusqu'à deux ans. Ce n'est pas une protection. Pendant ce temps, les personnes concernées doivent survivre. Comment ? Elles ne peuvent pas attendre décembre 2026 ni la fin d'un projet informatique. Je rappelle que des avertissements avaient été émis sur les risques du système. Aujourd'hui, nous en voyons les conséquences. Un seul mois de retard, vous le savez bien, peut déjà entraîner une résiliation de bail, selon la loi - un seul mois. Et pendant ce temps, au moindre manquement, un assuré est immédiatement sanctionné et perdra des jours d'indemnités. Où est l'égalité de traitement dans ce cas ? 
+Nous ne pouvons pas rester passifs. Ce qui est fait aujourd'hui est insuffisant. C'est pourquoi je demande instamment de simplifier et systématiser les avances pour répondre à l'urgence, en application de l'article 19 de la loi fédérale sur la partie générale du droit des assurances sociales (LGPA) ; de revenir provisoirement à l'ancien système Sipac - on me dit que c'est impossible, mais impossible n'est pas français ; de renforcer immédiatement les moyens humains - je pense qu'il faut des moyens provisoires humains pour résoudre ces problèmes informatiques qui ne peuvent plus attendre encore juin ou la fin de l'année ; d'envisager des indemnités dans les cas les plus graves, nonobstant l'article 26 de la LGPA ; et de présenter un rapport à la session de juin. C'est aujourd'hui qu'il faut que les assurés puissent toucher les prestations auxquelles ils ont droit, les anciens assurés comme les nouveaux, dans un contexte où le chômage augmente en Suisse, où 800 postes de travail ont été perdus dans l'Arc jurassien. 
+Au-delà de la technique, c'est la crédibilité de l'assurance-chômage qui est en jeu. La protection sociale ne doit pas dépendre d'un système informatique défaillant, elle doit être garantie pour toutes et tous, maintenant.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'aimerais tout d'abord commencer en vous assurant que le Conseil fédéral est conscient de la situation difficile dans laquelle se trouvent les personnes concernées et qu'il la déplore. La situation, de manière générale, se stabilise. Les caisses de chômage, soutenues par le SECO, travaillent sans relâche pour résorber le retard pris dans le traitement des dossiers de personnes nouvellement inscrites au chômage. Je vais maintenant répondre aux questions de manière groupée, par thématique.
+Tout d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'aimerais tout d'abord commencer en vous assurant que le Conseil fédéral est conscient de la situation difficile dans laquelle se trouvent les personnes concernées et qu'il la déplore. La situation, de manière générale, se stabilise. Les caisses de chômage, soutenues par le SECO, travaillent sans relâche pour résorber le retard pris dans le traitement des dossiers de personnes nouvellement inscrites au chômage. Je vais maintenant répondre aux questions de manière groupée, par thématique.
+Tout d'abord, le processus et la décision de déploiement : le projet Sipacfutur a fait l'objet d'une préparation minutieuse. Il était assorti d'un processus de validation formelle comprenant notamment la possibilité d'un retour à la version précédente - ce qu'on appelle un "rollback" -, ainsi que des procédures alternatives pour le déploiement du nouveau système de paiement. Celles-ci n'ont cependant pas dû être activées, puisque la mise en service échelonnée de Sipac 2.0 au début du mois de janvier de cette année s'est déroulée de manière stable sur le plan technique. Le 5 janvier, le comité de pilotage du projet a donc donné son feu vert pour une utilisation à l'échelon national dès le lendemain. Ce n'est qu'après le déploiement à l'échelon national que des dysfonctionnements, parfois importants, sont apparus. Les conséquences en ont été une prolongation des délais de traitement et une accumulation de tâches au sein des caisses de chômage, ce qui a causé des retards pour certains paiements. Ces dysfonctionnements techniques importants ont, depuis, été corrigés. Malgré les difficultés rencontrées après la mise en service, le système a fonctionné de bout en bout en février, et les paiements escomptés ont globalement pu être effectués. Le système est aujourd'hui stable. La vitesse de traitement n'a pas encore atteint le niveau souhaité, mais elle s'améliore progressivement. La lenteur du système crée une surcharge de travail pour les employés des caisses de chômage, qui doivent travailler souvent le soir ou le week-end pour assurer un paiement rapide des prestations. Je les remercie sincèrement pour cet engagement exceptionnel. Les optimisations techniques se poursuivront durant la phase dite de stabilisation - qu'on appelle "hypercare". Cette phase est prévue jusqu'au mois de juin de cette année.
+Concernant la gouvernance et les recommandations du Contrôle fédéral des finances (CDF) : le comité de pilotage du projet réunit des spécialistes du DEFR, du SECO et de ses prestataires externes, des représentants des caisses de chômage publiques et privées ainsi que des autorités cantonales. Sipacfutur étant un projet informatique clé de la Confédération, il a fait l'objet d'audits de la part du CDF, qui a publié, cela a été dit, au total six rapports à ce sujet. Le SECO a accepté toutes les recommandations et les a mises ou les met en oeuvre. Comme c'est généralement le cas pour les grands projets menés par la Confédération, une analyse structurée de la clôture du projet sera effectuée d'ici, probablement, la fin 2026.
+Quelle est la situation actuelle en matière de paiements ? Les paiements sont désormais en bonne voie. Pour garantir la rapidité des paiements, des mesures ont été mises en place pour les mois de janvier à avril 2026. Les caisses de chômage bénéficient d'une plus grande marge d'appréciation pour l'examen des dossiers. De plus, l'examen du droit des personnes récemment inscrites au chômage a été simplifié sur certains points. Depuis la mise en service de Sipac 2.0 le 6 janvier et jusqu'au 17 mars 2026, près de 1181 millions de francs ont été versés. Cela représente 95,7 pour cent du montant attendu selon les estimations. Il n'y a malheureusement pas de chiffres disponibles sur le nombre de personnes affectées par les délais de paiement plus longs. Chaque paiement dépend, en effet, d'un dossier individuel et de l'examen du droit aux indemnités. Indépendamment du système de paiement, l'expérience montre que l'examen, pour les nouvelles inscriptions, prend généralement plusieurs semaines et peut être nettement plus long dans des cas complexes. La raison en est que la personne assurée doit fournir de nombreux documents qui nécessitent, selon la situation, des clarifications auprès d'employeurs précédents, d'autres autorités ou de la personne assurée elle-même. Il existe donc des lenteurs qui sont liées au nouveau système de paiement, mais aussi d'autres durées de traitement plus longues qui ne sont pas liées au changement de système.
+Concernant les demandes de compensation, une caisse de chômage doit verser l'indemnité de chômage, en règle générale, dans le courant du mois suivant la période de contrôle écoulée, ainsi que le précise l'article 30 de l'ordonnance sur l'assurance-chômage (OACI).
+Toutefois, les caisses de chômage ont souvent effectué les versements plus vite que les exigences légales, ce qui reste d'ailleurs l'objectif. Par conséquent, au sens juridique, il n'est question de retard de paiement qu'au terme du mois suivant au plus tôt. La loi ne prévoit pas de compensation générale pour des lenteurs dans le système de versement de l'indemnité. Un versement tardif des prestations déclenche en premier lieu le mécanisme de l'intérêt moratoire. Ce droit à l'intérêt moratoire est réglé à l'article 26 de la loi fédérale sur la partie générale du droit des assurances sociales. Un tel intérêt moratoire n'est dû que lorsque deux années se sont écoulées depuis la naissance du droit.
+Concernant la possibilité des avances, le Conseil fédéral est conscient qu'un délai prolongé pour le traitement du versement de l'indemnité de chômage peut avoir des conséquences pour les personnes concernées et il le regrette. Selon l'article 31 de l'ordonnance sur l'assurance-chômage, une personne au chômage peut demander une avance à sa caisse de chômage si elle est confrontée à des difficultés financières avant le versement de son indemnité. 
+J'en viens maintenant au postulat Gysi 25.4737, "Combler durablement les lacunes dans les assurances sociales". L'objectif de ce postulat est de charger le Conseil fédéral d'exposer dans un rapport commun si une assurance générale du revenu permettrait de combler les lacunes du système suisse d'assurances sociales de manière durable et financièrement responsable. La raison invoquée est notamment la nécessité de combler les lacunes en matière de couverture en cas de maladie. Une assurance générale du revenu va toutefois bien au-delà des domaines de la maladie, des accidents et de l'invalidité : elle couvrirait également la perte de revenu due au chômage, à la maternité ou au service militaire. Le Conseil fédéral est conscient que les pertes de gain peuvent entraîner des charges personnelles et financières considérables pour les personnes concernées. Cela peut notamment être le cas lors de maladies chroniques ou d'évolution prolongée et difficilement prévisible de la maladie. À titre d'exemples, on peut mentionner le COVID long ou le syndrome de fatigue chronique.
+Pour le Conseil fédéral, il n'y a toutefois pas de lacune à combler dans le système suisse d'assurance sociale en matière de perte de gain en cas de maladie temporaire, car celle-ci est largement couverte par les assurances d'indemnités journalières. Comme l'ont montré divers avis et rapports, le système actuel, qui comprend différentes assurances sociales et assurances facultatives, garantit à une grande partie de la population active une protection suffisante en cas de maladie temporaire ou d'accident. Une modification de l'ordonnance sur l'assurance-accidents (OLAA) est en consultation. Elle vise à abaisser le seuil d'entrée afin de permettre à un plus grand nombre d'indépendants d'accéder à l'assurance-accidents facultative. 
+Les situations de perte de gain suite à des maladies chroniques ont quant à elles gagné en importance. Le Conseil fédéral est conscient que ces situations peuvent poser des défis majeurs pour les personnes concernées. Ici, l'assurance indemnités journalières en cas de maladie et l'assurance-invalidité (AI) jouent un rôle primordial. Il convient de relever que, dans une première phase, la perte de gain n'entraîne que peu d'incertitudes grâce à une bonne coordination des prestations, et ce, malgré l'absence d'assurance obligatoire d'indemnités journalières en cas de maladie.
+Il est en outre important qu'une annonce en temps utile soit faite auprès de l'AI. Cela permet de garantir que lorsque la perte de gain se prolonge de manière durable, les prestations de l'AI remplacent sans interruption celles de l'assurance d'indemnités journalières en cas de maladie si les conditions d'octroi sont remplies. De plus, le Conseil fédéral a été chargé, avec la motion von Falkenstein 23.3808, "Accélérer la procédure AI et garantir la sécurité financière des assurés durant celle-ci", de prendre des mesures pour accélérer la procédure AI et pour garantir la sécurité financière des personnes concernées. Sa mise en oeuvre est en cours d'examen.
+J'aborde maintenant la perte de revenu en cas de chômage. Les personnes ayant perdu leur emploi en raison d'une incapacité durable peuvent, en principe, être couvertes par l'assurance-chômage. Cette dernière garantit en effet une compensation convenable du manque à gagner. En cas d'annonce à l'AI ou auprès d'une autre assurance sociale, la personne peut bénéficier d'une indemnité pleine de l'assurance-chômage. Pour cela, elle doit notamment être disposée et en mesure de prendre un emploi convenable correspondant à 20 pour cent au moins d'un emploi à plein temps.
+Concernant les rapports disponibles et les travaux en cours, de nombreux documents de référence, analyses et rapports existent ou sont en cours d'élaboration concernant les supposées lacunes mentionnées par le présent postulat dans le domaine des indemnités journalières en cas de maladie. Il convient en outre de se référer à la motion Romano 21.4209, "Assurance perte de gain obligatoire en cas de maladie", adoptée par votre conseil et suspendue par la Commission de la sécurité sociale et de la santé publique du Conseil des États dans l'attente du rapport en réponse à son postulat visant un état des lieux en vue d'un développement de l'assurance perte de gain en cas de maladie.
+Le Conseil fédéral est, dans ce cadre, notamment chargé d'analyser les problèmes actuels, de discuter de différentes solutions possibles et d'en présenter les avantages et les inconvénients. Le rapport est en cours d'élaboration. Il sera adopté par le Conseil fédéral, vraisemblablement cet été.
+Enfin, le Conseil fédéral s'est récemment également penché à plusieurs reprises sur la couverture sociale de différents groupes professionnels. C'est le cas, par exemple, dans le rapport "Protection sociale des indépendants", en réponse au postulat Roduit 20.4141. En raison des travaux en cours dans ce domaine, ce rapport n'a pas approfondi la question de l'assurance d'indemnités journalières en cas de maladie. Aucune mesure n'a été jugée nécessaire dans les autres domaines de la sécurité sociale.
+En conclusion, on peut retenir que le système actuel d'assurance sociale, structuré de manière différenciée, garantit à une grande partie des personnes actives une protection suffisante en cas de perte de gain. Une assurance générale du revenu modifierait fondamentalement ce système et soulèverait d'importantes questions d'ordre systémique et financier, sans offrir de valeur ajoutée évidente. En ce qui concerne l'assurance d'indemnités journalières en cas de maladie, il convient de se référer au rapport existant et à ceux en cours d'élaboration. Tant que les résultats correspondants ne seront pas disponibles, le Conseil fédéral estime qu'un nouveau rapport ne serait pas pertinent.
+Au vu de ces considérations, je vous invite, au nom du Conseil fédéral, à rejeter ce postulat.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C'est pour cela, Monsieur le conseiller national Amoos, qu'à la fin de tout projet comme celui-ci, qui est un projet clé au niveau de la Confédération, il y aura une analyse de fond qui fera le point sur tout ce qui n'a pas bien fonctionné, que ce soit au SECO ou ailleurs dans les caisses de chômage. C'est ce que nous ferons à la fin, sur demande du Contrôle fédéral des finances, mais aussi certainement sur demande de la Délégation des finances.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -607,8 +661,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I19" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I19"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1362,6 +1416,89 @@
         <v>89</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>93</v>
+      </c>
+      <c r="I17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>99</v>
+      </c>
+      <c r="I19" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-20
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -349,20 +349,21 @@
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
-Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem </t>
+Bei der Massnahme 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
+Bei der Massnahme 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem En</t>
   </si>
   <si>
     <t xml:space="preserve">Ich spreche zu Block 4 für die SVP-Fraktion und dann auch noch zu meinen Minderheiten. In Block 4 geht es um die Bereiche Wissenschaft, Bildung und Kultur. Wir unterstützen im gesamten Block die Stossrichtung des Bundesrates.
-Bei der Massnahmen 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
-Bei der Massnahmen 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
+Bei der Massnahme 6 unterstützen wir die Minderheit I (Stettler) und bei der Massnahme 7 die Minderheit II (Stettler), die dem Entwurf des Bundesrates folgen wollen.
+Bei der Massnahme 9, "Massnahmen im Kulturbereich", folgen wir dem Beschluss des Ständerates und also dem Entwurf des Bundesrates. Den Minderheitsantrag Funiciello lehnen wir ab.
 Bei der Massnahme 11, "Kürzung der Subventionen für ausserschulische Kinder- und Jugendförderung", folgen wir dem Entwurf des Bundesrates. Die Kürzung dieser 1,5 Millionen Franken ist verkraftbar. Die Minderheitsanträge I (Zybach) und II (Gredig) lehnen wir dementsprechend ab.
 Bei den Massnahmen 27 und 30 folgen wir der Mehrheit der Finanzkommission und dem Beschluss des Ständerates.
 Ich komme zu meinen Minderheiten in diesem Block.
-Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
+Bei der Massnahme 26, "Stärkung der Nutzerfinanzierung der kantonalen Hochschulen", beantrage ich mit meiner Minderheit II, beim Entwurf des Bundesrates zu bleiben. Der Bund richtet unter anderem Grundbeiträge an die zehn kantonalen Universitäten und neun Fachhochschulen aus. Die Grundbeiträge betragen bei den Universitäten 20 Prozent bzw. bei den Fachhochschulen 30 Prozent des Gesamtbetrags der sogenannten Referenzkosten. Der Bundesrat sieht vor, den Satz bei den Universitäten um 1,6 Prozentpunkte und bei den Fachhochschulen um 3 Prozentpunkte zu senken. Der Gesamtbetrag der Referenzkosten wird vom Hochschulrat - Bund und Trägerkantone der Hochschulen - für eine BFI-Periode festgelegt. 
+2024 betrugen die jährlichen Studiengebühren an den zehn kantonalen Universitäten durchschnittlich 1445 Franken für Inländer bzw. 2510 Franken für Ausländer. An den Fachhochschulen waren es 1544 bzw. 2808 Franken pro Jahr. Bei Erträgen aus Studiengebühren von 179 Millionen Franken bei den kantonalen Universitäten und 141 Millionen Franken bei den kantonalen Fachhochschulen im Jahr 2022 können die Hochschulen mit der erwähnten Erhöhung der Studiengebühren zusätzliche Erträge von geschätzt 300 Millionen bei den Universitäten bzw. 200 Millionen Franken bei den Fachhochschulen generieren. Die Nutzerfinanzierung bzw. die Ausbildungsgebühren sind auf einem Niveau, das wirklich Anpassungen zulässt. Für uns ist diese Erhöhung durchaus zumutbar, denn höhere Gebühren befruchten auch die Bereitschaft, Teilpensen in der Wirtschaft anzunehmen, um das Studium zu finanzieren. Wenn man schaut, wie hoch die Ausbildungsgebühren bei Zweitausbildungen und berufsbegleitenden Weiterbildungen sind, ist diese Massnahme durchaus vertretbar.
 Ich komme zu meiner Minderheit II bei der Massnahme 28, "Kürzung des Bundesbeitrags für Innosuisse". Die Innosuisse fördert wissenschaftsbasierte Innovationen in der Schweiz durch finanzielle Beiträge, professionelle Beratung und Netzwerke. Über 90 Prozent dieses Finanzierungsbeitrages werden für die Förderung eingesetzt, der Rest deckt die Funktionskosten der Innosuisse. Die Bundesbeiträge sollen hier um rund 10 Prozent gekürzt werden; das sieht der Bundesrat vor. Die Umsetzungsmassnahmen sind plausibel und wurden nur geringfügig angepasst. Durch die Kürzung stehen den Hochschulen, vor allem den Fachhochschulen und den ETH, weniger Fördermittel zur Verfügung. Gleichzeitig beteiligen sich aber die Projektpartner aus der Wirtschaft mit einem höheren Anteil an den Projektkosten. Für die Finanzplanjahre 2027 bis 2029 stehen nach wie vor im Durchschnitt gut 300 Millionen Franken zur Verfügung. Ich beantrage Ihnen, dem Bundesrat zu folgen und diese zumutbare Einsparung von 10 Prozent zu unterstützen. Die Projektanforderungen sind sehr hoch, und bei einer gewissen Verzögerung dieser Projekte wird die Einsparung am Schluss ziemlich wenig Veränderung bringen. 
 Bei der Massnahme 29, "Aufhebung der Förderbestimmungen im Weiterbildungsgesetz", habe ich die Minderheit III eingereicht. Das Weiterbildungsgesetz ist seit 2017 in Kraft. Auch hier beantrage ich, dem Entwurf des Bundesrates zu folgen. Es geht in erster Linie um die Unterstützungsbeiträge in der Erwachsenenbildung. Der Weiterbildungsmarkt ist weitgehend privatwirtschaftlich organisiert und funktioniert zu weiten Teilen ohne staatliche Eingriffe. Gemäss einer Überprüfung der EFK aus dem Jahr 2021 ist unklar, für welche Leistungen die Organisationen der Weiterbildung überhaupt Beiträge erhalten und welche Wirkung diese Beiträge im gesamten Weiterbildungssystem entfalten. Natürlich ist es den Kantonen selbst überlassen, in welchem Umfang sie in Zukunft die Erwachsenenbildung fördern wollen. Daher unterstützen wir hier ebenfalls den Entwurf des Bundesrates.
-Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
+Abschliessend kann ich sagen, dass die SVP-Fraktion in Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
   </si>
   <si>
@@ -378,10 +379,10 @@
     <t xml:space="preserve">G</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12.[NB]September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12.[NB]September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der Zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds von AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
 Ziel des Vorhabens ist die umfassende Modernisierung der Organisation, der Geschäftsprozesse und der Informatiksysteme der ZAS, die als operatives Rückgrat der ersten Säule zentrale Register führt, die Finanzflüsse steuert und weltweit über eine Million Renten auszahlt. Die bestehenden Systeme seien technisch überaltert und stark fragmentiert, was die Automatisierung hemme, die Anpassung an gesetzliche Änderungen verteuere und die Datensicherheit gefährde. Ohne eine tiefgreifende Transformation wäre die ZAS laut eigenen Aussagen künftig nicht mehr in der Lage, die Qualität und Effizienz ihrer Leistungen sicherzustellen. 
 Das Programm ist ein Schlüsselprojekt der Bundesverwaltung und als solches eingestuft. Es umfasst rund zehn miteinander verknüpfte Projekte, die in drei Phasen bis ins Jahr 2032 laufen. Kernpunkte sind die Umgestaltung der Prozesse hin zu vier bereichsübergreifenden Querschnittsprozessen, die Migration auf die standardisierte IT-Architektur, die Integration marktgängiger Lösungen und die Einführung eines neuen Betriebsmodells. Damit sollen die Silostrukturen aufgebrochen, die Automatisierung vorangetrieben und die Interoperabilität mit anderen Projekten der ersten Säule gewährleistet werden.
 Die Transformation soll es ermöglichen, das wachsende Arbeitsvolumen ohne zusätzliche Stellen zu bewältigen. Das Einsparpotenzial wird auf bis zu 80 Vollzeitäquivalente über zehn Jahre geschätzt, wobei die tatsächliche Wirkung vom Automatisierungsgrad und der Stabilität der Prozesse abhängen wird. Neben Effizienzgewinnen werden kürzere Bearbeitungszeiten, eine höhere Datensicherheit und eine bessere Anpassungsfähigkeit an gesetzliche Änderungen erwartet. 

</xml_diff>

<commit_message>
Update debates data - 2026-04-29
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -166,10 +166,10 @@
 La disposition proposée par la majorité vise donc à inscrire cette collaboration dans la loi et à lui donner un cadre contraignant bienvenu. Elle correspond en outre à la recommandation formulée dans le rapport du Contrôle fédéral des finances sur la numérisation dans le premier pilier.
 Je vous invite dès lors à suivre la majorité de la commission et à rejeter la proposition de minorité de Courten.
 Une autre minorité de Courten vise, quant à elle, la suppression des règles relatives à la transparence des coûts ainsi qu'à la standardisation et à l'interopérabilité des systèmes d'information. Il s'agit toutefois de conditions essentielles, là aussi, pour que la Confédération puisse exercer efficacement sa fonction de pilotage, mais aussi sa fonction de surveillance. Le Contrôle fédéral des finances a d'ailleurs invité l'OFAS à utiliser de manière plus systématique ces instruments de pilotage existants, notamment en ce qui concerne les coûts informatiques. Là aussi, je vous invite à suivre la majorité de votre commission.
-Enfin, la minorité Reichsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
+Enfin, la minorité Rechsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
 Das Anliegen ist nachvollziehbar. Der Antrag der Minderheit würde jedoch unserer Meinung nach zu weit gehen. Es würde der Militär- und der Unfallversicherung Zugang zu allen Daten der ersten Säule gewähren. Wir dürfen nicht vergessen, dass es sich dabei teilweise um besonders sensible Daten handelt, insbesondere um Daten zur Gesundheit oder zur Invalidität. Das BSV hat in Zusammenarbeit mit den betroffenen Versichern ein Projekt lanciert. Ziel ist es, die Datenflüsse zu analysieren und die notwendigen rechtlichen Grundlagen zu klären, um einen gezielten und nachvollziehbaren Datenaustausch zu ermöglichen.
 Cependant, nous l'avons indiqué en commission, ce projet de discussions n'est pas encore suffisamment avancé à l'heure actuelle. J'ai demandé à l'OFAS de mettre la priorité sur ces discussions. Je crois que tout le monde est intéressé à clarifier la nature des données à transmettre pour faciliter et favoriser le travail de concertation entre les assurances, mais aussi pour aller en faveur des assurés. L'objectif est de pouvoir présenter une disposition correspondante, donc d'être pragmatique, en faisant une proposition au Conseil des États.
-Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Reichsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
+Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Rechsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-02
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -41,157 +41,109 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
-    <t xml:space="preserve">373984</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20260429</t>
+    <t xml:space="preserve">374600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260602</t>
   </si>
   <si>
     <t xml:space="preserve">N</t>
   </si>
   <si>
-    <t xml:space="preserve">Silberschmidt Andri</t>
+    <t xml:space="preserve">Götte Michael</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Depar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019.
+Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
+Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken. Hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
+Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
+Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
+Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
+Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf.
+Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
+Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
+Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
+Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
+Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">374870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schaffner Barbara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Ei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
+Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
+Das ist Steuersubventionitis, eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Sätze, Befreiungen oder Abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">374713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giacometti Anna</t>
   </si>
   <si>
     <t xml:space="preserve">RL</t>
   </si>
   <si>
-    <t xml:space="preserve">ZH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wir sprechen heute über das Bundesgesetz über Informationssysteme in den Sozialversicherungen (BISS), das es für die Digitalisierung der ersten Säule zwingend braucht. Vereinfacht gesagt geht es darum, dass Bürgerinnen und Bürger einen einfachen digitalen Zugriff auf die Informationen ihrer eigenen Sozialversicherungen erhalten, z. B. in der AHV. Heute besteht ein analoger Prozess, wenn man wissen will, wie viel man in die AHV einbezahlt hat, wie hoch die eigene Rente ausfallen wird und ob Beitr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wir sprechen heute über das Bundesgesetz über Informationssysteme in den Sozialversicherungen (BISS), das es für die Digitalisierung der ersten Säule zwingend braucht. Vereinfacht gesagt geht es darum, dass Bürgerinnen und Bürger einen einfachen digitalen Zugriff auf die Informationen ihrer eigenen Sozialversicherungen erhalten, z. B. in der AHV. Heute besteht ein analoger Prozess, wenn man wissen will, wie viel man in die AHV einbezahlt hat, wie hoch die eigene Rente ausfallen wird und ob Beitragslücken bestehen, die man noch begleichen will. Dieser Prozess dauert Tage, wenn nicht Wochen, und ist sehr komplex, weil sich die verschiedenen Durchführungsstellen untereinander abstimmen müssen. Dabei ist zu klären, wo eine Person überall AHV-Beiträge geleistet hat; anschliessend müssen die Daten zusammengeführt und der betroffenen Person in Form eines individuellen Kontoauszuges mitgeteilt werden. Mit dem BISS soll sich dies ändern. Künftig soll es in der ganzen Schweiz ein Portal geben, über das sich Bürgerinnen und Bürger bzw. versicherte Personen einloggen und per Knopfdruck alle relevanten Informationen abrufen können, d. h. etwa die voraussichtliche Rentenhöhe oder bestehende Beitragslücken.
-Weshalb braucht es nun dieses Gesetz? Grundsätzlich gilt, dass alles staatliche Handeln eine gesetzliche Grundlage benötigt. Die Regulierung der ersten Säule, d. h. der AHV, der IV, der EO und der Familienzulagen, liegt bereits heute beim Bund; die Leistungen sind national geregelt. Die Durchführung der ersten Säule ist jedoch bei den Kantonen und teilweise auch bei den Verbandsausgleichskassen angesiedelt. Es bestehen öffentliche und private Ausgleichskassen, die die erste Säule abwickeln. Für die Digitalisierung ergibt es jedoch wenig Sinn, wenn zehn oder zwanzig unterschiedliche Onlineportale bestehen. Dies hat auch die Eidgenössische Finanzkontrolle erkannt. Allen, die argumentieren, es brauche keine Lösung des Bundes, sondern eine der Kantone, sei der Bericht der EFK zur Lektüre empfohlen. Er fällt bezüglich der bisherigen Digitalisierungsanstrengungen der Ausgleichskassen leider wenig schmeichelhaft aus. Er zeigt, dass diese bisher hohe Kosten verursacht haben und dass keine gemeinsame Lösung erzielt werden konnte. Auch aus diesem Grund ist es im Interesse der Steuerzahler sinnvoller, ein einziges Portal statt mehrere Dutzend Portale zu betreiben.
-Übrigens machen wir im Gesundheitswesen derzeit genau das Gleiche: das Patientendossier, das neu "Gesundheitsdossier" heisst. Auch dort ist man zur Überzeugung gelangt, dass es in einem Land mit 9 Millionen Einwohnern keinen Wettbewerb bei der digitalen Grundinfrastruktur braucht. Bei der Autobahn und beim Schienennetz haben wir ja auch keinen Wettbewerb. So ist es auch hier sinnvoll, dass wir eine einheitliche Infrastruktur haben, die den Bürgerinnen und Bürgern einen einfachen Zugang zu ihren Vorsorgedaten gibt.
-Dieses relativ schlanke Bundesgesetz über Informationssysteme in den Sozialversicherungen setzt also gemeinsame Standards. Es übernimmt nicht die Aufgaben der Durchführungsstellen; es ist ganz klar und bewusst so gemacht, dass diese weiterhin bei den Kantonen bleiben. Aber es definiert in Zukunft Standards, wie man digital miteinander kommuniziert und wie die Versicherten entsprechend an die Informationen kommen, die sie betreffen. Wir haben jetzt gehört, dass dies langfristig weniger Kosten verursacht, weil der heutige papierlastige Prozess zwar nicht hinfällig, aber sicherlich abnehmen wird.
-Wir von der Mehrheit haben auch Folgendes gemacht: Wir haben selbstverständlich die Kritik aus der Vernehmlassung ernst genommen und wollen einen Passus ins Gesetz schreiben, mit dem den Durchführungsstellen explizit auch das Recht eingeräumt wird, in die Entwicklung dieser Plattform eingebunden zu werden. Das ist auch mir persönlich ein grosses Anliegen. Die Durchführungsstellen leisten in den Kantonen eine sehr wichtige und hervorragende Arbeit. Wir müssen sie einbeziehen, wenn auf nationaler Ebene eine solche Plattform entwickelt wird. Das soll nun explizit im Gesetz verankert werden. Ich danke auch den Durchführungsstellen, dass sie sich so engagiert haben.
-Das Bundesgesetz über Informationssysteme in den Sozialversicherungen ist auch eine Grundlage für ein digitales Vorsorgeportal. Wir regeln hier bewusst lediglich die staatliche Sozialversicherung und nicht die private, also nicht die zweite und die dritte Säule. Aber wenn wir einen guten digitalen Zugang zur ersten Säule ermöglichen, ist es viel einfacher, auch Portale zu bauen, die den Leuten eine Gesamtübersicht über die eigene Vorsorgesituation bieten. Dazu leistet dieses Gesetz ebenfalls einen wichtigen Beitrag.
-Ich bitte Sie, auf die Vorlage einzutreten und sie nicht an den Bundesrat zurückzuweisen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte gerne auf Artikel 22a und Artikel 22b eingehen, welche wir in der Kommission eingeführt haben. Es geht hier um das Steuerungs- und Mitwirkungsgremium. 
-Ich verstehe nicht, weshalb der Minderheitssprecher das ablehnt, zumal es der SVP-Fraktion in der Beratung ein Anliegen war, dass die kantonalen Durchführungsstellen in die Gesetzgebung einbezogen werden. Genau das stellen wir mit diesem Artikel 22a sicher. Wir stellen sicher, dass nicht ausschliesslich der Bund Standards festlegen kan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich möchte gerne auf Artikel 22a und Artikel 22b eingehen, welche wir in der Kommission eingeführt haben. Es geht hier um das Steuerungs- und Mitwirkungsgremium. 
-Ich verstehe nicht, weshalb der Minderheitssprecher das ablehnt, zumal es der SVP-Fraktion in der Beratung ein Anliegen war, dass die kantonalen Durchführungsstellen in die Gesetzgebung einbezogen werden. Genau das stellen wir mit diesem Artikel 22a sicher. Wir stellen sicher, dass nicht ausschliesslich der Bund Standards festlegen kann, sondern dass ein Gremium mit Vertreterinnen und Vertretern des BSV, der ZAS sowie der Durchführungsstellen verbindlich die Standards festlegt, die Digitalisierungsprojekte priorisiert und die Umsetzungsmodalitäten festlegt. Genau das, was die Minderheitssprecher moniert haben, haben wir in diesen Artikel 22a aufgenommen. Die Durchführungsstellen werden nicht nur angehört, sondern sind Teil des Steuerungs- und Mitwirkungsgremiums. 
-Artikel 22b ist wie auch Artikel 22a inspiriert von der Analyse der Eidgenössischen Finanzkontrolle, deren Bericht ich wirklich zur Lektüre empfehlen kann. Hier verlangen wir, dass das BSV verbindliche Vorgaben bei der Standardisierung, bei der Interoperabilität wie auch bei der einheitlichen Erfassung der IKT-Kosten macht. Ich denke, Absatz 1 Buchstabe a wird man im Ständerat streichen können, weil das im AHVG bereits geregelt ist. Die Buchstaben b und c sowie Absatz 2 sind hingegen nach wie vor wichtig; deshalb unterstützen wir diese auch. 
-Ich möchte noch kurz auf den Antrag der Minderheit Rechsteiner Thomas zu sprechen kommen, welchen wir ebenfalls unterstützen. Wenn ich den Antrag dieser Minderheit lese, steht klar geschrieben, dass die Unfallversicherung wie auch die Militärversicherung nur dort Zugriff auf die Daten haben, wo das zur Koordinierung der Leistungen notwendig ist. Es ist also nicht ein Blankoscheck, wie vorhin erwähnt wurde. Unserer Meinung nach ist es richtig, dass die Unfallversicherung wie auch die Militärversicherung Teil dieser Plattform sein können, weil wir sonst wieder neue Medienbrüche haben. Deshalb ist es aus unserer Sicht sehr wichtig, dass wir diese Minderheit Rechsteiner Thomas unterstützen. Wie gesagt, es ist kein Blankoscheck; es steht im Gesetz klar, dass nur dort Zugriff gewährt wird, wo es zur Koordination der Leistungen notwendig ist. 
-Das Datenschutzgesetz findet natürlich auch im Bundesgesetz über die Informationssysteme in den Sozialversicherungen Anwendung. Wenn jetzt gesagt wird, es gebe ja noch ein Datenschutzgesetz, dann ist das in der Tat so. Das Gesetz, das wir beraten, setzt das Datenschutzgesetz nicht ausser Kraft. In diesem Sinne finde ich die Begründung dagegen ein bisschen überzogen. Ich denke, wir sollten diese Minderheit unterstützen. Wenn man dann in dieser Gruppe, wo man das jetzt definieren will, weitergekommen ist, kann man im Ständerat noch die eine oder andere Präzisierung vornehmen. Ich denke, es ist wichtig, dass wir in diesem Gesetz alle Sozialversicherungen einbeziehen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechsteiner Thomas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M-E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich informiere Sie über die Diskussion in der Kommission, und zwar nicht nur zu den Artikeln mit Minderheitsanträgen, sondern auch zu den Artikeln, die von der Kommission in die Vorlage eingearbeitet wurden und zu denen kein Minderheitsantrag vorhanden ist. 
-Zuerst zum Antrag der Minderheit Aeschi zu Artikel 4 Absatz 2bis: Dieser Antrag wurde in der Abstimmung in der Kommission mit 16 zu 8 Stimmen abgelehnt. Demnach soll der Zugang zur elektronischen Kommunikation Personen verwehrt sein, welche </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich informiere Sie über die Diskussion in der Kommission, und zwar nicht nur zu den Artikeln mit Minderheitsanträgen, sondern auch zu den Artikeln, die von der Kommission in die Vorlage eingearbeitet wurden und zu denen kein Minderheitsantrag vorhanden ist. 
-Zuerst zum Antrag der Minderheit Aeschi zu Artikel 4 Absatz 2bis: Dieser Antrag wurde in der Abstimmung in der Kommission mit 16 zu 8 Stimmen abgelehnt. Demnach soll der Zugang zur elektronischen Kommunikation Personen verwehrt sein, welche keinen gültigen Aufenthaltsstatus in der Schweiz haben. Die Mehrheit der Kommission ist der Meinung, dass die Verankerung einer solchen Zugangsbeschränkung im Spezialgesetz BISS systemfremd ist. Weder die Zentrale Ausgleichsstelle noch die Durchführungsstellen sind die richtigen Ansprechpartner für den Abgleich des ausländerrechtlichen Status.
-Tatsächlich gibt es Menschen in der Schweiz, welche trotz illegalem Aufenthalt eine AHV-Nummer haben. Grundgedanke der Minderheit war, dass kein Zugang zu Leistungen möglich ist, wenn jemand im Status eines illegalen Aufenthalts hier ist. Da die Versicherten aber die Daten weiterhin auch analog bestellen können, wäre diese Einschränkung des elektronischen Zugriffs nicht wirkungsvoll. Für die Kommissionsmehrheit stand zudem der digitale Austausch im Zentrum und nicht die Prüfung des rechtlichen Aufenthaltsstatus. 
-Zu Artikel 5 Buchstabe abis: Dort ist zwar kein Minderheitsantrag vorhanden, aber ich mache dennoch kurz eine Erläuterung: Die Kommission hat da eingearbeitet, dass den versicherten Personen jährlich automatisch ein einfach verständlicher Auszug aus dem individuellen Konto der AHV zur Verfügung gestellt wird. Sie haben es gehört: Er soll jährlich und automatisch erfolgen und verständlich sein. Es liegt in der Handlungskompetenz des Bundesrates bzw. der Zentralen Ausgleichsstelle, wie das gemacht wird. Gedacht ist, dass alle Versicherten erfahren können, ob sie Beitragslücken haben, und diese gegebenenfalls schnell schliessen können. Dass diese Information zur Verfügung gestellt wird, erscheint der Kommission wichtig. 
-Ich komme zu Artikel 22a, zum Steuerungs- und Mitwirkungsgremium: Dort gibt es einen Antrag der Minderheit de Courten. Der entsprechende Antrag wurde in der Kommission mit 17 zu 8 Stimmen abgelehnt. Bei Artikel 22a wird von der Mehrheit der Umstand berücksichtigt, dass bisher noch zu unklar ist, wer beim BSV, bei der ZAS und bei den Durchführungsstellen genau welche Verantwortung hat. Deshalb will die Kommissionsmehrheit unter dem Abschnitt "Governancebestimmungen" das Steuerungs- und Mitwirkungsgremium verankern, dessen Zusammensetzung benennen und auch dessen Aufgaben aufführen. Sie will diese Massnahme auch aufgrund der Vernehmlassung und den Anhörungen einführen, bei welchen diese als notwendig erachtet wurde. 
-Bei Artikel 22b wurde der entsprechende Antrag der Minderheit de Courten mit 17 zu 8 Stimmen abgelehnt.
-Wie ich bei der Vorstellung des Geschäfts angetönt habe, hat die Kommission auch Punkte aus dem Bericht der Eidgenössischen Finanzkontrolle aufgenommen. Dort wurde reklamiert, dass bei den Durchführungsstellen grosse Intransparenz über die Kosten, einschliesslich der IT-Kosten, herrsche. Deshalb sollen gemäss Mehrheit neu die Verwaltungskosten nach einheitlichem Standard erfasst und ausgewiesen werden. Ergänzend dazu sollen auch Vorgaben zur Standardisierung der Schnittstellen und zur Interoperabilität gemacht werden. Damit werden Datenaustausch, Anbindung der Systeme, Effizienzgewinne und Transparenz möglich. 
-In den Artikeln 37a bis 37c geht es um die Änderung anderer Erlasse, konkret um das ASTG. Dort ist auch kein Minderheitsantrag vorhanden. Es geht um die elektronische Kommunikation der Versicherungen untereinander und mit den Versicherten. Artikel 37a hält die Anforderungen an die Plattform für die elektronische Kommunikation, welche die Versicherungen anbieten müssen, fest.
-Auch zu Artikel 49 Absatz 1bis ist kein Minderheitsantrag vorhanden, aber die Kommission hat hier eine Ergänzung beschlossen. Es geht hier um Verfügungen, welche der Versicherungsträger, zum Beispiel die AHV, IV oder die Militärversicherung (MV), schriftlich erlässt. Da sollen Medienbrüche verhindern werden. Konkret sollen diese Verfügungen der Sozialversicherungen auch elektronisch übermittelt werden können, wenn entweder die Pflicht zur elektronischen Kommunikation besteht oder diese verlangt wird. Gemäss Artikel 37c BISS hat die versicherte Person die Möglichkeit, die elektronische Kommunikation zu verlangen.
-Letztlich informiere ich Sie über die Minderheit Rechsteiner Thomas, übernommen von Hess Lorenz, welche erstmals bei Artikel 50a Absatz 1 Buchstabe b1 AHVG erwähnt wird. Der ursprüngliche Antrag in der Kommission wurde mit 16 zu 8 Stimmen abgelehnt. Die Mehrheit der Kommission will die automatische und vollständige Datenbekanntgabe zwischen AHV, IV, Unfallversicherung und Militärversicherung für die Koordination von Leistungen, die Abklärung der Versicherungspflicht, das Festsetzen der Versicherungspflicht, der Versicherungsprämien oder der Renten nicht ermöglichen. Gemäss der Minderheit ist diese gesetzliche Grundlage notwendig, damit der Austausch möglich ist, da heute die Datenanfrage in dieser Sache einzelfallweise und jeweils mit Begründung erfolgen muss und damit sehr aufwendig ist. Dieser Automatismus ist für die Kommissionsmehrheit aufgrund von Datenschutzbestimmungen noch nicht angebracht.
-Ihre Kommission hat dem BISS sowie den Änderungen im ATSG in der Gesamtabstimmung mit 17 zu 7 Stimmen zugestimmt. Gleichzeitig hat die Kommission auch der Abschreibung von zwei Motionen zugestimmt. Das ist einerseits die Motion 23.4041, "Sozialversicherung. Umfassende und einheitliche Rechtsgrundlage für das elektronische Verfahren schaffen (eATSG)" - BISS ist nun quasi die Umsetzung davon -, andererseits meine Motion 23.4435, "AHV endlich digitalisieren". Aus diesen Gründen bitte ich Sie im Namen der Kommission, die Mehrheitsanträge zu unterstützen, die beiden Motionen abzuschreiben und das Geschäft in der Schlussabstimmung anzunehmen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373974</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baume-Schneider Elisabeth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dans le cadre du traitement du présent projet de loi, plusieurs questions critiques ont été soulevées - je dois bien le dire - de manière légitime. Elles ont été débattues en commission et je peux vous assurer que pour le présent projet de loi un certain nombre de critiques a été pris en considération. 
-Premièrement, pourquoi une nouvelle loi ? Cet aspect a été discuté, débattu et critiqué lors de la consultation aussi bien par les cantons - cela a été dit - que par les organes d'exécution. Je p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dans le cadre du traitement du présent projet de loi, plusieurs questions critiques ont été soulevées - je dois bien le dire - de manière légitime. Elles ont été débattues en commission et je peux vous assurer que pour le présent projet de loi un certain nombre de critiques a été pris en considération. 
-Premièrement, pourquoi une nouvelle loi ? Cet aspect a été discuté, débattu et critiqué lors de la consultation aussi bien par les cantons - cela a été dit - que par les organes d'exécution. Je peux véritablement désormais affirmer que nous avons abordé et examiné de manière approfondie cette question, qui était légitime et nécessaire. Si la plateforme était intégrée dans la LPGA, elle devrait être utilisée par toutes les assurances sociales, y compris les assureurs maladie et - cela a été dit - possiblement par des assureurs privés, ce qui serait complexe. À l'inverse, l'absence de loi spécifique impliquerait d'introduire des références complexes et peu lisibles dans toutes les lois spéciales du premier pilier. 
-La minorité Aeschi demande le renvoi du projet en argumentant qu'une plateforme électronique décentralisée permettrait d'aboutir à une solution plus efficace et moins coûteuse. Néanmoins, le projet prend en considération les enseignements tirés d'autres projets numériques, notamment du dossier électronique du patient. Certaines solutions techniques doivent être gérées de manière centralisée, afin que l'ensemble des assurés, indépendamment de leur lieu de résidence ou encore indépendamment de leur employeur, disposent du même accès à leurs données. La plateforme centrale proposée constitue donc un élément clé du projet.
-Die Idee einer zentralen Plattform beim Bund löst bei den Durchführungsstellen teilweise Ängste aus. Klar ist jedoch, dass das Projekt nicht auf eine Zentralisierung der ersten Säule abzielt. Die dezentrale föderale Organisation der ersten Säule funktioniert gut und soll nicht infrage gestellt werden. Sie muss aber modernisiert werden, um mit den technologischen Entwicklungen Schritt zu halten. Weder das neue Gesetz noch die elektronische Plattform ersetzen zudem die bestehenden IT-Systeme der IV-Stellen und AHV-Ausgleichskassen.
-Ces dernières années, les assurances sociales, comme l'AVS, l'AI ou le régime des APG, ont numérisé un certain nombre de leurs processus. Toutefois, la communication électronique reste encore insuffisante et insuffisamment automatisée et standardisée aujourd'hui. La nouvelle loi fédérale sur les systèmes d'information des assurances (LSIAS) représente ainsi une avancée majeure dans la stratégie numérique de la Confédération et elle fait progresser la numérisation du premier pilier.
-La majorité de votre commission partage cette appréciation et propose ainsi l'entrée en matière sur le projet, par 16 voix contre 8. Une minorité de Courten demande de ne pas entrer en matière, alors qu'une minorité de Aeschi demande le renvoi du projet au Conseil fédéral afin de prendre en considération les demandes des cantons et des caisses cantonales de compensation. La LSIAS crée le cadre nécessaire pour une communication électronique sécurisée et efficace pour l'exécution des assurances sociales du premier pilier. Au coeur du projet figure donc la mise en place d'une plateforme électronique centrale qui est destinée aux offices AI, aux caisses de compensation AVS, aux autres instances administratives - on peut penser aux assurances-accidents ou encore aux services cantonaux des impôts - et surtout et en premier lieu aux assurés, c'est-à-dire à l'ensemble de la population.
-Für die Versicherten bietet die Plattform einen einfachen, sicheren und direkten Zugang zu ihren Daten der ersten Säule. Sie wird von der Zentralen Ausgleichsstelle verwaltet und ermöglicht es, eine automatisierte Simulation ihrer AHV-Rente durchzuführen; denn nur gut informierte Personen können fundierte Entscheidungen treffen.
-Les bénéficiaires de prestations AI ou encore d'allocations pour perte de gains pourront également disposer de la plateforme pour déposer des demandes de remboursement directement en ligne avec un traitement plus rapide. La plateforme permettra enfin aux autorités de transmettre en toute sécurité des documents tels que des décisions et des factures.
-Outre les dispositions prévues dans la LSIAS, le projet prévoit également des modifications de la loi fédérale sur la partie générale du droit des assurances sociales (LPGA). La plus importante concerne la communication électronique. L'ensemble des assurances sociales relevant de la LPGA, donc également l'assurance-chômage, l'assurance-maladie, l'assurance-accidents, seront tenues de communiquer entre elles par voie électronique. Les assurés resteront quant à eux libres de choisir. Ils pourront donc utiliser la nouvelle offre numérique ou alors continuer à échanger avec leur assurance par voie postale.
-Le projet présente également un potentiel d'économies, car il réduit les coûts administratifs grâce à la communication électronique. En effet, aujourd'hui, les fonds de compensation de l'AVS, de l'AI et des APG consacrent chaque année 25 millions de francs en frais postaux, auxquels s'ajoutent environ 10 millions pour couvrir les frais d'administration. Une partie de ces coûts pourra dès lors être économisée.
-Cela a été mentionné également, l'audit de la transformation numérique du premier pilier, réalisé par le Contrôle fédéral des finances, a été critique, disons-le de manière transparente. Je cite un élément qu'il a mentionné ; il parle effectivement de la nécessité de numérisation, en mentionnant qu'elle "ne pourra aboutir que si tous les acteurs concernés, et plus particulièrement l'OFAS et les organes d'exécution, coordonnent leur action dans un esprit de coopération." Grâce aux travaux en commission, cette coopération a été non seulement abordée, mais inscrite désormais dans la loi.
-En conclusion, le projet constitue une étape importante pour la modernisation du premier pilier. Il améliore l'accès des assurés à leurs informations. Ces informations leur appartiennent. Il simplifie également la communication entre les institutions et il rend l'exécution des assurances sociales plus efficace.
-Dès lors, je vous remercie de suivre la majorité, d'entrer en matière et de rejeter les propositions de minorité de Courten et Aeschi.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373986</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La commission a donc examiné de manière approfondie le projet de loi et les discussions ont permis d'aboutir à des adaptations qui permettent d'améliorer l'efficacité et la portée de la plateforme, ainsi que de la numérisation du premier pilier. Néanmoins, je vous proposerai de rejeter les différentes minorités.
-Premièrement, la minorité Aeschi prévoit que les personnes sans statut de séjour valable en Suisse n'auront pas accès à la plateforme. Or, il est important de le préciser : la plateforme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La commission a donc examiné de manière approfondie le projet de loi et les discussions ont permis d'aboutir à des adaptations qui permettent d'améliorer l'efficacité et la portée de la plateforme, ainsi que de la numérisation du premier pilier. Néanmoins, je vous proposerai de rejeter les différentes minorités.
-Premièrement, la minorité Aeschi prévoit que les personnes sans statut de séjour valable en Suisse n'auront pas accès à la plateforme. Or, il est important de le préciser : la plateforme centrale est conçue comme une plateforme purement informative, qui ne crée aucun droit à des prestations. Avec la plateforme, il est uniquement prévu de donner aux assurés un accès numérique facilité à leurs données de prévoyance. L'accès est d'ailleurs déjà limité. Il nécessite une identification par le biais d'une identité électronique reconnue, par exemple le numéro AVS. Dès lors, n'auront accès à la plateforme que les personnes qui ont ou qui avaient une assurance sociale en Suisse. Si ces conditions sont remplies, il est pratiquement impossible, d'un point de vue technique, d'en empêcher l'accès. De plus, la plateforme n'est pas le seul moyen d'accéder aux données de prévoyance ; la personne peut y accéder par le biais des caisses de compensation ou des offices AI cantonaux.
-Pour ces raisons, je vous invite à suivre la majorité et à rejeter la minorité Aeschi.
-Une minorité de Courten propose en outre de renoncer à créer un organe de pilotage et de participation pour les systèmes d'information à l'échelle nationale. Toutefois, la numérisation du premier pilier ne peut fonctionner que si la Confédération, c'est-à-dire l'OFAS et la Centrale de compensation, collabore étroitement et de manière durable avec les organes d'exécution, notamment dans le cadre d'instances communes. Dans ce contexte, des travaux sont en cours afin de clarifier et de préciser, avec l'ensemble des acteurs, les rôles, les compétences et les mécanismes de décision. C'est extrêmement important pour aboutir à des systèmes non seulement qui fonctionnent, mais qui créent aussi de la confiance.
-La disposition proposée par la majorité vise donc à inscrire cette collaboration dans la loi et à lui donner un cadre contraignant bienvenu. Elle correspond en outre à la recommandation formulée dans le rapport du Contrôle fédéral des finances sur la numérisation dans le premier pilier.
-Je vous invite dès lors à suivre la majorité de la commission et à rejeter la proposition de minorité de Courten.
-Une autre minorité de Courten vise, quant à elle, la suppression des règles relatives à la transparence des coûts ainsi qu'à la standardisation et à l'interopérabilité des systèmes d'information. Il s'agit toutefois de conditions essentielles, là aussi, pour que la Confédération puisse exercer efficacement sa fonction de pilotage, mais aussi sa fonction de surveillance. Le Contrôle fédéral des finances a d'ailleurs invité l'OFAS à utiliser de manière plus systématique ces instruments de pilotage existants, notamment en ce qui concerne les coûts informatiques. Là aussi, je vous invite à suivre la majorité de votre commission.
-Enfin, la minorité Rechsteiner Thomas souhaite permettre un accès automatisé aux données, par exemple de l'AI pour les assureurs-accidents. La question est sensible sur l'obligation de la motivation préalable et sur le volume ou sur la nature des données à transmettre.
-Das Anliegen ist nachvollziehbar. Der Antrag der Minderheit würde jedoch unserer Meinung nach zu weit gehen. Es würde der Militär- und der Unfallversicherung Zugang zu allen Daten der ersten Säule gewähren. Wir dürfen nicht vergessen, dass es sich dabei teilweise um besonders sensible Daten handelt, insbesondere um Daten zur Gesundheit oder zur Invalidität. Das BSV hat in Zusammenarbeit mit den betroffenen Versichern ein Projekt lanciert. Ziel ist es, die Datenflüsse zu analysieren und die notwendigen rechtlichen Grundlagen zu klären, um einen gezielten und nachvollziehbaren Datenaustausch zu ermöglichen.
-Cependant, nous l'avons indiqué en commission, ce projet de discussions n'est pas encore suffisamment avancé à l'heure actuelle. J'ai demandé à l'OFAS de mettre la priorité sur ces discussions. Je crois que tout le monde est intéressé à clarifier la nature des données à transmettre pour faciliter et favoriser le travail de concertation entre les assurances, mais aussi pour aller en faveur des assurés. L'objectif est de pouvoir présenter une disposition correspondante, donc d'être pragmatique, en faisant une proposition au Conseil des États.
-Au vu de ces considérations, je vous invite donc à suivre la majorité de votre commission et à rejeter la minorité Rechsteiner Thomas, qui sera reprise en fonction des propositions au Conseil des États.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piller Carrard Valérie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notre commission s'est penchée sur les différents articles qui composent ce projet de loi. Nous avons apporté plusieurs adaptations, acceptées à l'unanimité, afin de préciser certains éléments, notamment la collaboration entre l'administration, la Centrale de compensation et les organes d'exécution, comme à l'article 4 alinéa 2ter et à l'article 18, mais aussi pour apporter plus de sécurité juridique dans la gestion des canaux pour permettre des transferts de données de système d'information à s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notre commission s'est penchée sur les différents articles qui composent ce projet de loi. Nous avons apporté plusieurs adaptations, acceptées à l'unanimité, afin de préciser certains éléments, notamment la collaboration entre l'administration, la Centrale de compensation et les organes d'exécution, comme à l'article 4 alinéa 2ter et à l'article 18, mais aussi pour apporter plus de sécurité juridique dans la gestion des canaux pour permettre des transferts de données de système d'information à système d'information, comme à l'article 37a alinéa 2, lettres a, b et c, ou encore à l'article 49, où nous avons modifié l'alinéa 1bis afin de clarifier la communication de décisions qui peuvent être notifiées valablement par voie électronique non seulement aux personnes assurées, mais aussi à l'ensemble des parties, notamment les employeurs.
-En ce qui concerne les différentes propositions de minorité, à l'article 4 alinéa 2bis, la minorité Aeschi propose que l'accès à la plateforme ne soit pas accordé aux personnes résidant en Suisse sans statut de séjour valable. La commission a rejeté cette proposition, par 16 voix contre 8. Elle estime que l'instauration d'une telle restriction d'accès serait contraire au fonctionnement du système, qui est conçu comme une plateforme purement informative. Cette loi ne crée donc aucun droit à des prestations, mais rend simplement transparentes et accessibles les informations qui existent déjà. Aussi, les caisses de compensation ne sont pas les instances compétentes pour vérifier le statut au regard du droit des étrangers. Cette tâche relève de la compétence d'autres autorités.
-Pour ce qui est des propositions de minorité de biffer les articles 22a et 22b, ces deux articles s'inscrivent directement dans les conclusions du rapport du Contrôle fédéral des finances "Audit de la transformation numérique du 1er pilier" qui nous a été présenté en commission en février dernier. Dans ce rapport, plusieurs recommandations avaient été émises, notamment sur la gouvernance qui n'était pas suffisamment claire et sur le manque de transparence en matière de coûts. C'est pourquoi la majorité de la commission propose, à l'article 22a, que l'OFAS mette en place un organe de pilotage permanent à l'échelle nationale pour les systèmes d'information régis par la LSIAS, avec la participation des organismes d'exécution. Cet organe devra notamment définir les normes nationales, les modalités de mise en oeuvre et prioriser les projets.
-À l'article 22b, nous avons intégré les aspects de la transparence, de la standardisation et de l'obligation de rendre compte ; éléments qui faisaient défaut à ce projet de loi. Nous devons disposer en effet de données comparables et saisies uniformément, afin d'identifier les fausses incitations économiques. Il est donc essentiel que l'OFAS collecte ces données et les rende publiques.
-Nous vous invitons donc, pour ces deux articles, à soutenir les propositions de la majorité de la commission, qui ont été acceptées par 17 voix contre 8, et qui sont également soutenues par le Conseil fédéral.
-Concernant la minorité Rechsteiner Thomas à l'article 50a de la loi sur l'AVS, à l'article 97 de la loi sur l'assurance-accidents et à l'article 95a de la loi sur l'assurance militaire, cette proposition de minorité est un concept concernant la communication de données entre les différentes assurances mentionnées en vue de la coordination des prestations, de la détermination de l'assujettissement à l'assurance, de la fixation des primes d'assurance ou de la rente. Pour la minorité, c'est la seule façon d'assurer une communication électronique fluide et sans rupture de média. Pour que cela soit conforme à la loi sur la protection des données, il faut un ancrage légal. La majorité de la commission, qui, d'après ce que j'ai pu entendre, aurait évolué, ne souhaite pas pour le moment donner une carte blanche aux transferts de données, notamment du point de vue de la protection des données. Avec cette proposition de minorité, nous donnons à l'assurance-accidents un accès à l'ensemble des données du premier pilier.
-Pour réglementer cela de manière plus précise, il faudrait clarifier dans la loi quelles données sont transmises grâce à une cartographie des flux de données. Comme expliqué en commission par l'administration, l'examen actuel des flux de données avec les assureurs-accidents et l'assurance militaire prend un certain temps, mais ce délai pourrait suffire pour préciser les flux de données avant l'examen en deuxième lecture. Il vaut donc la peine, dans l'intérêt de la qualité de la loi, d'attendre la cartographie des flux de données, puis de procéder aux adaptations légales nécessaires. Nous avons par conséquent refusé cette proposition de minorité Rechsteiner Thomas, par 16 voix contre 8.
+    <t xml:space="preserve">GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
+Il disavanzo del bilancio straordinario è dovuto soprattutto ai contributi versati ai Cantoni per le persone con statuto di protezione S provenienti dall'Ucraina, 700 milioni, e al contributo unico alle FFS, 850 milioni, compensati in parte da entrate straordinarie della Banca nazionale svizzera.
+L'avanzo dell'amministrazione ordinaria raggiunge 1,2 miliardi di franchi, mentre la regola del freno all'indebitamento avrebbe consentito un deficit di 262 milioni di franchi. Ne risulta quindi un saldo strutturale positivo di 1,4 miliardi, nettamente superiore al valore previsto nel preventivo.
+Le entrate ordinarie superano il budget di 1,9 miliardi e il risultato dell'anno precedente di ben 3,3 miliardi. La crescita è dovuta soprattutto all'imposta federale diretta sulle imprese, che beneficia delle entrate temporanee dal Cantone di Ginevra per circa 1,5 miliardi di franchi.
+Anche l'imposta federale diretta sui redditi aumenta di 0,5 miliardi, mentre l'IVA aumenta di 700 milioni, grazie alla crescita dell'economia nominale e all'effetto ritardato dell'aumento dell'aliquota dal 2024. Le entrate dell'imposta preventiva, invece, risultano inferiori alle attese.
+Le spese totali sono aumentate del 4 percento e ammontano a 87,6 miliardi di franchi. 
+I principali aumenti riguardano la previdenza sociale, le finanze e imposte, i trasporti, l'istruzione e la ricerca e l'esercito.
+Nel 2025 il numero di posti nella Confederazione è cresciuto di 240 unità, più 0,6 per cento, mentre le spese per il personale sono aumentate di 79 milioni di franchi, soprattutto per il rincaro dell'1 per cento.
+Il debito netto scende leggermente a 140 miliardi di franchi. Il conto di ammortamento del debito Covid si riduce per la prima volta di circa 500 milioni, grazie al saldo strutturale positivo e alle entrate straordinarie, e ammonta a 26,3 miliardi di franchi. Il conto di compensazione rimane stabile a circa 20 miliardi di franchi.
+Nella seduta dell'11 e 12 maggio 2026, la commissione ha proceduto all'esame di dettaglio del consuntivo. Le sue quattro sottocommissioni hanno presentato le conclusioni delle rispettive analisi approfondite dei consuntivi dei singoli servizi federali realizzate nel corso del mese di aprile.
+Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla sua commissione i risultati delle tre verifiche relative al Consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del Fondo per l'infrastruttura ferroviaria e quella del Fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
+Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del Fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma ancora irrisolte. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
+Il Controllo federale delle finanze conferma che il consuntivo rispetta le prescrizioni legali e le regole del freno all'indebitamento previste dall'articolo 126 della Costituzione federale. Per questo motivo raccomanda all'Assemblea federale di approvare il conto annuale.
+Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
+La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
+Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
 </t>
   </si>
 </sst>
@@ -240,8 +192,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -608,27 +560,27 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -637,105 +589,22 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5"/>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
         <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6"/>
-      <c r="F6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-06-03
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -144,6 +144,73 @@
 Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
 La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
 Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jauslin Matthias Samuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen Halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
+Die GLP steht für Freiheit, Eigenverantwortung, Innovation und einen starken Rechtsstaat ein. Gerade deshalb unterstützen wir die Revision des Nachrichtendienstgesetzes. Freiheit und Sicherheit sind keine Gegensätze. Freiheit kann nur dort bestehen, wo Menschen sicher leben können, wo demokratische Institutionen geschützt werden und wo der Staat seine grundlegenden Funktionen wahrnehmen kann. Der Staat muss in der Lage sein, Bedrohungen frühzeitig zu erkennen und angemessen darauf zu reagieren.
+Die geopolitische Lage hat sich in den vergangenen Jahren deutlich verschärft. Spätestens seit dem russischen Angriffskrieg gegen die Ukraine ist klar geworden, dass Europa wieder verstärkt im Fokus nachrichtendienstlicher und hybrider Operationen steht. Die Schweiz bildet dabei keine Ausnahme, im Gegenteil: Als international vernetzter Wirtschafts-, Forschungs- und Diplomatiestandort ist sie besonders exponiert. Fremde Nachrichtendienste nutzen die Schweiz als Operationsraum, während gleichzeitig unsere Unternehmen, Hochschulen und Forschungsinstitutionen vermehrt Ziel von Spionageversuchen werden. Wer glaubt, die Schweiz könne sich diesen Entwicklungen entziehen, verkennt die Realität.
+Das angepasste Gesetz schafft die Voraussetzungen dafür, dass der Nachrichtendienst seinen Auftrag auch unter den Bedingungen des digitalen Zeitalters erfüllen kann. Kriminelle und feindliche Akteure nutzen verschlüsselte Kommunikationskanäle, globale Datennetze und moderne Technologien. Ein Nachrichtendienst, der auf Instrumenten des letzten Jahrhunderts basiert, kann diesen Herausforderungen nicht wirksam begegnen. Wer von den Sicherheitsbehörden erwartet, dass sie Gefahren erkennen und verhindern, muss ihnen auch die dafür notwendigen Mittel und Tools zur Verfügung stellen.
+Die Erfahrungen der letzten Jahre haben gezeigt, dass Radikalisierung häufig lange vor einer konkreten Tat sichtbar wird. Sicherheitsbehörden müssen deshalb die Möglichkeit haben, verdächtige Entwicklungen rechtzeitig zu erkennen und Risiken zu beurteilen. Es geht nicht darum, Menschen unter Generalverdacht zu stellen. Es geht darum, konkrete Gefahren frühzeitig zu erkennen.
+Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
+Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
+Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu diesem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wichtig sind auch klare Datenschutzgarantien im Gesetz - insbesondere, wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
+Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
+Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
+Für die GLP ist entscheidend, dass Sicherheit nicht auf Kosten der Freiheit erreicht wird. Die vorliegende Revision ermöglicht eine ausgewogene Balance zwischen wirksamer Gefahrenabwehr und dem Schutz der Grundrechte. Sie stärkt die Handlungsfähigkeit des Staates dort, wo dies notwendig ist, und setzt gleichzeitig klare Grenzen.
+Aus diesen Gründen tritt die GLP-Fraktion auf die Vorlage ein.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addor Jean-Luc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été : dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
+Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front - heureusement d'ailleurs - et les optimistes peuvent donc croire que "ça n'arrivera jamais". Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux ? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
+Le SRC, dans ce pays où l'on n'a pas la culture du renseignement, où l'on se méfie de toute zone grise, doit régater avec des homologues étrangers qui, eux, sont depuis longtemps sur le pied de guerre, et il doit le faire avec des moyens dramatiquement insuffisants et des procédures dont la lourdeur excessive fait parfois que certaines opérations nécessaires et urgentes sont simplement impossibles à mener.
+Pouvons-nous nous payer encore longtemps ce luxe de beau temps ? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
+Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission ? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
+La commission propose à son conseil d'apporter des modifications au projet de loi sur un certain nombre de points. J'en cite quelques-uns. D'abord, une extension des tâches du SRC en matière de recherche d'informations est nécessaire afin de couvrir également les activités d'influence du fait d'États étrangers dirigées contre l'ordre démocratique, le fonctionnement de l'État ou de la société. Il faut également étendre, en particulier, les compétences du service aux évènements relevant de la politique de sécurité qui se produisent dans le cyberespace. Le cyberespace est une notion que la commission a souhaité définir plus précisément en reprenant la formulation figurant dans la cyberstratégie nationale. Afin de rendre la lutte contre le financement du terrorisme et l'espionnage plus efficace, la commission préconise que le SRC puisse, en cas de graves menaces, collecter également des données auprès d'intermédiaires financiers et de négociants au moyen de mesures de recherche soumises à autorisation. Elle propose néanmoins que les conditions de cette obligation de fournir des renseignements soient définies plus clairement dans la loi fédérale sur le renseignement, sur la base des dispositions de la loi sur le blanchiment d'argent, afin de garantir la sécurité du droit.
+La commission estime en outre justifié qu'en cas d'urgence, le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif : si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
+La commission souhaite renforcer davantage la collaboration intercantonale et, dans ce sens, elle propose que les autorités d'exécution cantonales aient l'obligation de s'accorder réciproquement un accès en ligne aux données qu'elles ont obtenues sur la base de la loi sur le renseignement. La commission juge en effet insuffisant l'accès seulement facultatif que propose le Conseil fédéral. Par ailleurs, la commission demande que les services de renseignement cantonaux puissent également transmettre, avec l'accord du SRC, des données qu'ils ont reçues de celui-ci aux polices cantonales dans le cadre de mandats précis.
+La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances. - On voit déjà que c'est simple ! Je m'arrête deux secondes ici : c'est peut-être un objet de réflexion. - Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
+La commission a rejeté toutes les autres propositions d'amendement. À cet égard, le débat s'est cristallisé, entre autres, sur les points qui sont énumérés dans la seconde minorité Chollet, celle qui demande un renvoi du projet au Conseil fédéral.
+Il a d'abord été question de la problématique - je ne dirais pas "phare", mais enfin elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
+Sur ce point, la majorité de la commission, avec le Conseil fédéral d'ailleurs, considère que les dispositions proposées dans ce projet sont conformes à notre ordre juridique, tout en fournissant au SRC les compétences supplémentaires dont celui-ci a besoin pour notre sécurité.
+Un autre élément qui a suscité certains débats : ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, de ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
+Au bilan, la question se pose de savoir si, avec la révision telle que proposée par la commission, qui tient dans un volumineux document de 205 pages, nous aurons simplifié suffisamment les procédures pour garantir au SRC l'efficacité que les décideurs de ce pays attendent de lui, cela dans le respect de la sphère privée des citoyens - c'est évidemment un défi. La question lancinante des effectifs du SRC reste en outre sans la moindre réponse en ces temps d'allègements budgétaires.
+Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
 </sst>
@@ -192,8 +259,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I4" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -607,6 +674,64 @@
         <v>30</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-08
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -303,6 +303,31 @@
 Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">375897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260608</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moser Tiana Angelina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
+Die Resolution verdient eine besondere Aufmerksamkeit. Sie stammt nicht nur von einzelnen Organisationen, sondern von denjenigen, die die Folgen der PFAS-Belastung im Interesse und zum Schutz der Bevölkerung bewältigen müssen. Die Brunnenmeister beispielsweise sind zuständig für die Sicherung der Wasserqualität und die Versorgung der Bevölkerung. 
+PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
+Vor diesem Hintergrund ist die Stellungnahme des Bundesrates zu Frage 2 meiner Interpellation besonders bemerkenswert. Der Bundesrat anerkennt ausdrücklich den Nutzen des Human Biomonitoring für die Erfassung der Belastung der Bevölkerung. Genau solche Daten bräuchten wir, um Risiken frühzeitig zu erkennen und entsprechende Entwicklungen zu verfolgen. Umso weniger verständlich ist es, dass ausgerechnet dieses Instrument aus Spargründen eingestellt worden ist. Die Kosten des Human Biomonitoring stehen in keinem Verhältnis zu den Folgekosten der PFAS-Belastung, die sich, Sie haben es gehört, im Milliardenbereich bewegen. Auf das Monitoring zu verzichten, heisst, auf Wissen zu verzichten, das helfen könnte, gesundheitliche Risiken frühzeitig zu erkennen und Schäden zu begrenzen. 
+Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind wie gesagt nur die Beispiele zum Gewässer. 
+Es ist offensichtlich, dass es sich hier um eine schweizweite Herausforderung handelt. Wir stehen bei der PFAS-Thematik erst am Anfang, und gerade deshalb können wir es uns nicht leisten, auf Wissen zu verzichten. Entsprechend wichtig wäre eine Wiederaufnahme des Human Biomonitoring im Rahmen des Aktionsplans zur Reduktion der Ewigkeitschemikalien. Diese Einschätzung wurde im Übrigen auch von der Eidgenössischen Finanzkontrolle 2024 geteilt. Gerade angesichts der gesundheitlichen Risiken und der möglichen Folgekosten sowie der grossen Wissenslücken wäre das eine sehr wichtige Aussage, um auch das Vertrauen der Bevölkerung zu steigern. 
+In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -349,8 +374,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -851,6 +876,35 @@
         <v>46</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-09
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -328,6 +328,27 @@
 In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">376183</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parmelin Guy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
+Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
+C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -374,8 +395,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I9"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -905,6 +926,33 @@
         <v>52</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-11
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -67,17 +67,15 @@
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
 Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
-Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019.
-Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
-Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken. Hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
+Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken - hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
 Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
 Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
-Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf.
-Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
+Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf. Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
 Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
 Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
 Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
@@ -104,8 +102,8 @@
     <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
 Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
-Das ist Steuersubventionitis, eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
-Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Sätze, Befreiungen oder Abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Das ist "Steuersubventionitis", eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte -sätze, -befreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
 Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
 </t>
   </si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-14
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -63,23 +63,26 @@
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Depar</t>
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20.[NB]Februar 2026 darüber orientiert. Am 20.[NB]März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die</t>
   </si>
   <si>
     <t xml:space="preserve">Als Kommissionssprecher beginne ich gerne mit den Ausführungen zur Staatsrechnung 2025.
-Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20. Februar 2026 darüber orientiert. Am 20. März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11. und 12. Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
+Im Februar 2026 informierte der Bundesrat über das provisorische Rechnungsergebnis 2025; die Finanzkommission des Nationalrates wurde am 20.[NB]Februar 2026 darüber orientiert. Am 20.[NB]März 2026 verabschiedete der Bundesrat zuhanden des Parlamentes die Botschaft zur Staatsrechnung 2025. Ende April prüften die vier Subkommissionen die Abschlüsse der Departemente und ihrer Ämter vertieft. Vorgängig hatten die Departemente und Ämter schriftliche Fragen erhalten, die sie mündlich beantworteten. Die Mitglieder der Subkommissionen stellten daraufhin weitere Fragen, auf die, wo nötig, Antworten schriftlich nachgeliefert wurden. Am 11.[NB]und 12.[NB]Mai 2026 beriet die Finanzkommission die Staatsrechnung gemeinsam mit dem Bericht der Eidgenössischen Finanzkontrolle (EFK) als Gesamtkommission, und die Subkommissionen erstatteten Bericht über ihre jeweiligen Beratungen.
 Als departementsübergreifende Querschnittthemen wurden in den Subkommissionen insbesondere die Umsetzung der Querschnittkürzungen, mögliche Sparpotenziale im Hinblick auf das Entlastungspaket 2027, die Praxis bei externen Mandaten sowie die Entwicklung bei Spesenentschädigungen untersucht. Ein eigenständiges, wiederkehrendes Thema bildeten die Informatikprojekte der Bundesverwaltung. Mehrere Subkommissionen haben Fragen zu den Projekten des Bundesamtes für Informatik und Telekommunikation (BIT) gestellt; diese wurden in einer separaten Sitzung vertieft.
-Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. 
-Budgetiert war ein ursprünglich nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken - hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
-Einnahmeseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte.
-Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent, dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39 202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
+Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. 
+Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. Budgetiert war ursprünglich ein nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. 
+Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken, hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie wegen des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
+Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
+Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent; dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39[NB]202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
 Bei Skyguide weist das Covid-Darlehen des Bundes von 250 Millionen Franken aus dem Jahr 2021 per Ende 2025 noch einen Restbuchwert von 164 Millionen Franken auf. Die finanzielle Lage von Skyguide bleibt fragil und hängt wesentlich von der Umsetzung des Entlastungspakets 2027 sowie von der Genehmigung des Leistungsplans durch die Europäische Kommission ab.
-Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
+Zum Stand der Sonderrechnung: Die EFK wies ausdrücklich darauf hin, dass die Reserven im Bahninfrastrukturfonds spätestens 2028 vollständig aufgebraucht sein werden. Es braucht entsprechende Korrekturen. 
+Im Zusammenhang mit den ausserordentlichen Ausgaben hat die EFK betont, dass der Begriff der Ausserordentlichkeit sehr restriktiv anzuwenden sei. Die Kommission nimmt zudem zur Kenntnis, dass im Zusammenhang mit der Abschreibung der AT1-Anleihen durch die Credit Suisse Rechtsverfahren beim Bundesverwaltungsgericht und beim Bundesgericht hängig sind. Die EFK gelangte zusammen mit den zuständigen Anwälten zur Einschätzung, dass eine Rückstellung nicht notwendig sei. Sie wies aber darauf hin, dass sich die Beurteilung im weiteren Verfahren ändern könne. 
 Auch in den Subkommissionen wurden verschiedene Themen diskutiert. Dazu gehörten die stetig steigenden Kosten beim Eidgenössischen Personalamt, Fragen zur Transparenz bei den Informatikprojekten des Bundes, insbesondere beim BIT, das Investitionscockpit bei der Gruppe Verteidigung im Eidgenössischen Departement für Verteidigung, Bevölkerungsschutz und Sport und weitere Punkte. 
 Ich möchte mich im Namen der Kommission herzlich bei der Vorsteherin des Finanzdepartements, bei der Eidgenössischen Finanzverwaltung, bei der EFK sowie bei den Generalsekretariaten und den Ämtern bedanken, die uns umfassend und sehr präzise über die Staatsrechnung 2025 und die dazugehörigen Unterlagen Auskunft erteilt haben. 
-Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
+Ich komme zum Abstimmungsresultat: Die Finanzkommission hat die drei Bundesbeschlüsse einstimmig mit 24 Stimmen angenommen. 
+Ihre Finanzkommission beantragt Ihnen damit einstimmig, den Bundesbeschluss I über die Eidgenössische Staatsrechnung für das Jahr 2025, den Bundesbeschluss II über die Rechnung des Bahninfrastrukturfonds für das Jahr 2025 und den Bundesbeschluss III über die Rechnung des Nationalstrassen- und Agglomerationsverkehrsfonds für das Jahr 2025 zu genehmigen.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-06-15
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -72,7 +72,7 @@
 Die Staatsrechnung 2025 umfasst die Bundesrechnung und die Sonderrechnungen für den Bahninfrastrukturfonds (BIF) sowie den Nationalstrassen- und Agglomerationsverkehrsfonds (NAF). Bei Gesamteinnahmen von 87,8 Milliarden Franken und Gesamtausgaben von 87,6 Milliarden Franken schliesst die Bundesrechnung 2025 mit einem Finanzierungsüberschuss von 259 Millionen Franken ab. Nach mehreren Jahren mit Defiziten infolge Covid-Pandemie und Ukraine-Konflikt ist dies das erste positive Rechnungsergebnis seit dem Jahr 2019. Das ist erfreulich. Es wäre jedoch falsch, dieses Ergebnis als Normalisierung zu deuten. 
 Im ordentlichen Haushalt verzeichnet der Bund einen Finanzierungsüberschuss von 1,185 Milliarden Franken. Die Schuldenbremse hätte konjunkturbedingt ein ordentliches Defizit von 262 Millionen Franken zugelassen. Der strukturelle Finanzierungssaldo gemäss Schuldenbremse belief sich damit auf 1,4 Milliarden Franken. Budgetiert war ursprünglich ein nahezu ausgeglichener Haushalt. Die Verbesserung ist hauptsächlich auf eine sehr dynamische Einnahmenentwicklung zurückzuführen. 
 Im ausserordentlichen Haushalt hingegen überstiegen die Ausgaben die Einnahmen um 925 Millionen Franken, hauptsächlich wegen der Globalzahlung an die Kantone für Schutzsuchende aus der Ukraine von 700 Millionen Franken sowie wegen des einmaligen Kapitalzuschusses an die SBB von 850 Millionen Franken. Kompensiert wurde dies teilweise durch Zusatzausschüttungen der Nationalbank von 333 Millionen Franken und die Sonderzuweisung aus nicht umgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Der strukturelle Überschuss wurde dem Amortisationskonto gutgeschrieben und ermöglicht erstmals seit der Corona-Pandemie einen Abbau des Fehlbetrags um 521 Millionen Franken. Der verbleibende negative Saldo des Amortisationskontos beträgt 26,3 Milliarden Franken, der bis spätestens 2039 ausgeglichen werden muss. Die Nettoverschuldung hat leicht abgenommen und beträgt 140,1 Milliarden Franken. 
-Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundessteuergesetz, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
+Einnahmenseitig stiegen die ordentlichen Einnahmen gegenüber dem Vorjahr um 3,3 Milliarden Franken, mit einem besonders starken Wachstum bei der direkten Bundessteuer; das sind plus 2,3 Milliarden bzw. plus 7,7 Prozent. Dabei spielten temporäre Mehreinnahmen aus dem Kanton Genf von rund 1,5 Milliarden Franken eine zentrale Rolle. Hintergrund ist, dass der Kanton Genf aufgrund eines Problems im kantonalen IT-System die direkte Bundessteuer für mehrere Steuerperioden nicht fristgerecht in Rechnung gestellt hat - ein Verstoss gegen das Bundesgesetz über die direkte Bundessteuer, der durch die EFK gerügt wurde und dann im Herbst 2025 bereinigt werden konnte. Ebenfalls bemerkenswert ist die erste Gewinnausschüttung der Nationalbank seit 2022 im Umfang von 1 Milliarde Franken. Die Kommission betont, dass diese Sondereffekte nicht struktureller Natur sind und in den folgenden Jahren abflachen werden. 
 Ausgabenseitig stiegen die ordentlichen Ausgaben um 3,5 Prozent; dies ist ein deutlich stärkeres Wachstum als das normale Wirtschaftswachstum, welches mit 1,7 Prozent ausgewiesen wird. Hierin liegt der zentrale Befund der Kommission: Zum ersten Mal seit der Einführung der Schuldenbremse lagen die ordentlichen Ausgaben um rund 200 Millionen Franken über dem Budget. Es gab keine Kreditreste mehr im ordentlichen Haushalt. Die Ausgaben für die soziale Wohlfahrt machten mit rund 30 Milliarden Franken mehr als ein Drittel der Gesamtausgaben aus. Die Ausgaben für die Sicherheit stiegen auf 7,2 Milliarden Franken. Der Personalbestand wuchs um 240 Stellen auf 39[NB]202 Vollzeitstellen. Die Personalausgaben stiegen somit auf 79 Millionen Franken.
 Die EFK hat die Staatsrechnung geprüft und festgestellt, dass die Jahresrechnung des Bundes den gesetzlichen Vorgaben sowie den Bestimmungen der Schuldenbremse gemäss Artikel 126 der Bundesverfassung entspricht. Die EFK empfiehlt der Bundesversammlung, die Jahresrechnung zu genehmigen, Kreditüberschreitungen von 1,86 Milliarden Franken zu genehmigen sowie die Bildung neuer Reserven von 569 Millionen Franken zu beschliessen. Aus dem Prüfbericht der EFK hebt die Kommission folgende kritische Punkte hervor: 
 Beim Bundesamt für Zoll und Grenzsicherheit ist die Nachvollziehbarkeit der LSVA-Einnahmen über den European Electronic Toll Service (EETS) sowie der Einnahmen aus der E-Vignette weiterhin stark eingeschränkt. Mängel im IT-System und im internationalen Kontrollsystem bestehen seit Jahren. Die EFK musste die Risiken durch Falschdarstellungen mit aufwendigen Zusatzprüfungen abdecken.
@@ -98,16 +98,17 @@
     <t xml:space="preserve">ZH</t>
   </si>
   <si>
-    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "Steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Ei</t>
   </si>
   <si>
-    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
+    <t xml:space="preserve">Frau Bundesrätin Keller-Sutter hat es vorhergesehen: Ich komme jetzt mit einem Postulat, das mehr Daten fordert, im Sinne von "Steter Tropfen höhlt den Stein". Das ist ein Tropfen zusätzlich zu jenen, die seit 20 bis 25 Jahren stetig den Stein höhlen.
 1997 hat die Eidgenössische Finanzverwaltung erstmals im Rahmen des Subventionsberichtes über Steuervergünstigungen berichtet. Bei 46 untersuchten Subventionen wurden Einnahmeausfälle von 2,6 Milliarden Franken geschätzt. 2005 identifizierte die Eidgenössische Finanzkontrolle 121 Abweichungen von der Steuernorm, die potenziell als Steuersubventionen zu kategorisieren sind. Sie empfahl der Finanzverwaltung in ihrem Bericht mehr Transparenz, eine breitere Erfassung und eine öffentliche Publikation der Zahlen. 2011 versuchte die Studie der Eidgenössischen Steuerverwaltung "Welche Steuervergünstigungen gibt es beim Bund?" diese Frage zu beantworten. Die Antwort lautete: rund 100 Vergünstigungen mit Steuerausfällen in der geschätzten Höhe von 25 Milliarden Franken. Das ist bereits eine enorme Summe, und dies, obwohl in den Tabellen aus dem Bericht zur Studie zahlreiche Fragezeichen anstelle von Beträgen enthalten waren, die nicht geschätzt werden konnten und in diesen 25 Milliarden Franken entsprechend noch nicht enthalten sind. Dieser Betrag war also schon 2011 deutlich höher.
 Seither sind die versteckten Subventionen nicht kleiner geworden, sondern es wurden weitere Vergünstigungen eingeführt und kaum eine abgeschafft. Immerhin war der Bundesrat letztes Jahr bereit, ein Postulat der Finanzkommission anzunehmen und ein Update des Berichtes von 2011 vorzulegen, wenn auch unter dem Vorbehalt, dass es schwierig sei, Daten zu Steuersubventionen von den Kantonen einzufordern. Jetzt hat Frau Bundesrätin Keller-Sutter eben gesagt, sie könne das aufgrund des Bundesstatistikgesetzes. Das hat sie auch in der Antwort zur Motion Feller 24.3514 so begründet. Es leuchtet mir einfach nicht ein, dass man es beim einen kann, beim anderen nicht. Dabei ist zu vermuten, dass Steuersubventionen massiv höher liegen als offen ausgewiesene Subventionen. Während wir in der Budgetdebatte jeden Franken der offen ausgewiesenen Subventionen zweimal umdrehen, werden Steuersubventionen laufend ausgebaut, auch bei Fördertatbeständen, die die Grünliberale Fraktion inhaltlich unterstützt, aktuell zum Beispiel die LSVA-Befreiung für Elektrolastwagen. Auch da müssen wir uns selber an der Nase nehmen.
 Das ist "Steuersubventionitis", eine schleichende Krankheit, bei der das System immer mehr Ausnahmen produziert - jede einzelne gut begründet -, was im Gesamtbild zu einer Verzerrung der Steuer- und Subventionssysteme führt, die niemand bewusst so beschlossen hat. 
-Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte -sätze, -befreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
-Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
+Mit meinem Postulat fordere ich nichts anderes als Transparenz. Was der Staat durch Steuerausnahmen, reduzierte Steuersätze, Steuerbefreiungen oder -abzüge auf der Einnahmenseite verschenkt, taucht in keiner Rechnung auf. Es ist unsichtbar, unkontrollierbar und entzieht sich dem Budgetentscheid des Parlamentes. Still und heimlich können sich Giesskannensubventionen entwickeln, die niemand mehr hinterfragt. 
+Nachdem wir also im Rahmen des Entlastungspakets 27 vor allem die Ausgaben unter die Lupe genommen haben, ist es nun Zeit, auch die andere Seite der Medaille zu beleuchten. 
+Ich bitte Sie deshalb: Unterstützen Sie dieses Postulat.
 </t>
   </si>
   <si>
@@ -287,21 +288,21 @@
     <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégique</t>
   </si>
   <si>
-    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été : dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
-Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front - heureusement d'ailleurs - et les optimistes peuvent donc croire que "ça n'arrivera jamais". Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux ? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
+    <t xml:space="preserve">Voilà plus de quatre ans qu'une guerre meurtrière fait rage en Ukraine, aux portes de l'Europe. Les empires sont en train de tailler en pièces ce qui subsistait de l'ordre fragile que les vainqueurs de la Deuxième Guerre mondiale avaient mis en place. Une coalition israélo-américaine mène au Proche-Orient de multiples opérations qui nous exposent quotidiennement au risque d'une escalade majeure et menacent d'ores et déjà nos intérêts et notre approvisionnement en certaines ressources stratégiques. Un potentiel de radicalisation violente demeure, notamment en lien avec l'islamisme. Bref, le monde est redevenu ou resté ce qu'il a toujours été[NB]: dangereux. Et pourtant, la Suisse dort toujours du sommeil du juste.
+Sans même parler de modernisation, le simple équipement complet de notre armée est en panne, faute de la volonté d'une majorité de lui donner les moyens dont elle a besoin pour garantir notre sécurité. Mais le canon ne tonne pas à la frontière. Nos soldats ne sont pas au front, heureusement, d'ailleurs, et les optimistes peuvent donc croire que ça n'arrivera jamais. Mais il en est qui, eux, ne peuvent pas croire cela. Ils ne sont pas simplement en réserve, mais déjà à l'engagement. Ils le sont toujours, d'ailleurs. Ils sont notre première ligne de défense. Ils sont les yeux et les oreilles du pays. Eux[NB]? Ce sont les collaborateurs du Service de renseignement de la Confédération (SRC).
 Le SRC, dans ce pays où l'on n'a pas la culture du renseignement, où l'on se méfie de toute zone grise, doit régater avec des homologues étrangers qui, eux, sont depuis longtemps sur le pied de guerre, et il doit le faire avec des moyens dramatiquement insuffisants et des procédures dont la lourdeur excessive fait parfois que certaines opérations nécessaires et urgentes sont simplement impossibles à mener.
-Pouvons-nous nous payer encore longtemps ce luxe de beau temps ? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
-Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission ? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
+Pouvons-nous nous payer encore longtemps ce luxe de beau temps[NB]? Le Conseil fédéral croit que non. La majorité de notre Commission de la politique de sécurité, non plus. Personne, aujourd'hui, n'ose vraiment parler de renforcer les effectifs du SRC, pourtant dérisoires en comparaison internationale.
+Mais parlons déjà des compétences du service. L'objet de ce projet est de les renforcer, avec pour objectif de permettre au SRC de mieux remplir ses missions, notamment dans le domaine préventif. Qu'est-il donc ressorti des travaux de notre commission[NB]? Sa majorité estime qu'il est urgent d'agir, en particulier en matière de détection précoce et de lutte contre les menaces résultant du terrorisme, de l'extrémisme violent, de l'espionnage et des cyberattaques. Elle préconise pour cela de renforcer les compétences du SRC. Afin de préserver l'équilibre entre protection des droits fondamentaux et protection contre les menaces, cet élargissement des compétences doit évidemment s'accompagner d'un renforcement de la surveillance indépendante.
 La commission propose à son conseil d'apporter des modifications au projet de loi sur un certain nombre de points. J'en cite quelques-uns. D'abord, une extension des tâches du SRC en matière de recherche d'informations est nécessaire afin de couvrir également les activités d'influence du fait d'États étrangers dirigées contre l'ordre démocratique, le fonctionnement de l'État ou de la société. Il faut également étendre, en particulier, les compétences du service aux évènements relevant de la politique de sécurité qui se produisent dans le cyberespace. Le cyberespace est une notion que la commission a souhaité définir plus précisément en reprenant la formulation figurant dans la cyberstratégie nationale. Afin de rendre la lutte contre le financement du terrorisme et l'espionnage plus efficace, la commission préconise que le SRC puisse, en cas de graves menaces, collecter également des données auprès d'intermédiaires financiers et de négociants au moyen de mesures de recherche soumises à autorisation. Elle propose néanmoins que les conditions de cette obligation de fournir des renseignements soient définies plus clairement dans la loi fédérale sur le renseignement, sur la base des dispositions de la loi sur le blanchiment d'argent, afin de garantir la sécurité du droit.
-La commission estime en outre justifié qu'en cas d'urgence, le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif : si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
+La commission estime en outre justifié qu'en cas d'urgence le directeur du SRC puisse désormais ordonner l'intrusion dans des systèmes informatiques à l'étranger, procédure similaire à celle applicable aux mesures de recherche soumises à autorisation (MRSA), sans attendre l'autorisation du chef du DDPS, avec toutefois un correctif[NB]: si le chef du DDPS refuse ensuite de poursuivre la mesure, le SRC doit se charger de la destruction immédiate des données obtenues.
 La commission souhaite renforcer davantage la collaboration intercantonale et, dans ce sens, elle propose que les autorités d'exécution cantonales aient l'obligation de s'accorder réciproquement un accès en ligne aux données qu'elles ont obtenues sur la base de la loi sur le renseignement. La commission juge en effet insuffisant l'accès seulement facultatif que propose le Conseil fédéral. Par ailleurs, la commission demande que les services de renseignement cantonaux puissent également transmettre, avec l'accord du SRC, des données qu'ils ont reçues de celui-ci aux polices cantonales dans le cadre de mandats précis.
-La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances. - On voit déjà que c'est simple ! Je m'arrête deux secondes ici : c'est peut-être un objet de réflexion. - Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
+La commission souhaite encore clarifier la répartition des compétences de surveillance entre la Délégation des Commissions de gestion, l'Autorité de surveillance indépendante des activités de renseignement (AS-Rens) et le Contrôle fédéral des finances - on voit déjà que c'est simple[NB]; je m'arrête deux secondes ici, c'est peut-être un objet de réflexion. Elle propose donc d'apporter les précisions nécessaires dans diverses dispositions. Enfin, la commission est favorable à ce que le DDPS veille à la mise en oeuvre des recommandations de l'AS-Rens, mais propose que le chef du DDPS, et non pas le Conseil fédéral in corpore, soit autorisé, dans des cas exceptionnels justifiés, à décider le cas échéant de ne pas mettre en oeuvre une recommandation.
 La commission a rejeté toutes les autres propositions d'amendement. À cet égard, le débat s'est cristallisé, entre autres, sur les points qui sont énumérés dans la seconde minorité Chollet, celle qui demande un renvoi du projet au Conseil fédéral.
-Il a d'abord été question de la problématique - je ne dirais pas "phare", mais enfin elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
+Il a d'abord été question de la problématique - je ne dirais pas "phare", mais, enfin, elle a suscité passablement de débats en commission - de l'exploration du réseau câblé, en lien notamment avec un arrêt récent du Tribunal administratif fédéral.
 Sur ce point, la majorité de la commission, avec le Conseil fédéral d'ailleurs, considère que les dispositions proposées dans ce projet sont conformes à notre ordre juridique, tout en fournissant au SRC les compétences supplémentaires dont celui-ci a besoin pour notre sécurité.
-Un autre élément qui a suscité certains débats : ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, de ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
+Un autre élément qui a suscité certains débats[NB]: ce qu'on pourrait appeler la police politique. Certains s'inquiètent, pas seulement à gauche, que ce qui devrait rester l'exception aille au-delà des critères actuels de lutte contre l'espionnage et contre l'extrémisme violent.
 Au bilan, la question se pose de savoir si, avec la révision telle que proposée par la commission, qui tient dans un volumineux document de 205 pages, nous aurons simplifié suffisamment les procédures pour garantir au SRC l'efficacité que les décideurs de ce pays attendent de lui, cela dans le respect de la sphère privée des citoyens - c'est évidemment un défi. La question lancinante des effectifs du SRC reste en outre sans la moindre réponse en ces temps d'allègements budgétaires.
-Toujours est-il qu'avec 21 voix contre 4, la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
+Toujours est-il qu'avec 21 voix contre 4 la commission vous propose de rejeter la minorité Chollet demandant de ne pas entrer en matière sur ce projet. Par 17 voix contre 6 et 2 abstentions, elle vous propose de rejeter la minorité Chollet demandant le renvoi du projet au Conseil fédéral, car qu'il est urgent que les modifications proposées puissent être mises en oeuvre.
 </t>
   </si>
   <si>
@@ -348,6 +349,39 @@
     <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
 Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
 C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376778</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herzog Eva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Staatsrechnung 2025 des Bundes schliesst mit einem Finanzierungsüberschuss von 259 Millionen Franken. Sie fällt damit deutlich besser aus als erwartet; veranschlagt war ein Defizit von 815 Millionen Franken. Der negative ausserordentliche Finanzierungssaldo von 926 Millionen Franken wurde durch den positiven ordentlichen Finanzierungssaldo von 1,185 Milliarden Franken mehr als ausgeglichen. Dies ist vor allem auf temporär höhere Gewinnsteuereinnahmen aus dem Kanton Genf im Umfang von 1,5 Mil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Staatsrechnung 2025 des Bundes schliesst mit einem Finanzierungsüberschuss von 259 Millionen Franken. Sie fällt damit deutlich besser aus als erwartet; veranschlagt war ein Defizit von 815 Millionen Franken. Der negative ausserordentliche Finanzierungssaldo von 926 Millionen Franken wurde durch den positiven ordentlichen Finanzierungssaldo von 1,185 Milliarden Franken mehr als ausgeglichen. Dies ist vor allem auf temporär höhere Gewinnsteuereinnahmen aus dem Kanton Genf im Umfang von 1,5 Milliarden Franken zurückzuführen. 
+Die ordentlichen Einnahmen fielen insgesamt um 1,9 Milliarden Franken bzw. 2,2 Prozent höher aus als budgetiert und um 3,3 Milliarden Franken höher als im Vorjahr. Zugleich lagen die ordentlichen Ausgaben des Bundes 2025 erstmals seit der Einführung der Schuldenbremse im Jahr 2003 über dem Budgetwert. Dies ist unter anderem auf den Nachtragskredit für Horizon Europe zurückzuführen. Der ordentliche Finanzierungssaldo war positiv. Aus der Differenz ergibt sich ein struktureller Überschuss von 1,4 Milliarden Franken. In diesem Umfang war der ordentliche Finanzierungssaldo höher als von der Schuldenbremse vorgegeben. 
+Nennenswert sind im ausserordentlichen Haushalt die Mehreinnahmen aus der Zusatzausschüttung der Schweizerischen Nationalbank von 333 Millionen Franken und die budgetierte Sonderzuweisung der SNB aus den nicht ausgetauschten Banknoten der sechsten Serie von 237 Millionen Franken. Die beiden grössten Posten auf der Ausgabenseite sind die ausserordentlichen Ausgaben für die Schutzsuchenden aus der Ukraine sowie der einmalige Kapitalzuschuss an die SBB von 850 Millionen Franken, die ursprünglich für 2024 budgetiert waren.
+Weitere wichtige Kennzahlen: Erstmals seit der Corona-Pandemie konnte der Fehlbetrag des Amortisationskontos um 500 Millionen Franken reduziert werden. Neu beläuft sich der Fehlbetrag auf 26,3 Milliarden Franken. Das Ausgleichskonto hat unverändert einen positiven Stand von rund 20 Milliarden Franken. Die Nettoverschuldung hat 2025 leicht abgenommen und beträgt neu 140,1 Milliarden Franken. Die Nettoschuldenquote ging ebenfalls zurück, und zwar auf 16,1 Prozent des BIP. 
+Die Finanzkommission erhielt an ihrer Sitzung vom 26. Februar 2026 erste Informationen zum Ergebnis der Staatsrechnung. Anschliessend tagten die Subkommissionen. An der Sitzung vom 18. Mai 2026 hat die Finanzkommission die Rechnung 2025 und den Nachtrag I zum Voranschlag 2026 beraten. Im Gegensatz zur Einnahmenseite gab es auf der Ausgabenseite keine ausserordentlichen Vorkommnisse. Die Departemente sind daran, die beschlossenen Sparmassnahmen umzusetzen. Die Kommission hat zur Kenntnis genommen, dass die Digitalisierung allgemein vorangeht, aber nicht so schnell wie gewünscht, was auch an den Budgetkürzungen seitens des Parlamentes liegt. Weiter wurde berichtet, dass die erstinstanzlich hängigen Asylgesuche rückläufig sind. Ein Abbau der Gesuche war möglich, die Zahlen beim Bundesverwaltungsgericht sind aber weiter angestiegen. Die Verfahrensdauer ist nach wie vor weit weg von der ursprünglichen Zielsetzung im Rahmen der letzten Asylreform.
+Berichtet wurde über die ersten Gespräche mit dem neuen Leiter des Nachrichtendienstes des Bundes und über die höheren Ausgaben beim NDB.
+Thematisiert wurden ebenfalls die Probleme mit dem neuen Auszahlungssystem der Arbeitslosenkasse, Asalfutur. Die Kommission wurde darüber informiert, dass auf Ende März die Rückstände aufgeholt und alles ausbezahlt worden sei.
+Angesprochen wurde auch die Thematik, dass der Kapitalbezug der zweiten Säule nicht in den nationalen Finanzausgleich integriert ist. Die FK-S wird das Thema weiterverfolgen. 
+Informationen hat die Kommission auch erbeten bezüglich der Verhandlungen über die neue Vereinbarung mit der Schweizerischen Nationalbank. Auslöser waren die Aussagen des SNB-Präsidenten von Ende April in den Medien. Er sagte, dass für die SNB eine Eigenkapitalquote von 15 bis 20 Prozent zu tief sei. Aktuell sind es 19 Prozent. Eine Erhöhung würde bedeuten, dass statt einer Verbesserung sogar eine Verschlechterung gegenüber der heutigen Ausschüttungsvereinbarung drohen könnte, was in der Kommission kritisch gesehen wurde. Die Eidgenössische Finanzverwaltung erläuterte der Kommission die Rückstellungspolitik der SNB und bestätigte, dass sich die SNB eine Eigenkapitalquote zwischen 20 und 30 Prozent vorstelle, während andere Zentralbanken viel tiefere Werte hätten; so hätten beispielsweise die Fed oder die Bank of England eine Eigenkapitalquote von 1 Prozent, in Australien und Schweden sei das Eigenkapital negativ, in Singapur liege die Eigenkapitalquote bei 10 Prozent. Wenn die SNB mit ihrer Rückstellungspolitik tatsächlich dieses Ziel verfolge, müssten sich Bund und Kantone keine Hoffnungen auf höhere Ausschüttungen machen. Die Kommission wird das Thema weiterverfolgen, im Wissen, dass die Entscheide beim Bankrat angesiedelt sind. 
+Die Finanzministerin gab der Kommission auch einen Ausblick auf den Voranschlag 2027 und die kommenden Jahre.
+Nach Verabschiedung des EP 27 in beiden Räten ging der Bundesrat am 15. April noch von einem strukturellen Finanzierungsdefizit von 600 Millionen Franken aus und schlug erste mögliche Massnahmen zu dessen Bereinigung vor. An der Sitzung der FK-S vom 18. Mai konnte Bundesrätin Karin Keller-Sutter Entwarnung geben für den Voranschlag 2027, obwohl das Finanzdepartement für 2027 nochmals mit einer Verschlechterung um voraussichtlich rund 400 Millionen Franken rechnet, insbesondere aufgrund von Schätzkorrekturen bei den Sozialversicherungen und der Migration. Grund dafür sind deutliche Verbesserungen bei der Gewinnsteuer für juristische Personen, auch in anderen Kantonen als Genf. Zwar wies die Finanzministerin darauf hin, dass sich dieses ausserordentliche Wachstum auf einige wenige Unternehmen konzentriere. Sie sagte aber auch, dass die positive Entwicklung der Gewinnsteuern über diese Effekte hinaus breit abgestützt sei. Eine Mehrheit der Kantone habe Anfang Mai gemeldet, dass sie höhere Gewinnsteuereinnahmen hätten.
+Die Mehreinnahmen aus Genf waren hier ja schon mehrfach ein Thema, deshalb lediglich noch ein Wort zu ihrer Verbuchung. Die Eidgenössische Finanzkontrolle (EFK) hat verlangt, dass 1,5 Milliarden Franken schon im Jahr 2025 verbucht werden, ich habe diese eingangs erwähnt. 2026 sind es dann 1,3 Milliarden und 2027 noch 400 Millionen Franken. Es wäre auch denkbar gewesen, die Einnahmen über die Jahre zu glätten und kommende Budgets zu entlasten, doch die EFK bot nicht Hand dazu. So warnte die Finanzministerin auch bereits davor, dass die Lage angesichts der weiterhin bestehenden Herausforderungen, insbesondere bei der Armeefinanzierung und der AHV, ab 2028 wieder schwierig werden dürfte.
+Wenn keine zusätzlichen Einnahmen erschlossen werden könnten, würden ab 2028 beträchtliche strukturelle Defizite drohen. Ein Drittel der vom Bundesrat vorgesehenen Erhöhung der Mehrwertsteuer von 0,8 Prozent soll allein das bereits beschlossene Wachstum der Armee finanzieren, also den Aufwuchs auf 1 Prozent des BIP bis 2032. Der Bundesrat wird die Botschaft zur Armeefinanzierung nach der Sommerpause verabschieden. Neben der federführenden SiK wird sich auch die Finanzkommission in einem Mitbericht mit dem Geschäft befassen.
+Die Kommission tagte stets in Anwesenheit von Bundesrätin Karin Keller-Sutter und der Direktorin der Eidgenössischen Finanzverwaltung Sabine D'Amelio-Favez sowie weiteren Mitarbeiterinnen und Mitarbeitern des EFD, und sie tagte teilweise in Anwesenheit des Leiters der Finanzkontrolle Pascal Stirnimann und der zuständigen Mitarbeiterin. Ich danke den Beteiligten für ihre Begleitung unserer Diskussionen und für die guten Auskünfte.
+Nach Kenntnisnahme der Revisionsberichte der Eidgenössischen Finanzkontrolle sowie der Erwägungen und Schlussfolgerungen der Subkommissionen der FK-S beantragt die Kommission einstimmig, die Staatsrechnung 2025, die Sonderrechnungen für den Bahninfrastrukturfonds sowie den Nationalstrassen- und Agglomerationsverkehrsfonds, die Kreditüberschreitungen von 1,86 Milliarden Franken und die Bildung neuer Reserven in Höhe von 569 Millionen Franken zu genehmigen. Zum Schluss geht mein Dank an das Sekretariat der Finanzkommission für die umsichtige Vorbereitung, Organisation und Begleitung der Sitzungen.
 </t>
   </si>
 </sst>
@@ -396,8 +430,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I10"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -954,6 +988,35 @@
         <v>58</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-16
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -161,12 +161,12 @@
     <t xml:space="preserve">AG</t>
   </si>
   <si>
-    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
-Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass dieser Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
-Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen Halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass der Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Schweiz steht heute vor sicherheitspolitischen Herausforderungen, die sich grundlegend von jenen früherer Jahrzehnte unterscheiden. Mit Verweis auf das von den Grünen genannte Bild des Heuhaufens lässt sich sagen, dass der Heuhaufen tatsächlich sehr, sehr gross geworden ist, sodass wir neue Instrumente brauchen. 
+Cyberangriffe auf kritische Infrastrukturen, internationale Terrornetzwerke, gewalttätiger Extremismus, hybride Bedrohungen, Spionage gegen Forschungseinrichtungen und Unternehmen sowie gezielte Einflussnahmen auf demokratische Prozesse gehören längst zur Realität. Diese Gefahren machen nicht an Landesgrenzen halt. Sie sind digital, international vernetzt und entwickeln sich mit hoher Geschwindigkeit weiter. Wer die Sicherheit in der Schweiz gewährleisten will, muss dieser Realität ins Auge schauen.
 Die GLP steht für Freiheit, Eigenverantwortung, Innovation und einen starken Rechtsstaat ein. Gerade deshalb unterstützen wir die Revision des Nachrichtendienstgesetzes. Freiheit und Sicherheit sind keine Gegensätze. Freiheit kann nur dort bestehen, wo Menschen sicher leben können, wo demokratische Institutionen geschützt werden und wo der Staat seine grundlegenden Funktionen wahrnehmen kann. Der Staat muss in der Lage sein, Bedrohungen frühzeitig zu erkennen und angemessen darauf zu reagieren.
 Die geopolitische Lage hat sich in den vergangenen Jahren deutlich verschärft. Spätestens seit dem russischen Angriffskrieg gegen die Ukraine ist klar geworden, dass Europa wieder verstärkt im Fokus nachrichtendienstlicher und hybrider Operationen steht. Die Schweiz bildet dabei keine Ausnahme, im Gegenteil: Als international vernetzter Wirtschafts-, Forschungs- und Diplomatiestandort ist sie besonders exponiert. Fremde Nachrichtendienste nutzen die Schweiz als Operationsraum, während gleichzeitig unsere Unternehmen, Hochschulen und Forschungsinstitutionen vermehrt Ziel von Spionageversuchen werden. Wer glaubt, die Schweiz könne sich diesen Entwicklungen entziehen, verkennt die Realität.
 Das angepasste Gesetz schafft die Voraussetzungen dafür, dass der Nachrichtendienst seinen Auftrag auch unter den Bedingungen des digitalen Zeitalters erfüllen kann. Kriminelle und feindliche Akteure nutzen verschlüsselte Kommunikationskanäle, globale Datennetze und moderne Technologien. Ein Nachrichtendienst, der auf Instrumenten des letzten Jahrhunderts basiert, kann diesen Herausforderungen nicht wirksam begegnen. Wer von den Sicherheitsbehörden erwartet, dass sie Gefahren erkennen und verhindern, muss ihnen auch die dafür notwendigen Mittel und Tools zur Verfügung stellen.
@@ -174,8 +174,8 @@
 Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
 Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
 Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
-Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu diesem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
-Wichtig sind auch klare Datenschutzgarantien im Gesetz - insbesondere, wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wichtig sind auch klare Datenschutzgarantien im Gesetz, insbesondere wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
 Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
 Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
 Für die GLP ist entscheidend, dass Sicherheit nicht auf Kosten der Freiheit erreicht wird. Die vorliegende Revision ermöglicht eine ausgewogene Balance zwischen wirksamer Gefahrenabwehr und dem Schutz der Grundrechte. Sie stärkt die Handlungsfähigkeit des Staates dort, wo dies notwendig ist, und setzt gleichzeitig klare Grenzen.
@@ -343,12 +343,12 @@
     <t xml:space="preserve">VD</t>
   </si>
   <si>
-    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du Délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
-Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés ; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
-C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter - il n'y en a pas beaucoup, mais de temps en temps, il faut que les choses soient claires.
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que, compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil fédéral reconnaît l'importance d'une évaluation rigoureuse des projets financés dans le cadre du Programme Ukraine 2025-2028, ce programme étant le programme bilatéral le plus grand de la coopération internationale suisse. Il souligne toutefois que, compte tenu du caractère innovant de ce programme, notamment en raison de l'implication accrue du secteur privé suisse, des structures spécifiques de pilotage et de suivi ont déjà été mises en place. Concrètement, un groupe de travail dédié, placé sous la direction du délégué du Conseil fédéral pour l'Ukraine, a été institué afin d'assurer une mise en oeuvre cohérente et coordonnée du programme. Le cadre juridique et les responsabilités sont clairement définis dans une ordonnance.
+Le Conseil fédéral a chargé mon département ainsi que le Département fédéral des affaires étrangères et la Chancellerie fédérale d'évaluer cette organisation au plus tard d'ici octobre 2029. Par ailleurs, les instruments classiques de la coopération internationale sont pleinement mobilisés[NB]; cela inclut un suivi interne régulier et des évaluations externes indépendantes fondées sur des indicateurs précis d'impact et d'efficience. En complément, un audit spécifique du Contrôle fédéral des finances est prévu au premier semestre 2027, en particulier pour les mesures impliquant le secteur privé. Le Conseil fédéral prévoit également de recourir à des expertises externes pour analyser certains projets ciblés, ainsi qu'une évaluation externe globale de l'ensemble du Programme Ukraine. Dans ce contexte, il estime naturellement qu'il sera pertinent, dès que les premiers résultats seront disponibles, d'en proposer une synthèse claire et structurée, qui pourra servir de réponse au postulat.
+C'est dans ce sens que le Conseil fédéral vous prie d'accepter ce postulat. C'est l'un des postulats que nous proposons d'accepter. Il n'y en a pas beaucoup, mais, de temps en temps, il faut que les choses soient claires.
 </t>
   </si>
   <si>
@@ -382,6 +382,70 @@
 Wenn keine zusätzlichen Einnahmen erschlossen werden könnten, würden ab 2028 beträchtliche strukturelle Defizite drohen. Ein Drittel der vom Bundesrat vorgesehenen Erhöhung der Mehrwertsteuer von 0,8 Prozent soll allein das bereits beschlossene Wachstum der Armee finanzieren, also den Aufwuchs auf 1 Prozent des BIP bis 2032. Der Bundesrat wird die Botschaft zur Armeefinanzierung nach der Sommerpause verabschieden. Neben der federführenden SiK wird sich auch die Finanzkommission in einem Mitbericht mit dem Geschäft befassen.
 Die Kommission tagte stets in Anwesenheit von Bundesrätin Karin Keller-Sutter und der Direktorin der Eidgenössischen Finanzverwaltung Sabine D'Amelio-Favez sowie weiteren Mitarbeiterinnen und Mitarbeitern des EFD, und sie tagte teilweise in Anwesenheit des Leiters der Finanzkontrolle Pascal Stirnimann und der zuständigen Mitarbeiterin. Ich danke den Beteiligten für ihre Begleitung unserer Diskussionen und für die guten Auskünfte.
 Nach Kenntnisnahme der Revisionsberichte der Eidgenössischen Finanzkontrolle sowie der Erwägungen und Schlussfolgerungen der Subkommissionen der FK-S beantragt die Kommission einstimmig, die Staatsrechnung 2025, die Sonderrechnungen für den Bahninfrastrukturfonds sowie den Nationalstrassen- und Agglomerationsverkehrsfonds, die Kreditüberschreitungen von 1,86 Milliarden Franken und die Bildung neuer Reserven in Höhe von 569 Millionen Franken zu genehmigen. Zum Schluss geht mein Dank an das Sekretariat der Finanzkommission für die umsichtige Vorbereitung, Organisation und Begleitung der Sitzungen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377091</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260616</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weichelt Manuela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das vergangene Geschäftsjahr stand im Zeichen eines wichtigen rechtsstaatlichen Jubiläums: 150 Jahre Bundesgericht. Tragen wir Sorge zu unseren Errungenschaften. Respektieren wir die Gewaltenteilung und achten wir unsere Bundesverfassung sowie die Gesetze.
+Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden GPK haben ihre Aufsichtssitzung im April zum Geschäftsbericht traditionsgemäss in Lausanne am Bundesgericht durchgeführt. An der Mai-Sitzung des Plenums der GPK-N haben zudem sowohl de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das vergangene Geschäftsjahr stand im Zeichen eines wichtigen rechtsstaatlichen Jubiläums: 150 Jahre Bundesgericht. Tragen wir Sorge zu unseren Errungenschaften. Respektieren wir die Gewaltenteilung und achten wir unsere Bundesverfassung sowie die Gesetze.
+Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden GPK haben ihre Aufsichtssitzung im April zum Geschäftsbericht traditionsgemäss in Lausanne am Bundesgericht durchgeführt. An der Mai-Sitzung des Plenums der GPK-N haben zudem sowohl der Gerichtspräsident als auch die Subkommission entsprechend informiert.
+Bis auf das Patentgericht haben alle Gerichte einen Geschäftsanstieg zu verzeichnen. Das Bundesgericht hat einen Anstieg von rund 7 Prozent gegenüber dem Vorjahr zu verzeichnen. Dieser im Vergleich zu früheren Jahren geringere Anstieg zeigt, dass die Neuorganisation vor einigen Jahren allmählich Früchte trägt. Die durchschnittliche Verfahrensdauer verkürzte sich um einige Tage. Leicht weniger Beschwerden wurden gutgeheissen. Das Bundesgericht veröffentlichte 213 Urteile, auch, um die Transparenz der Rechtsprechung zu gewährleisten.
+Im Vergleich zum Bundesgericht verfügt das Bundesstrafgericht über eine kurze institutionelle Geschichte. Die Strafkammer konnte die Zahl der hängigen Verfahren reduzieren, hatte aber gleichzeitig mehrere grosse bedeutende Verfahren zu bearbeiten, beispielsweise bezüglich Bestechung fremder Amtsträger im internationalen Handel mit Erdölprodukten.
+Die Beschwerdekammer hatte Ende des Jahres mehr hängige Verfahren. Dies unter anderem aufgrund der Zunahme der Verfahren im Verwaltungsstrafrecht und im Bereich der internationalen Rechtshilfe.
+Die Berufungskammer hatte eine weitere Zunahme der Verfahren zu verzeichnen; diese betrafen das Unternehmensstrafrecht, Geldwäscherei, Insider Tradings, Terrorismus sowie die Bankomatensprengungen.
+Es wurde auch darauf hingewiesen, dass die nebenamtlichen Richterpersonen aufgrund ihrer hauptberuflichen Auslastung zeitlich nicht so flexibel sind, wie es ursprünglich angedacht war.
+Interessant für das Parlament sind auch immer die Hinweise an den Gesetzgeber. So hat das Bundesstrafgericht beispielsweise den EFK-Bericht bezüglich den Einziehungen und Ersatzforderungen nach Artikel 70 ff. StGB ernst genommen. Damit sich der Grundsatz "Strafbares Handeln soll sich nicht lohnen" auch richtig umsetzen lässt, wird angeregt, ein vereinfachtes Vollstreckungsverfahren zu schaffen, damit die Ersatzforderungen schnell eingetrieben werden können. Das ist ein wichtiger Punkt bei der Bekämpfung der Wirtschaftskriminalität.
+Das Bundesverwaltungsgericht verzeichnet erneut einen markanten Anstieg der Geschäftslast. Eine bessere Koordination zwischen dem SEM und dem Bundesverwaltungsgericht wäre mehr als wünschenswert. Es gab 70 neue Stellen beim SEM, aber nur eine Mikroerhöhung des Stellenetats beim Bundesverwaltungsgericht in St. Gallen. Eine bessere Koordination hätte da zu einer besseren Lösung führen können.
+Die durchschnittliche Verfahrensdauer konnte man jedoch reduzieren. Gleichzeitig hat man in St. Gallen aber auch viel in die Digitalisierung investiert. Das Ziel, Papier definitiv beiseite zu lassen, rückt immer näher. Die Spruchkörperbildung soll ab 2027 mit dem System "Diva" durchgeführt werden und den Abteilungspräsidien eine grosse Entlastung bringen.
+Das Bundespatentgericht verzeichnete einen Rückgang an Eingängen. Kein Fall ist länger als zwei Jahre hängig. Der Grund liegt vermutlich in der Bildung des Einheitlichen Patentgerichts (EPG). Dieses erlässt Verbote, die für bis zu 18 Länder gelten, und kann Patente für alle angeschlossenen Länder für ungültig erklären. Die Teilnahme am System steht nur für EU-Staaten offen, hat aber auch Auswirkungen auf die Schweiz.
+Das Bundespatentgericht in der Schweiz hat sich das Ziel gesetzt, das schnellste Gericht in Europa zu werden. Hierfür hat es unter anderem ein beschleunigtes Nichtigkeitsverfahren eingeführt.
+Ich sage noch einige wenige Worte zum Militärkassationsgericht. Dieses gehört nicht zum Bundesgericht, wie Sie wissen, aber auch hier hat die Bundesversammlung die Oberaufsicht. Deshalb erlaube ich mir dazu noch zwei, drei Sätze.
+Die zuständigen Subkommissionen des Ständerates und Nationalrates konnten vom Geschäftsbericht des Militärkassationsgerichtes keine Kenntnis nehmen. Grund: Wir haben keinen erhalten. Das ist unbefriedigend und nicht tolerierbar.
+Einige Worte zur Arbeit in der GPK im Zusammenhang mit den Gerichten: Wir haben einige Motionen und Berichte gemacht. Ich möchte Ihnen ganz kurz den Stand mitteilen:
+1. Die parlamentarische Initiative der GPK, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", ist zurzeit in der RK-S.
+2. Die Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes und der anderen erstinstanzlichen Gerichte wurde von der RK-N im Rahmen einer grösseren Revision behandelt.
+3. Die Motion zur Reorganisation des Bundesstrafgerichtes wurde in der RK-N einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die RK auf den Bericht der GPK von 2022.
+4. Den Bericht zum System der nebenamtlichen Richterinnen und Richter konnte die Subkommission Gerichte in der RK-N vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv werden.
+Ich möchte nicht schliessen, ohne dem Präsidenten des Bundesgerichtes und allen, die zum reibungslosen Funktionieren der Bundesjustiz beitragen, sowie dem Sekretariat der Geschäftsprüfungskommission für ihre Arbeit ganz herzlich zu danken. Es versteht sich von selbst, dass beaufsichtigte Stellen nicht alle Fragen der Aufsicht lieben. Das müssen sie auch nicht. Wir haben alle das gleiche Ziel: eine gut funktionierende und von der Politik unabhängige Justiz. Eine solche ist unabdingbar für eine Demokratie, in der heutigen Zeit mehr denn je.
+Ich bitte Sie, den Geschäftsbericht 2025 des Bundesgerichtes zu genehmigen. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salzmann Werner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
+Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
+Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.
+Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
+Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
+Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
 </t>
   </si>
 </sst>
@@ -430,8 +494,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I12"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1017,6 +1081,64 @@
         <v>64</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-17
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -127,24 +127,24 @@
     <t xml:space="preserve">IT</t>
   </si>
   <si>
-    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del Consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Commissione delle finanze aveva già preso atto del risultato del consuntivo 2025 della Confederazion nel mese di febbraio. Per la prima volta dopo la crisi di Covid-19, il consuntivo chiude con un risultato positivo, registrando un'eccedenza di finanziamento di 259 milioni di franchi. Questo risultato, che rappresenta un chiaro miglioramento rispetto al deficit preventivato di 815 milioni di franchi, risulta da un'eccedenza di 1,185 miliardi nel bilancio ordinario a fronte di un deficit di 925 milioni iscritto nel bilancio straordinario. Il risultato favorevole è riconducibile principalmente alle entrate fiscali supplementari provenienti da alcune imprese nel Cantone di Ginevra.
 Il disavanzo del bilancio straordinario è dovuto soprattutto ai contributi versati ai Cantoni per le persone con statuto di protezione S provenienti dall'Ucraina, 700 milioni, e al contributo unico alle FFS, 850 milioni, compensati in parte da entrate straordinarie della Banca nazionale svizzera.
 L'avanzo dell'amministrazione ordinaria raggiunge 1,2 miliardi di franchi, mentre la regola del freno all'indebitamento avrebbe consentito un deficit di 262 milioni di franchi. Ne risulta quindi un saldo strutturale positivo di 1,4 miliardi, nettamente superiore al valore previsto nel preventivo.
 Le entrate ordinarie superano il budget di 1,9 miliardi e il risultato dell'anno precedente di ben 3,3 miliardi. La crescita è dovuta soprattutto all'imposta federale diretta sulle imprese, che beneficia delle entrate temporanee dal Cantone di Ginevra per circa 1,5 miliardi di franchi.
 Anche l'imposta federale diretta sui redditi aumenta di 0,5 miliardi, mentre l'IVA aumenta di 700 milioni, grazie alla crescita dell'economia nominale e all'effetto ritardato dell'aumento dell'aliquota dal 2024. Le entrate dell'imposta preventiva, invece, risultano inferiori alle attese.
-Le spese totali sono aumentate del 4 percento e ammontano a 87,6 miliardi di franchi. 
+Le spese totali sono aumentate del 4 per cento e ammontano a 87,6 miliardi di franchi. 
 I principali aumenti riguardano la previdenza sociale, le finanze e imposte, i trasporti, l'istruzione e la ricerca e l'esercito.
 Nel 2025 il numero di posti nella Confederazione è cresciuto di 240 unità, più 0,6 per cento, mentre le spese per il personale sono aumentate di 79 milioni di franchi, soprattutto per il rincaro dell'1 per cento.
 Il debito netto scende leggermente a 140 miliardi di franchi. Il conto di ammortamento del debito Covid si riduce per la prima volta di circa 500 milioni, grazie al saldo strutturale positivo e alle entrate straordinarie, e ammonta a 26,3 miliardi di franchi. Il conto di compensazione rimane stabile a circa 20 miliardi di franchi.
 Nella seduta dell'11 e 12 maggio 2026, la commissione ha proceduto all'esame di dettaglio del consuntivo. Le sue quattro sottocommissioni hanno presentato le conclusioni delle rispettive analisi approfondite dei consuntivi dei singoli servizi federali realizzate nel corso del mese di aprile.
-Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla sua commissione i risultati delle tre verifiche relative al Consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del Fondo per l'infrastruttura ferroviaria e quella del Fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
-Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del Fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma ancora irrisolte. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
+Il Controllo federale delle finanze, quale organo di revisione, ha presentato alla vostra commissione i risultati delle tre verifiche relative al consuntivo 2025 della Confederazione: la revisione del conto annuale, la verifica del fondo per l'infrastruttura ferroviaria e quella del fondo per le strade nazionali e il traffico d'agglomerato. Ogni revisione è stata condotta separatamente e richiede un'approvazione da parte del Parlamento.
+Le verifiche mostrano che i conti rispettano gli standard contabili e che non vi sono carenze significative nei controlli interni. Tuttavia, la situazione finanziaria dei fondi presenta rischi. Le riserve del fondo per l'infrastruttura ferroviaria saranno esaurite entro il 2028, violando la riserva minima legale di 300 milioni di franchi. Le cause principali sono l'aumento dei costi di esercizio e di manutenzione, la riduzione delle entrate e la restituzione di anticipi. Le sfide finanziarie del fondo sono note, ma i problemi ancora irrisolti. Anche il fondo per le strade nazionali e il traffico d'agglomerato rischia, senza misure correttive, di scendere sotto le riserve minime previste dalla legge.
 Il Controllo federale delle finanze conferma che il consuntivo rispetta le prescrizioni legali e le regole del freno all'indebitamento previste dall'articolo 126 della Costituzione federale. Per questo motivo raccomanda all'Assemblea federale di approvare il conto annuale.
 Nel rapporto vengono richiamati due aspetti già evidenziati negli anni precedenti. Il primo riguarda il fatto che la contabilità non permette una valutazione completa della situazione patrimoniale, poiché non considera il capitale proprio del fondo dell'infrastruttura ferroviaria, che è negativo. Se fosse incluso, il capitale proprio della Confederazione risulterebbe inferiore di 1,9 milioni di franchi, ma il metodo attuale è conforme alla legge. Il secondo punto concerne la riscossione dell'imposta federale diretta, che è effettuata dai Cantoni. Il Controllo federale delle finanze sottolinea che le competenze di revisione in questo ambito spettano alle autorità cantonali e non a quelle federali.
-La vostra commissione vi propone all'unanimità di approvare il Consuntivo 2025 della Confederazione come pure i conti speciali concernenti il Fondo per le strade nazionali e il traffico d'agglomerato e il Fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
+La vostra commissione vi propone all'unanimità di approvare il consuntivo 2025 della Confederazione come pure i conti speciali concernenti il fondo per le strade nazionali e il traffico d'agglomerato e il fondo per l'infrastruttura ferroviaria. La commissione si allinea così alla posizione del Controllo federale delle finanze, che in qualità di organo di revisione ha raccomandato l'approvazione del consuntivo, del sorpasso di credito di 1,86 miliardi di franchi e della costituzione di nuove riserve pari a 569 milioni di franchi.
 Concludo ringraziando il Consiglio federale, in particolare la consigliera federale Karin Keller-Sutter, l'Amministrazione federale delle finanze, il Segretariato commissionale e il Controllo federale delle finanze.
 </t>
   </si>
@@ -306,6 +306,32 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">375543</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Lieber ein Ende mit Schrecken als ein Schrecken ohne Ende" - ich habe noch eine Motion, die ich von Kollege Glättli geerbt habe und hier kurz vorstelle. Es geht um die Beschaffung des F-35. Sie erinnern sich: Im Februar 2025 informierten die USA die Schweiz schriftlich, dass der vertraglich vereinbarte Festpreis aus ihrer Sicht ein Missverständnis sei. Es zeigte sich: Der Festpreis, der uns ziemlich vehement und über Jahre als solcher verkauft wurde, war keiner und ist den USA gegenüber auch ni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Lieber ein Ende mit Schrecken als ein Schrecken ohne Ende" - ich habe noch eine Motion, die ich von Kollege Glättli geerbt habe und hier kurz vorstelle. Es geht um die Beschaffung des F-35. Sie erinnern sich: Im Februar 2025 informierten die USA die Schweiz schriftlich, dass der vertraglich vereinbarte Festpreis aus ihrer Sicht ein Missverständnis sei. Es zeigte sich: Der Festpreis, der uns ziemlich vehement und über Jahre als solcher verkauft wurde, war keiner und ist den USA gegenüber auch nicht durchsetzbar. Je nach Berechnung können mit dem vom Volk bewilligten Budget nur noch zwischen 24 und 30 Maschinen beschafft werden statt der geplanten und versprochenen 36.
+Zusätzlich steigen die Infrastrukturkosten substanziell. Statt 120 Millionen sollen die Anpassungen der Militärflugplätze mindestens 200 Millionen Franken kosten. Die Eidgenössische Finanzkontrolle hat weitere Projekte von über 50 Millionen Franken identifiziert, die da obendrauf kommen. Das ist nicht ganz die Beschaffung, die uns 2021 verkauft wurde.
+Nun aber zu einer Frage, die zu wenig oft gestellt wird: Wofür braucht die Schweiz ein Kampfflugzeug? Die Hauptaufgabe ist die Luftpolizei, also das Identifizieren, Begleiten und nötigenfalls Abfangen von Flugzeugen im Schweizer Luftraum. Dafür braucht es Verfügbarkeit, Reaktionsgeschwindigkeit und Interoperabilität mit europäischen Partnern. Der F-35 ist als erstes Tarnkappenflugzeug der Geschichte zertifiziert, um Atomwaffen zu tragen. Im Juni 2025 drangen F-35A als erste Flugzeuge in den iranischen Luftraum ein, um Luftabwehrsysteme zu unterdrücken und B2-Bomber beim Angriff auf unterirdische Atomanlagen zu eskortieren. Das ist das Profil des F-35: Erstschlag tief im feindlichen Territorium, sogar mit nuklearer Bestückung und Tarnkappe.
+Die Schweiz ihrerseits eskortiert Privatjets über den Alpen und schützt vor allem Konferenzen in Genf und Davos. Die Stealth-Fähigkeit ist für diese Aufgaben schlicht irrelevant. Europäische Alternativen wie der Eurofighter oder die Rafale beherrschen den Luftpolizeidienst vollständig. Das hat auch ein ehemaliger Bundesrat ganz beeindruckend erlebt, als er von zwei Rafales eskortiert wurde. Offenbar kann dieses Flugzeug Luftpolizei.
+Auch sonst würden beispielsweise Eurofighter, Rafale oder Gripen das, was man sich vom F-35 erhofft, auch können, aber mit mehr operativer Unabhängigkeit. Sie würden auch zur Strategie des Bundesrates passen, künftig 60 Prozent aller Rüstungsbeschaffungen in der Schweiz und 30 Prozent in Europa zu tätigen und eben nur den Rest, 10 Prozent, ausserhalb Europas, sprich: mehr oder weniger in den USA. Eine Grossbeschaffung, die das gesamte Kampfflugzeugbudget exklusiv in die USA leitet, widerspricht diesem Ziel fundamental.
+Der Bundesrat hat die richtige Strategie formuliert und zieht die falschen Konsequenzen. Dazu kommt die operative Abhängigkeit. Die wichtigsten Stärken des F-35, seine Sensorfähigkeiten und seine Vernetzung, hängen direkt von US-amerikanischen Software-Updates und Aktivierungscodes ab. Bei politischer Instabilität in Washington, und von dieser gibt es zur Genüge, könnte der Jet innerhalb weniger Tage unbrauchbar gemacht werden. Das Herz des Jets liegt nicht in Emmen, sondern in Fort Worth.
+Der Bundesrat warnt vor einer Fähigkeitslücke, und auch das nehmen wir ernst. Deshalb fordert die Motion nicht einfach ein Abbrechen ohne Konzept, sondern gleichzeitig die Prüfung europäischer Alternativen und den Aufbau von Kapazitäten zur Drohnenabwehr und bodengestützten Luftverteidigung. Das ist die Richtung, in die Europa ohnehin zieht. Ein Jet, dessen Operabilität von einem unzuverlässigen Partner in Washington abhängt, schützt uns nicht. Er macht uns erpressbar. Die Motion ist aktueller denn je.
+Ich bitte um Zustimmung.
+</t>
+  </si>
+  <si>
     <t xml:space="preserve">375897</t>
   </si>
   <si>
@@ -318,14 +344,14 @@
     <t xml:space="preserve">Moser Tiana Angelina</t>
   </si>
   <si>
-    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband; der Fachverband für Wasser, Gas und Wärme; der Schweizerische Berufsfischerverband; der Schweizerische Brunnenmeister-Verband; und der Verband der Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband, der Fachverband für Wasser, Gas und Wärme, der Schweizerische Berufsfischerverband, der Schweizerische Brunnenmeister-Verband, und der Verband Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letzten Donnerstag, den 4. Juni, haben die wichtigsten Verbände aus den Bereichen Fischerei, Trinkwasserversorgung und Gewässerschutz eine gemeinsame Resolution zum Umgang mit PFAS verabschiedet. Es sind dies der Schweizerische Fischerei-Verband, der Fachverband für Wasser, Gas und Wärme, der Schweizerische Berufsfischerverband, der Schweizerische Brunnenmeister-Verband, und der Verband Schweizer Abwasser- und Gewässerschutzfachleute. Die Botschaft dieser Resolution, die sie letzten Donnerstag verabschiedet haben, ist unmissverständlich. Es braucht ein rasches und auch ein konsequenteres Vorgehen des Bundesrates. Die Schweiz müsse jetzt handeln, um eine weitere Anreicherung von PFAS in Gewässern, Böden, Trinkwasser und Lebensmitteln zu verhindern und somit auch langfristige Schäden abzuwenden.
 Die Resolution verdient eine besondere Aufmerksamkeit. Sie stammt nicht nur von einzelnen Organisationen, sondern von denjenigen, die die Folgen der PFAS-Belastung im Interesse und zum Schutz der Bevölkerung bewältigen müssen. Die Brunnenmeister beispielsweise sind zuständig für die Sicherung der Wasserqualität und die Versorgung der Bevölkerung. 
-PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
+PFAS sind nicht einfach ein Umweltproblem. Es erwarten uns mittlerweile auch enorme volkswirtschaftliche Kosten. Eine SRF-Recherche schätzt die Kosten für die Sanierung PFAS-belasteter Böden, Gewässer und Trinkwasservorkommen in der Schweiz je nach Szenario auf bis zu 26 Milliarden Franken. Damit bewegen wir uns in einer Grössenordnung, die die Kosten vieler bisheriger Altlastensanierungen deutlich übersteigt. PFAS sind zunehmend auch ein Gesundheitsproblem. Diese sogenannten Ewigkeitschemikalien reichern sich selbstverständlich in der Umwelt an, aber eben auch im menschlichen Körper. Sie schwächen das Immunsystem, mindern die Wirkung von Impfungen, können Organe schädigen. Besonders beunruhigend ist, dass wir den Stoffen über Trinkwasser, Lebensmittel und die Umwelt täglich ausgesetzt sind. Deshalb wäre es auch wichtig, zu wissen, wie stark die Bevölkerung tatsächlich belastet ist. Dieses Wissen wäre gerade auch vertrauensfördernd. 
 Vor diesem Hintergrund ist die Stellungnahme des Bundesrates zu Frage 2 meiner Interpellation besonders bemerkenswert. Der Bundesrat anerkennt ausdrücklich den Nutzen des Human Biomonitoring für die Erfassung der Belastung der Bevölkerung. Genau solche Daten bräuchten wir, um Risiken frühzeitig zu erkennen und entsprechende Entwicklungen zu verfolgen. Umso weniger verständlich ist es, dass ausgerechnet dieses Instrument aus Spargründen eingestellt worden ist. Die Kosten des Human Biomonitoring stehen in keinem Verhältnis zu den Folgekosten der PFAS-Belastung, die sich, Sie haben es gehört, im Milliardenbereich bewegen. Auf das Monitoring zu verzichten, heisst, auf Wissen zu verzichten, das helfen könnte, gesundheitliche Risiken frühzeitig zu erkennen und Schäden zu begrenzen. 
-Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind wie gesagt nur die Beispiele zum Gewässer. 
+Die Resolution der Wasserfachleute fordert entsprechend eine Überwachung von Gewässern, Sedimenten, Böden, Lebensmitteln und des Trinkwassers, um Belastungen frühzeitig zu erkennen. Die Schweiz befindet sich beim Thema PFAS noch weitgehend im Ungewissen. Verschiedene Fälle beunruhigen die Bevölkerung, nur schon diejenigen, welche die Gewässer betreffen: Der Verkauf von Hecht und Egli aus dem Zugersee beispielsweise wurde wegen der PFAS-Belastung verboten. In Basel wurde der Bevölkerung empfohlen, den Verzehr von selbstgefangenem Fisch auf maximal einmal pro Monat zu reduzieren. Und in der Interpellation habe ich das Beispiel eines Fischers erwähnt, dessen Blutwert den Wert, der als unbedenklich gilt, um das 77-Fache überstieg. Das sind, wie gesagt, nur die Beispiele zum Gewässer. 
 Es ist offensichtlich, dass es sich hier um eine schweizweite Herausforderung handelt. Wir stehen bei der PFAS-Thematik erst am Anfang, und gerade deshalb können wir es uns nicht leisten, auf Wissen zu verzichten. Entsprechend wichtig wäre eine Wiederaufnahme des Human Biomonitoring im Rahmen des Aktionsplans zur Reduktion der Ewigkeitschemikalien. Diese Einschätzung wurde im Übrigen auch von der Eidgenössischen Finanzkontrolle 2024 geteilt. Gerade angesichts der gesundheitlichen Risiken und der möglichen Folgekosten sowie der grossen Wissenslücken wäre das eine sehr wichtige Aussage, um auch das Vertrauen der Bevölkerung zu steigern. 
 In diesem Sinne danke ich Ihnen herzlich für die Antworten und bin gespannt auf die weiteren Schritte.
 </t>
@@ -392,9 +418,6 @@
   </si>
   <si>
     <t xml:space="preserve">Weichelt Manuela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
   </si>
   <si>
     <t xml:space="preserve">ZG</t>
@@ -446,6 +469,37 @@
 Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
 Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
 Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377387</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binder-Keller Marianne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden Geschäftsprüfungskommissionen, also des Nationalrates und des Ständerates, tagen in der Regel gemeinsam. Traditionellerweise findet die Sitzung, in welcher sie den Geschäftsbericht des Bundesgerichtes diskutieren und zur Kenntnis nehmen, am Bundesgericht in Lausanne statt; dies - nebenbei bemerkt - in einem Raum mit ikonischen Bildern. Eines zeigt die archaische Szene des salomonischen Urteils und bringt mich jedes Mal ins Grübeln, wenn </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Subkommissionen Gerichte/Bundesanwaltschaft der beiden Geschäftsprüfungskommissionen, also des Nationalrates und des Ständerates, tagen in der Regel gemeinsam. Traditionellerweise findet die Sitzung, in welcher sie den Geschäftsbericht des Bundesgerichtes diskutieren und zur Kenntnis nehmen, am Bundesgericht in Lausanne statt; dies - nebenbei bemerkt - in einem Raum mit ikonischen Bildern. Eines zeigt die archaische Szene des salomonischen Urteils und bringt mich jedes Mal ins Grübeln, wenn ich ein Urteil wieder einmal als salomonisch loben will. Da kommen zwei Frauen zu Salomon mit einem Kind, beide behaupten, es sei ihres. König Salomon befiehlt, das Kind mit einem Schwert auseinanderzuhauen, damit jede Frau ihre Hälfte bekäme. Die eine Frau sagte dann, man solle es der anderen geben, damit das Kind überlebe. Voilà, da hat Salomon gemerkt, dass das die richtige Mutter ist. Wenn Sie also das Wort "salomonisch" bei einem Urteil verwenden, geht das auf diese Geschichte zurück. 
+Anwesend am 22. April 2026 in Lausanne war der Bundesgerichtspräsident, verschiedene weitere Mitglieder des Bundesgerichtes, die Präsidentinnen und Präsidenten der erstinstanzlichen Gerichte und weitere Mitglieder. In ihrer Plenarsitzung im Mai 2026 hat auch die Geschäftsprüfungskommission den Bericht zur Kenntnis genommen, der ihr dann auch vom Bundesgericht vorgestellt wurde.
+Zur Einordnung der Aufgaben der Geschäftsprüfungskommissionen gegenüber dem Bundesgericht: Die Bundesversammlung übt die Oberaufsicht über das Bundesgericht, die oberste gerichtliche Instanz der Eidgenossenschaft, aus. Das heisst, sie übt die Oberaufsicht über die Geschäftsführung des Bundesgerichtes aus, selbstverständlich geht es nicht um die Wertung von Urteilen. Das Bundesgericht übt seinerseits die Aufsicht über das Bundesstrafgericht, das Bundesverwaltungsgericht und das Bundespatentgericht aus, wobei das Bundesgericht nach wie vor nicht über die Befugnisse und Mittel verfügt, um in persönlichen Angelegenheiten umfassend einzugreifen. Wie die jüngsten Ereignisse jedoch zeigen, bereiten bestimmte Fälle nach wie vor Probleme. Wir werden bei der Prüfung des Geschäftsberichtes des Jahres 2026 darauf zurückkommen müssen.
+Im Jahr 2025 haben die verschiedenen Kammern des Bundesgerichtes über 7883 Fälle entschieden, was rund 7 Prozent mehr als dem Wert des Vorjahres entspricht; im Jahr 2024 wurden 7351 Fälle entschieden. Dieser geringere Anstieg als zuvor zeigt, dass die 2020 eingeleitete Reorganisation der Kammern allmählich Früchte trägt. Die durchschnittliche Verfahrensdauer verkürzte sich um einige Tage. Leicht weniger Beschwerden wurden gutgeheissen. Das Bundesgericht veröffentlichte 213 Urteile, auch um die Transparenz der Rechtsprechung zu gewährleisten. All dies ersehen Sie im Detail im Bericht des Bundesgerichtes. 
+Zu den erstinstanzlichen Gerichten: Das Bundesstrafgericht verzeichnete im Jahr 2025 insgesamt einen Anstieg der Eingänge auf 686 neue Fälle gegenüber 619 im Jahr 2024. Die Erledigungsquote blieb stabil bei 93 Prozent statt 94 Prozent im Jahr 2024. Die Strafkammer hatte mehrere bedeutende Verfahren zu bearbeiten, beispielsweise bezüglich Bestechung fremder Amtsträger im internationalen Handel mit Erdölprodukten. Die Beschwerdekammer hatte Ende des Jahres mehr hängige Verfahren, dies unter anderem aufgrund der Zunahme der Verfahren im Verwaltungsstrafrecht und im Bereich der internationalen Rechtshilfe. Die Berufungskammer hatte eine weitere Zunahme der Verfahren zu verzeichnen. Diese betrafen das Unternehmensstrafrecht, Geldwäscherei, Insiderhandel, Terrorismus sowie die Bankomatsprengungen. 
+Es wurde auch darauf hingewiesen, dass die nebenamtlichen Richterpersonen aufgrund ihrer hauptberuflichen Auslastung zeitlich nicht so flexibel sind, wie es ursprünglich angedacht war. 
+Interessant für das Parlament sind auch immer die Hinweise an den Gesetzgeber, die wir unterdessen auch noch direkt den Sachbereichskommissionen mitteilen. So hat das Bundesstrafgericht beispielsweise den EFK-Bericht bezüglich der Einziehungen und Ersatzforderungen nach Artikel 70 StGB ernst genommen. Damit sich der Grundsatz "Strafbares Handeln soll sich nicht lohnen" auch richtig umsetzen lässt, wird angeregt, ein vereinfachtes Vollstreckungsverfahren zu schaffen, damit die Ersatzforderungen schnell eingetrieben werden können. Das ist ein wichtiger Punkt bei der Bekämpfung der Wirtschaftskriminalität.
+Das Bundesverwaltungsgericht verzeichnet erneut einen markanten Anstieg der Geschäftslast. Eine bessere Koordination zwischen dem SEM und dem Bundesverwaltungsgericht wäre wünschenswert. Es gab 70 neue Stellen beim SEM, aber nur eine Mikroerhöhung des Stellenetats beim Bundesverwaltungsgericht in St. Gallen. Eine bessere Koordination hätte da, wie betont, zu einer besseren Lösung führen können. Die durchschnittliche Verfahrensdauer konnte man jedoch reduzieren. Gleichzeitig hat man in St. Gallen auch viel in die Digitalisierung investiert. Das Ziel, Papier definitiv beiseitezulassen, rückt näher.
+Das Bundespatentgericht verzeichnete einen Rückgang an Eingängen. Kein Fall ist länger als zwei Jahre hängig. Der Grund liegt vermutlich in der Bildung des Einheitlichen Patentgerichtes. Dieses erlässt Verbote, die für bis zu 18 Länder gelten, und kann Patente für alle angeschlossenen Länder für ungültig erklären. Die Teilnahme am System steht nur EU-Staaten offen, das System hat aber auch Auswirkungen auf die Schweiz. Das Bundespatentgericht hat sich zum Ziel gesetzt, das schnellste Gericht in Europa zu werden. Hierfür hat es unter anderem ein beschleunigtes Nichtigkeitsverfahren eingeführt.
+Einige Worte noch zur Arbeit in der Geschäftsprüfungskommission im Zusammenhang mit den Gerichten: Wir haben einige Vorstösse und Berichte ausgearbeitet. Ganz kurz zum Stand: 
+Erstens hat die GPK-S die parlamentarische Initiative 25.401, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", eingereicht. Dieser Vorstoss, dieses Anliegen liegt zurzeit in der Kommission für Rechtsfragen des Ständerates. Die Motion 22.4250, "Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes, des Bundesverwaltungsgerichtes und des Bundesstrafgerichtes", wurde von der Kommission für Rechtsfragen des Nationalrates im Rahmen einer grösseren Revision behandelt. Die Motion 25.4395 der RK-S, "Reorganisation des Bundesstrafgerichtes", wurde ebenfalls in der Kommission für Rechtsfragen des Nationalrates einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die Kommission für Rechtsfragen auf den Bericht der GPK aus dem Jahre 2022. Weiter konnte die GPK-Subkommission Gerichte/BA den Bericht zum System der nebenamtlichen Richterinnen und Richter in der Kommission für Rechtsfragen des Nationalrates vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv wird.
+Letztlich sei daran erinnert, dass das Bundesgericht im Jahr 2025 sein 150-jähriges Bestehen feierte. Zu diesem Anlass wurden unter anderem ein wissenschaftliches Kolloquium, eine Festschrift, eine offizielle Feier sowie Tage der offenen Tür mit etwa zweitausend Besuchern organisiert. 
+Ich möchte, Herr Bundesgerichtspräsident, diesen Bericht nicht abschliessen, ohne Ihre Arbeit zu verdanken, die gute Zusammenarbeit mit den Bundesbehörden und auch die Arbeit Ihres Sekretariats, unter anderem im Zusammenhang mit der Tätigkeit unserer Kommission.
 </t>
   </si>
 </sst>
@@ -494,8 +548,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I14"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1004,16 +1058,16 @@
         <v>48</v>
       </c>
       <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
@@ -1033,17 +1087,19 @@
         <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9"/>
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="G9" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="H9" t="s">
         <v>57</v>
@@ -1060,19 +1116,17 @@
         <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
-        <v>49</v>
-      </c>
+      <c r="E10"/>
       <c r="F10" t="s">
         <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
         <v>63</v>
@@ -1089,42 +1143,42 @@
         <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
         <v>67</v>
       </c>
       <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
         <v>68</v>
-      </c>
-      <c r="F11" t="s">
-        <v>69</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
       </c>
       <c r="H11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" t="s">
         <v>70</v>
-      </c>
-      <c r="I11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
         <v>72</v>
       </c>
-      <c r="B12" t="s">
-        <v>66</v>
-      </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
         <v>74</v>
@@ -1137,6 +1191,64 @@
       </c>
       <c r="I12" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-06-18
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -460,16 +460,10 @@
     <t xml:space="preserve">BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
-Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.
-Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.
-Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir schaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.
-Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.
-Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.
-</t>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evalua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich bitte Sie, auf alle drei Bundesbeschlüsse einzutreten, weil sie eben genau der wahrscheinlichsten Bedrohung entsprechen.Zum Bundesbeschluss über die Beschaffung der Kampfflugzeuge F-35A: Ich halte das gut aus, Frau Roth, was Sie sagen. Ich kann aber nicht stehen lassen, wenn Sie von irgendwelchen Lobbyisten Texte bekommen, die wir in der Sicherheitspolitischen Kommission gar nicht besprochen haben, und diese hier verbreiten. Wir haben den F-35A einer Evaluation unterziehen lassen. Die Evaluationsmethode wurde durch die Eidgenössische Finanzkontrolle geprüft und gutgeheissen. Der F-35A hat mit Abstand am besten abgeschnitten. Er ist preislich konkurrenzfähig und dient nicht nur der Sache des zivilen Luftpolizeidiensts, sondern auch der militärischen Sache. Er muss auch konkurrenzfähig sein, um jedes Kampfflugzeug aus dem Luftraum zu verdrängen oder zur Landung zu zwingen.Der F-35A ist, wie Frau Kollegin Gmür gesagt hat, eben auch ein Beispiel einer Kooperation in Europa, damit man Daten austauschen kann, 400 Kilometer weit über die Landesgrenze hinaussehen und gegnerische Flugzeuge erkennen kann, in Kombination mit unserem Bodluv-System und den Bodentruppen, was dann über die NDP läuft. Das ist das System, das wir beschaffen müssen. Alle anderen Flugzeuge auf dem Markt sind nicht Flugzeuge der fünften Generation und entsprechen nicht dem Level, das der F-35A hat.Wenn man natürlich immer und immer wieder über den F-35A herzieht und ihn kritisiert, dann kann man sich schon vorstellen, dass es Leute gibt, die glauben, dass es nicht das richtige Flugzeug sei. Aber das ist nicht so; es ist das richtige Flugzeug, und es ist auch kein Projekt, das kaputt gegangen ist. Einzig der Fixpreis, den man erwähnt hat, kann nicht eingehalten werden. Das ist die einzige Kritik, und das führt jetzt dazu, dass wir einen höheren Preis haben. Das ist aber nicht nur aufgrund des fehlenden Fixpreises so, sondern auch wegen der höheren Nachfrage, die die Marktpreise erhöht hat.Aus diesem Grund bitte ich Sie, dem Bundesbeschluss 3 ebenfalls zuzustimmen.</t>
   </si>
   <si>
     <t xml:space="preserve">377387</t>
@@ -500,6 +494,106 @@
 Erstens hat die GPK-S die parlamentarische Initiative 25.401, "Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken", eingereicht. Dieser Vorstoss, dieses Anliegen liegt zurzeit in der Kommission für Rechtsfragen des Ständerates. Die Motion 22.4250, "Erhöhung der Obergrenze der Gerichtsgebühren des Bundesgerichtes, des Bundesverwaltungsgerichtes und des Bundesstrafgerichtes", wurde von der Kommission für Rechtsfragen des Nationalrates im Rahmen einer grösseren Revision behandelt. Die Motion 25.4395 der RK-S, "Reorganisation des Bundesstrafgerichtes", wurde ebenfalls in der Kommission für Rechtsfragen des Nationalrates einstimmig gutgeheissen. Die Unabhängigkeit der ersten und zweiten Instanz soll damit besser gewährleistet werden. Dabei stützt sich die Kommission für Rechtsfragen auf den Bericht der GPK aus dem Jahre 2022. Weiter konnte die GPK-Subkommission Gerichte/BA den Bericht zum System der nebenamtlichen Richterinnen und Richter in der Kommission für Rechtsfragen des Nationalrates vorstellen. Wir gehen davon aus, dass sie diesbezüglich ebenfalls aktiv wird.
 Letztlich sei daran erinnert, dass das Bundesgericht im Jahr 2025 sein 150-jähriges Bestehen feierte. Zu diesem Anlass wurden unter anderem ein wissenschaftliches Kolloquium, eine Festschrift, eine offizielle Feier sowie Tage der offenen Tür mit etwa zweitausend Besuchern organisiert. 
 Ich möchte, Herr Bundesgerichtspräsident, diesen Bericht nicht abschliessen, ohne Ihre Arbeit zu verdanken, die gute Zusammenarbeit mit den Bundesbehörden und auch die Arbeit Ihres Sekretariats, unter anderem im Zusammenhang mit der Tätigkeit unserer Kommission.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377942</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fässler Daniel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. 
+Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. 
+Zur Detailberatung: Ich mache zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. 
+Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. 
+Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. 
+Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. 
+Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 
+1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 
+2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 
+3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. 
+Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dittli Josef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Postulat geht direkt auf unseren umfassenden Untersuchungsbericht vom 30. Januar 2026 zur Aufsicht und Steuerung der Ruag MRO zurück. Lassen Sie mich kurz rekapitulieren, worum es in dieser Untersuchung ging.
+Im Jahre 2023 beabsichtigte die Ruag MRO, 96 Leopard-1-Panzer nach Deutschland zu verkaufen. Die frühere Ruag Schweiz AG hatte die bereits seit Längerem ausser Dienst stehenden Panzer 2016 einer Agentur des italienischen Verteidigungsministeriums abgekauft. Sie wurden sodann in Itali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Postulat geht direkt auf unseren umfassenden Untersuchungsbericht vom 30. Januar 2026 zur Aufsicht und Steuerung der Ruag MRO zurück. Lassen Sie mich kurz rekapitulieren, worum es in dieser Untersuchung ging.
+Im Jahre 2023 beabsichtigte die Ruag MRO, 96 Leopard-1-Panzer nach Deutschland zu verkaufen. Die frühere Ruag Schweiz AG hatte die bereits seit Längerem ausser Dienst stehenden Panzer 2016 einer Agentur des italienischen Verteidigungsministeriums abgekauft. Sie wurden sodann in Italien gelagert. Bei diesem Geschäft traten Ungereimtheiten zutage. In der Folge veröffentlichte die Eidgenössische Finanzkontrolle in den Jahren 2024 und 2025 vier Berichte, die Mängel in der Compliance und Führung innerhalb der Ruag MRO, aber auch Probleme in der Aufsicht und Steuerung der Ruag MRO durch den Eigner, den Bund, aufzeigten.
+Unsere Kommission hat diese Vorfälle vertieft analysiert und festgestellt, dass die Probleme struktureller Natur sind. Die GPK richtete total sechs Empfehlungen zur Führung und Steuerung der Ruag MRO an den Bundesrat und beantragt dem Ständerat nun eben auch die Annahme dieses Postulates. Wir wollen damit den Bundesrat beauftragen, ergebnisoffen zu prüfen, ob die Corporate Governance des Bundes und das heutige duale Steuerungsmodell noch eine angemessene Wahrnehmung der Eignerinteressen erlauben. Er soll insbesondere prüfen, ob Anpassungen am aktuellen System nötig sind. Zudem soll er mögliche Alternativen, wie die Einsetzung einer einzigen zentralen Stelle für die Vorbereitung und Koordination aller eignerpolitischen Geschäfte zuhanden des Bundesrates, prüfen.
+Das heutige Modell birgt folgende Herausforderung. Das VBS ist nicht nur Miteigentümer, sondern auch der mit Abstand grösste Kunde der Ruag MRO. Die Eidgenössische Finanzverwaltung hingegen ist in dieser Kundenbeziehung nicht involviert und konzentriert sich rein auf die Finanzen. Dadurch entsteht ein Informationsgefälle. Die Eidgenössische Finanzverwaltung hat oft keinen Einblick in operative Sachverhalte, was das Risiko von blinden Flecken, etwa bei der Compliance, erhöht. Die GPK sieht daher möglichen Handlungsbedarf und identifiziert vier Schwachstellen des aktuellen Systems:
+1. Eine fehlende ganzheitliche Sicht: Da sich das VBS auf die Fachsicht und die Eidgenössische Finanzverwaltung auf die Finanzen fokussiert, fehlt oft eine kritische, ressortübergreifende Betrachtung.
+2. Uneinheitliche Umsetzung: Jedes Departement führt seine Unternehmen etwas anders. Eine bundesweite, einheitliche Linie fehlt.
+3. Komplexität: Die Betriebe sind hochkomplex und agieren am Markt. Übergeordnete Themen wie Governance oder Korruptionsbekämpfung erfordern gebündelte Expertise.
+4. Interessenkonflikte: Fachdepartemente sind oft Eigner, Kunde, Subventionsgeber und Regulator in Personalunion. Dies gefährdet eine objektive Aufsicht.
+Dies ganz kurz in etwa die Begründung des Postulates.
+Der Bundesrat beantragt die Ablehnung dieses Postulates. Seine Begründung ist vor allem formal. Man habe die Corporate Governance bereits 2018 und 2019 analysiert. Das Modell funktioniere gut, und mit dem neuen Artikel 24a der Regierungs- und Verwaltungsorganisationsverordnung (RVOV) sei die Aufgabenteilung nun rechtlich verankert. Ein Bericht bringe keine neuen Erkenntnisse.
+Die GPK-S teilt diese wohlwollende Sicht des Bundesrates nicht. Zu behaupten, die Ausgangslage habe sich seit 2019 nicht verändert, blendet die Realität aus. Die gravierenden Mängel bei der Ruag MRO, das Versagen bei den Compliance-Strukturen und die Intransparenz bei der Lagerverwaltung sind reale Befunde aus den Jahren 2024 und 2025. Sie traten also trotz der alten Berichte und trotz der neuen Verordnungstexte auf. Eine formale Aufgabenteilung auf dem Papier nützt uns nichts, wenn sie in der Praxis scheitert.
+Im Namen der GPK-S bitte ich Sie deshalb, das Postulat anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mühlemann Benjamin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Vorstoss von Kollege Regazzi verlangt einen Bericht zur Wirksamkeit, Zielgenauigkeit und volkswirtschaftlichen Wirkung von Bundessubventionen. Es geht insbesondere um die Fragen, welche Subventionen ihre Ziele erreichen, wo Fehlanreize oder Mitnahmeeffekte bestehen, wo Wettbewerbsverzerrungen entstehen können und wo Verbesserungen und allenfalls auch Reduktionen möglich wären.
+Ich finde, das ist ein sinnvoller und angemessener Auftrag, und deshalb beantrage ich Ihnen ebenfalls, das Postulat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Vorstoss von Kollege Regazzi verlangt einen Bericht zur Wirksamkeit, Zielgenauigkeit und volkswirtschaftlichen Wirkung von Bundessubventionen. Es geht insbesondere um die Fragen, welche Subventionen ihre Ziele erreichen, wo Fehlanreize oder Mitnahmeeffekte bestehen, wo Wettbewerbsverzerrungen entstehen können und wo Verbesserungen und allenfalls auch Reduktionen möglich wären.
+Ich finde, das ist ein sinnvoller und angemessener Auftrag, und deshalb beantrage ich Ihnen ebenfalls, das Postulat anzunehmen.
+Wir haben von Herrn Regazzi gehört, welches Instrumentarium bereits existiert. Darauf verweist auch der Bundesrat in seiner ablehnenden Stellungnahme. Nun ist das heutige Verfahren im Kern so angelegt: Die zuständigen Ämter nehmen zunächst eine Selbstbeurteilung vor. Die Eidgenössische Finanzverwaltung überprüft danach, ob die rechtlichen Grundlagen und die Subventionspraxis mit den Grundsätzen des Subventionsgesetzes übereinstimmen, und die Ergebnisse und allfällige Massnahmen werden dann im Rahmen der Staatsrechnung, bei entsprechenden Botschaften zu Finanzbeschlüssen oder bei Botschaften zu gesetzlichen Grundlagen ausgewiesen. Also, im Grundsatz ist das sicher ein wertvoller Prozess. Man muss dieses Instrument auch überhaupt nicht infrage stellen. Aber gerade weil dieses Instrument heute bereits besteht, sollten wir genauer hinschauen, um zu sehen, wie gut es tatsächlich wirkt.
+Die Eidgenössische Finanzkontrolle (EFK) hat dazu kürzlich einen sehr relevanten Bericht veröffentlicht, und ich melde mich genau deshalb zu Wort, damit dieser Bericht eine gewisse Öffentlichkeit erhält und nicht einfach in einer Schublade verschwindet. Dieser Bericht trägt den Titel "Prüfung des Prozesses und des Nutzens der periodischen Subventionsüberprüfung". Der Bericht ist vom Januar dieses Jahres.
+Die EFK kommt darin zu einem differenzierten Befund. Sie sagt nicht, dass das Verfahren nutzlos sei, im Gegenteil. Die periodische Überprüfung hat eine gewisse präventive Wirkung. Sie sensibilisiert die Verwaltungseinheiten für die Anforderungen des Subventionsgesetzes, und auch der administrative Aufwand wird von der EFK nicht als unverhältnismässig dargestellt. Aber die EFK zeigt ebenso klar auf, dass im Hinblick auf die eigentliche Steuerung der Bundessubventionen die Wirkung bisher zu gering ist. Das ist ein wichtiger Punkt, denn wir haben die Zahlen jetzt schon zwei-, dreimal gehört. Es geht bei diesem Volumen von 48 Milliarden Franken, das bereitgestellt wird, nicht um einen Randbereich des Bundeshaushalts. Die EFK nennt drei Punkte, die aus meiner Sicht für die heutige Diskussion ganz besonders wichtig sind. 
+Zum ersten Punkt: Die Überprüfung ist eben nicht vollständig. Die Finanzverwaltung stützt sich bei der Auswahl der zu prüfenden Subventionen auf die Ausgabenkredite. Bestimmte Formen von Subventionen werden dadurch nicht oder nicht systematisch erfasst. Dazu gehören etwa unentgeltliche oder vergünstigte Leistungen des Bundes. Dazu gehören Subventionen über Fonds oder Institutionen, die im Auftrag des Bundes handeln, sowie Steuervergünstigungen. Die EFK hält fest, dass die Finanzverwaltung über keine abschliessende Übersicht dieser Subventionsformen verfügt und auch das entsprechende Volumen nicht kennt. 
+Zum zweiten Punkt, der bemängelt wird: Die Ämter melden im Rahmen ihrer Selbstbeurteilung Abweichungen von den Grundsätzen des Subventionsgesetzes in der Regel nicht von sich aus. Die Finanzverwaltung kann zwar noch Probleme identifizieren und dann auch Massnahmen vorschlagen, aber diese Massnahmen werden in der Regel im Konsens mit den betroffenen Verwaltungseinheiten vereinbart, auch um eine Eskalation zu vermeiden. 
+Zum dritten Punkt, den die EFK bemängelt: Die finanziellen Auswirkungen bleiben bisher sehr, sehr bescheiden. Die EFK stellt fest, dass zwischen 2014 und 2024 nur vier Fälle identifiziert wurden, in denen Massnahmen zur Streichung einer Subvention oder zu einer effektiven Einsparung geführt haben. Das Einsparvolumen betrug insgesamt 2,3 Millionen Franken pro Jahr. Bei einem Subventionsvolumen von 48 Milliarden Franken ist das ja eigentlich nichts. 
+Persönlich komme ich zum Schluss, dass in der periodischen Subventionsüberprüfung Potenzial liegt, das heute nicht genügend ausgeschöpft wird. Genau hier setzt das Postulat Regazzi an. Er verlangt nicht, dass Subventionen pauschal infrage gestellt werden; das wäre auch nicht sachgerecht. Aber es braucht eine saubere Unterscheidung. Wir müssen wissen, welche Subventionen noch ihre Ziele erreichen, welche noch gerechtfertigt sind, welche allenfalls angepasst werden müssen. Wir müssen auch wissen, wo Mitnahmeeffekte da sind, wo Fehlanreize gesetzt werden und wo der Mitteleinsatz nicht mehr im Verhältnis zur Wirkung steht. 
+Es ist also sinnvoll, heute die Grundlagen für eine nächste Prüfung, die zweifelsohne stattfinden wird, zu verbessern. Es geht nicht darum, jetzt sofort ein neues, grosses Entlastungspaket zu schnüren. Es geht darum, im ordentlichen Prozess früher, systematischer und wirksamer zu erkennen, wo Handlungsbedarf besteht. Wenn wir in Zukunft grössere Sparrunden und hektische Entlastungsprogramme vermeiden wollen, dann müssen wir im Tagesgeschäft besser steuern. Die periodische Subventionsüberprüfung ist dafür ein geeignetes Instrument, aber, ich habe den Bericht der EFK erwähnt, eben noch kein genügend wirksames Instrument. Das Postulat Regazzi ist deshalb ein sachlicher und moderater Beitrag, um hier weiterzukommen. 
+Ich bitte Sie, dieses Postulat anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">378033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gapany Johanna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En voyant le vote de la commission, je me doute qu'il y a un vrai malaise autour de ce programme. Il y a autant de membres de la commission qui se sont abstenus que de membres qui se sont opposés à l'initiative de notre collègue Stark. Ce débat n'est donc pas totalement inutile vu ce résultat. Et même si on est tous d'accord, je crois, sur la nécessité de récolter et de traiter des données, la méthode pose problème. Personne, dans cette salle, ne conteste la nécessité d'un suivi sérieux, crédibl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En voyant le vote de la commission, je me doute qu'il y a un vrai malaise autour de ce programme. Il y a autant de membres de la commission qui se sont abstenus que de membres qui se sont opposés à l'initiative de notre collègue Stark. Ce débat n'est donc pas totalement inutile vu ce résultat. Et même si on est tous d'accord, je crois, sur la nécessité de récolter et de traiter des données, la méthode pose problème. Personne, dans cette salle, ne conteste la nécessité d'un suivi sérieux, crédible aussi, de l'utilisation des produits phytosanitaires. En fait, c'est ce qu'on avait défendu devant la population, et la population a massivement refusé les initiatives dont on parle et dont on parlait précédemment. Le suivi se fait d'ailleurs déjà et il se fera encore demain ; il se fera sans doute encore plus demain. Les produits utilisés sont beaucoup plus contrôlés que du temps de nos parents, c'est un fait. Ils le sont aussi beaucoup plus en Suisse que dans la plupart des autres pays dans le monde.
+Personne ne conteste non plus que notre agriculture doit pouvoir démontrer ses efforts, sa responsabilité et sa capacité à évoluer. Au contraire, on veut - et on le voit aussi quand on lit les perspectives de la politique agricole 2030 -, une agriculture moderne, capable de nourrir la population en utilisant le progrès. Alors, ce qu'on exige de l'agriculture, on doit être capable de l'appliquer aussi à l'administration fédérale : de la modernité, de l'efficacité et un système qui fonctionne dans la pratique. C'est tout simplement ce que demande notre collègue Stark.
+On parle aussi de surcharge bureaucratique, avec le Digiflux dans sa version actuelle. Ce n'est pas seulement un terme à la mode, cette surcharge bureaucratique. C'est un vrai fléau et un vrai frein à la production alimentaire, alors que déjà aujourd'hui, on parle de pénurie dans certains domaines. Personne ici - en tout cas j'imagine - ne pense d'ailleurs que les agriculteurs ou les PME s'ennuient au point qu'il faut leur donner du travail supplémentaire. La pression est déjà suffisante, entre la hausse généralisée des coûts, la multiplication des normes, les exigences administratives aussi, qui sont toujours plus nombreuses. On peut dire sans caricaturer que ceux qui nous nourrissent passent gentiment plus de temps devant leur ordinateur que sur le tracteur.
+Et sur ce constat, on vient ajouter une couche supplémentaire, sans gain pour la production. C'est d'autant plus un problème que c'est contraire à un principe qu'on avait voulu dans ce Parlement, le principe "once only", selon lequel chaque donnée doit être introduite une seule fois dans un système. C'est un principe de bon sens, un principe d'efficacité, et aujourd'hui, avec la version actuelle du Digiflux, clairement, on ne le met pas en oeuvre.
+Et puis, il y a un autre élément qui est quand même important : le Contrôle fédéral des finances a lui-même rendu un rapport et il a fait sept recommandations concrètes. Ce rapport était très clairement critique : il a relevé des lacunes dans le pilotage du projet, dans la clarté des bénéfices attendus et dans l'utilisation des données. Pour un projet dont le budget est quand même d'environ 16 millions de francs, quand on reçoit ce genre de remarques, notamment sur les lacunes au niveau du pilotage, mais aussi au niveau des bénéfices attendus, on ne peut pas simplement en prendre connaissance et passer à autre chose. C'est non seulement une question technique, mais c'est aussi une question de confiance. Celles et ceux qui livrent ces données doivent avoir la garantie que les données sensibles concernant leur activité, concernant leurs clients, soient traitées de manière transparente, avec une base légale claire et dans un objectif qui est précisément défini. Cette confiance est élémentaire si on veut que les acteurs du terrain adhèrent à ce système.
+La proposition de notre collègue Stark va précisément dans cette direction, et c'est la raison pour laquelle je la soutiens. Je la soutiens d'autant plus qu'elle ne remet pas en question les engagements de l'agriculture. Elle vise un système plus pragmatique, plus proportionné et utilisable aussi dans la pratique ; un système qui est compatible avec une agriculture moderne, qui respecte ses engagements environnementaux, mais sans être étouffée par des charges administratives dont les bénéfices ne sont pas clairs, comme l'a dit le Contrôle fédéral des finances.
+Je vous remercie pour votre attention et j'espère vous voir soutenir cette initiative parlementaire ainsi que l'initiative du canton de Berne en y donnant suite.
 </t>
   </si>
 </sst>
@@ -548,8 +642,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I14" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I18" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I18"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1251,6 +1345,122 @@
         <v>87</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>97</v>
+      </c>
+      <c r="I16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
+      </c>
+      <c r="I17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-19
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -174,7 +174,7 @@
 Die Schweiz gehört zu den am stärksten digitalisierten Volkswirtschaften der Welt. Unsere Stromversorgung, unser Finanzplatz, unsere Kommunikationsnetze und zahlreiche staatliche Dienstleistungen sind auf funktionierende digitale Infrastrukturen angewiesen. Cyberangriffe oder andere Angriffe können enorme wirtschaftliche Schäden verursachen. Der Nachrichtendienst spielt deshalb eine wichtige Rolle bei der Erkennung und Abwehr solcher Bedrohungen. Die vorliegende Gesetzesrevision stärkt seine Fähigkeit, Gefahren im digitalen Raum frühzeitig zu erkennen und relevante Informationen mit den zuständigen Behörden auszutauschen.
 Ein moderner Nachrichtendienst schützt zudem die Innovationskraft unseres Landes. Schweizer Hochschulen, Forschungsinstitutionen und Unternehmen verfügen über Wissen und Technologien von strategischer Bedeutung. Diese werden zunehmend Ziel ausländischer Spionage. Der Schutz geistigen Eigentums und sensibler Informationen ist deshalb nicht nur eine Frage der Sicherheit, sondern auch der wirtschaftlichen Zukunft unseres Landes.
 Gleichzeitig gilt: Mehr Kompetenzen verlangen mehr Verantwortung. Nachrichtendienstliche Tätigkeiten greifen in Grundrechte ein. Für die GLP-Fraktion ist deshalb klar, dass jede Erweiterung staatlicher Befugnisse von wirksamen rechtsstaatlichen Garantien begleitet werden muss.
-Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen - zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
+Wir dürfen die Herausforderungen der Zukunft nicht unterschätzen. Die erweiterten Kompetenzen im Cyberraum führen unweigerlich zu grösseren Datenmengen, zu einem, wie gesagt wurde, grösseren Heuhaufen. Insbesondere der Einsatz künstlicher Intelligenz und algorithmischer Auswertungen wirft neue Fragen auf. Deshalb müssen auch die Aufsichts- und Kontrollmechanismen laufend weiterentwickelt werden. Die Zusammenarbeit zwischen der Aufsichtsbehörde über den Nachrichtendienst, der Geschäftsprüfungsdelegation und der Eidgenössischen Finanzkontrolle verdient daher besondere Aufmerksamkeit.
 Wichtig sind auch klare Datenschutzgarantien im Gesetz, insbesondere wenn der NDB neu gegen gewalttätig-extremistische Personen genehmigungspflichtige Beschaffungsmassnahmen ergreifen kann und die Daten nicht mehr in getrennten Einzelsystemen bearbeitet werden müssen. Es ist zu begrüssen, dass weiterhin eine konsequente Zweckbindung und ein kontrollierter Zugriff, der nur besonders berechtigten Personen offensteht, vorgesehen sind.
 Kritikerinnen und Kritiker warnen vor einem Abbau der Privatsphäre. Diese Bedenken sind durchaus nachvollziehbar. Wer jedoch die bestehenden Kontrollmechanismen ausblendet, zeichnet ein unvollständiges Bild. Der Nachrichtendienst untersteht politischen, administrativen und rechtlichen Kontrollen. Die GLP-Fraktion wird an verschiedenen Stellen in der Vorlage für eine weitere Stärkung dieser Kontrollen eintreten.
 Die Frage lautet deshalb nicht, ob wir einen schlagkräftigen Nachrichtendienst brauchen. Die eigentliche Frage lautet, ob wir die Augen vor den realen Bedrohungen unserer Zeit verschliessen wollen. Terrorismus, Cyberangriffe, Spionage und ausländische Einflussnahme verschwinden nicht, wenn wir auf wirksame Instrumente verzichten. Das Gegenteil ist der Fall.
@@ -512,17 +512,7 @@
     <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. 
-Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. 
-Zur Detailberatung: Ich mache zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. 
-Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. 
-Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. 
-Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. 
-Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 
-1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 
-2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 
-3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. 
-Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
+    <t xml:space="preserve">Ich stelle nach der Abstimmung zum Eintreten fest, dass der Handlungsbedarf in unserem Rat - wie bereits vor zwei Jahren, als wir in unserem Rat über das Folgegeben entschieden hatten - nicht von allen anerkannt wird. Ich muss offenlegen, dass ich damals in unserem Rat gegen diese parlamentarische Initiative gestimmt habe. Wir haben dann aber festgestellt, dass der Rat einen solchen Erlassentwurf auf dem Tisch haben möchte. Wir haben diesen Auftrag erfüllt und Ihnen heute das Resultat vorgelegt. Ich möchte mich zuerst noch bei Ihnen, Frau Bundesrätin, für Ihre Ausführungen zu dem bedanken, was sich der Bundesrat noch überlegen muss, wenn der Erlassentwurf gutgeheissen wird. Zur Detailberatung: Ich mache jetzt in einem einzigen Votum zu allen Bestimmungen Ausführungen, weil sie auch zusammenhängen. Die bisherige Grundsatzbestimmung von Artikel 19 Absatz 4 des Bundespersonalgesetzes, wonach bei Beendigung eines Arbeitsverhältnisses im gegenseitigen Einvernehmen sowie in besonderen Fällen eine Entschädigung vorgesehen werden kann, bleibt unverändert bestehen. Ein solcher besonderer Fall liegt gemäss Absatz 3 vor, wenn die angestellte Person in einem Beruf arbeitet, nach dem keine oder nur eine schwache Nachfrage besteht, wenn das Arbeitsverhältnis lange gedauert hat oder die betroffene Person ein bestimmtes Alter erreicht hat. Mit einem neuen Absatz 4bis werden aber neu die Mitglieder der Geschäftsleitung von allfälligen Entschädigungen ausgenommen. Dies führt zu einer Gleichbehandlung mit den Mitgliedern der Geschäftsleitungen von börsenkotierten Gesellschaften gemäss Artikel 735c Ziffer 1 des Obligationenrechts. Gemäss dieser Bestimmung sind vertraglich vereinbarte oder statutarisch vorgesehene Abgangsentschädigungen unzulässig. Der Vorbehalt im zweiten Satzteil des neuen Absatzes 4bis von Artikel 19 ist für Fälle gemäss Absatz 3 nötig, um den verfassungsrechtlich garantierten Grundsatz der Rechtsgleichheit nicht zu verletzen. Diese Bestimmungen sollen aufgrund der Unterstellung unter das Bundespersonalgesetz nicht nur für die zentrale Bundesverwaltung, sondern gemäss Artikel 6a Absatz 2bis und Artikel 19 Absatz 4bis auch für weitere Geschäftsleitungen gelten, und zwar für die dem Bundespersonalgesetz unterstellten Verwaltungseinheiten wie zum Beispiel die Pensionskasse Publica, für die organisatorisch verselbständigten dezentralen Verwaltungseinheiten ohne Rechtspersönlichkeit wie zum Beispiel die Eidgenössische Finanzkontrolle und für die Sekretariate ausserparlamentarischer Kommissionen wie zum Beispiel die Weko. Die Kommission beantragt, das Bundespersonalgesetz mit dieser Vorlage mit einer Übergangsbestimmung zu ergänzen: Der neue Artikel 41b soll sicherstellen, dass die Änderung zu den Abgangsentschädigungen für bestehende altrechtliche Arbeitsverträge nicht gilt. Ohne diese Besitzstandsgarantie würde das schutzwürdige Vertrauen der betroffenen Personen in rechtlich ungerechtfertigter Weise beeinträchtigt. Damit die vorgesehene Änderung umfassend umgesetzt wird, genügt es nicht, nur das Bundespersonalgesetz zu ändern, auch diverse andere Erlasse müssen geändert werden. Sie finden die entsprechenden Anträge der Kommission auf den Seiten 7 bis 29 der Fahne. Ich beschränke meine Ausführungen dazu auf wenige Punkte: 1. Das ETH-Gesetz sah bisher als einziges Spezialgesetz explizit Abgangsentschädigungen vor. Es ist daher nötig, die entsprechende Bestimmung im ETH-Gesetz aufzuheben. 2. In den Spezialgesetzen der Skyguide, der Identitas AG, der Rüstungsunternehmen des Bundes und von Schweiz Tourismus fehlt bisher der Verweis auf Artikel 6a des Bundespersonalgesetzes. Damit die Bestimmungen über das Verbot von Abgangsentschädigungen auch für diese Unternehmen gelten, sind die entsprechenden Spezialgesetze mit einem Verweis auf Artikel 6a des Bundespersonalgesetzes zu ergänzen. 3. In den übrigen relevanten Gesetzen, die den Verweis auf Artikel 6a des Bundespersonalgesetzes bereits enthalten, muss schliesslich nur die Übergangsbestimmung aufgenommen werden. Ich komme damit zum Schluss: Die Kommission beantragt Ihnen, den Entwurf in allen Punkten in der vorliegenden Fassung anzunehmen.
 </t>
   </si>
   <si>

</xml_diff>